<commit_message>
docs: prepare workbook demos for Show HN
</commit_message>
<xml_diff>
--- a/Sudoku/sudoku.xlsx
+++ b/Sudoku/sudoku.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3373B9D-2E4A-8D4F-BFB2-1D98CB16392F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
@@ -4974,53 +4969,6 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{72189DE0-938E-0A48-A3F3-08380738F50D}">
-  <we:reference id="wa200010215" version="2.0.0.0" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="wa200010215" version="2.0.0.0" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="bps.codex_control.document_id" value="&quot;0d36fea8-eb1c-4367-a81f-74621330bc59&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
-<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{42140C96-38E2-C640-9422-7287D4D55172}">
-  <we:reference id="wa200003696" version="1.3.0.0" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200003696" version="1.3.0.0" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties/>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
-      <we:customFunctionIdList>
-        <we:customFunctionIds>_xldudf_LABS_GENERATIVEAI</we:customFunctionIds>
-      </we:customFunctionIdList>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A9B5CCF-D0DB-3147-8E44-107C505B5881}">
   <sheetPr codeName="Sheet1">

</xml_diff>

<commit_message>
Migrate Master candidate chain to production
</commit_message>
<xml_diff>
--- a/Sudoku/sudoku.xlsx
+++ b/Sudoku/sudoku.xlsx
@@ -1,9 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE03ACF-D307-B942-A61D-63EDE05F9C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB8E379-B146-B447-AB9F-81140D0CB4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -74,6 +79,33 @@
     <definedName name="SDK_SolveStatus">_xlfn.LAMBDA(_xlpm.board,IF(OR(ROWS(_xlpm.board)&lt;&gt;9,COLUMNS(_xlpm.board)&lt;&gt;9),"SEARCH ERROR",IFERROR(_xlfn.LET(_xlpm.result,SDK_Solve(_xlpm.board),IF(AND(ISNA(_xlpm.result)),"NO SOLUTION","VIABLE")),"SEARCH ERROR")))</definedName>
     <definedName name="SDK_SolveTry" comment="Recursive branch iterator used by SDK_Solve; tries candidate digits in order.">_xlfn.LAMBDA(_xlpm.board,_xlpm.r,_xlpm.c,_xlpm.options,_xlpm.i,IF(_xlpm.i&gt;LEN(_xlpm.options),NA(),_xlfn.LET(_xlpm.nextBoard,SDK_SetCell(_xlpm.board,_xlpm.r,_xlpm.c,--MID(_xlpm.options,_xlpm.i,1)),_xlpm.result,IFERROR(SDK_Solve(_xlpm.nextBoard),NA()),IF(IFERROR(AND(ROWS(_xlpm.result)=9,COLUMNS(_xlpm.result)=9),FALSE),_xlpm.result,SDK_SolveTry(_xlpm.board,_xlpm.r,_xlpm.c,_xlpm.options,_xlpm.i+1)))))</definedName>
     <definedName name="SDK_Uniqueness">_xlfn.LAMBDA(_xlpm.board,IFERROR(_xlfn.LET(_xlpm.n,SDK_CountSolutions(_xlpm.board,2),CHOOSE(_xlpm.n+1,"NO SOLUTION","UNIQUE","MULTIPLE SOLUTIONS")),"SEARCH ERROR"))</definedName>
+    <definedName name="SDKP_AdvancedHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_PointingRow(_xlpm.c),_xlpm.b,SDKP_PointingCol(_xlpm.c),_xlpm.d,SDKP_ClaimingRow(_xlpm.c),_xlpm.e,SDKP_ClaimingCol(_xlpm.c),_xlpm.f,SDKP_NakedPairRow(_xlpm.c),_xlpm.g,SDKP_NakedPairCol(_xlpm.c),_xlpm.h,SDKP_NakedPairBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,IF(_xlpm.e&lt;&gt;"",_xlpm.e,IF(_xlpm.f&lt;&gt;"",_xlpm.f,IF(_xlpm.g&lt;&gt;"",_xlpm.g,_xlpm.h))))))))</definedName>
+    <definedName name="SDKP_Apply">_xlfn.LAMBDA(_xlpm.c,_xlpm.h,_xlfn.LET(_xlpm.removeText,_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.h,"Remove ")," from "),_xlpm.targets,_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(_xlpm.h," from "), "."),_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
+    <definedName name="SDKP_ApplyStep">_xlfn.LAMBDA(_xlpm.c,_xlpm.s,_xlfn.LET(_xlpm.removeText,INDEX(_xlpm.s,1,3)&amp;"",_xlpm.targets,INDEX(_xlpm.s,1,4)&amp;"",_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.cur,INDEX(_xlpm.c,_xlpm.r,_xlpm.k)&amp;"",_xlpm.coord,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k,IF(OR(_xlpm.cur="",ISERROR(SEARCH(_xlpm.coord,_xlpm.targets))),_xlpm.cur,_xlfn.LET(_xlpm.chars,MID(_xlpm.cur,_xlfn.SEQUENCE(LEN(_xlpm.cur)),1),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.chars,ISERROR(SEARCH(_xlpm.chars,_xlpm.removeText)),"")))))))))</definedName>
+    <definedName name="SDKP_BasicHint">_xlfn.LAMBDA(_xlpm.c,_xlfn.LET(_xlpm.a,SDKP_Naked(_xlpm.c),_xlpm.b,SDKP_HiddenRow(_xlpm.c),_xlpm.d,SDKP_HiddenCol(_xlpm.c),_xlpm.e,SDKP_HiddenBox(_xlpm.c),IF(_xlpm.a&lt;&gt;"",_xlpm.a,IF(_xlpm.b&lt;&gt;"",_xlpm.b,IF(_xlpm.d&lt;&gt;"",_xlpm.d,_xlpm.e)))))</definedName>
+    <definedName name="SDKP_Chain">_xlfn.LAMBDA(_xlpm.board,_xlpm.lim,SDKP_ChainLoop(_xlpm.board,SDK_CandidateMatrix(_xlpm.board),0,_xlpm.lim,""))</definedName>
+    <definedName name="SDKP_ChainLoop">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlpm.steps,_xlpm.lim,_xlpm.log,_xlfn.LET(_xlpm.bad,SDKP_Contradiction(_xlpm.board,_xlpm.c),_xlpm.basic,IF(_xlpm.bad,"",SDKP_BasicHint(_xlpm.c)),_xlpm.emptyStep,_xlfn.HSTACK("","","","",""),_xlpm.rowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingRowStep(_xlpm.c)),_xlpm.rowText,INDEX(_xlpm.rowStep,1,5),_xlpm.colStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;""),_xlpm.emptyStep,SDKP_PointingColStep(_xlpm.c)),_xlpm.colText,INDEX(_xlpm.colStep,1,5),_xlpm.claimRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingRowStep(_xlpm.c)),_xlpm.claimRowText,INDEX(_xlpm.claimRowStep,1,5),_xlpm.claimColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_ClaimingColStep(_xlpm.c)),_xlpm.claimColText,INDEX(_xlpm.claimColStep,1,5),_xlpm.pairRowStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairRowStep(_xlpm.c)),_xlpm.pairRowText,INDEX(_xlpm.pairRowStep,1,5),_xlpm.pairColStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;"",_xlpm.pairRowText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairColStep(_xlpm.c)),_xlpm.pairColText,INDEX(_xlpm.pairColStep,1,5),_xlpm.pairBoxStep,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;"",_xlpm.rowText&lt;&gt;"",_xlpm.colText&lt;&gt;"",_xlpm.claimRowText&lt;&gt;"",_xlpm.claimColText&lt;&gt;"",_xlpm.pairRowText&lt;&gt;"",_xlpm.pairColText&lt;&gt;""),_xlpm.emptyStep,SDKP_NakedPairBoxStep(_xlpm.c)),_xlpm.pairBoxText,INDEX(_xlpm.pairBoxStep,1,5),_xlpm.step,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowStep,IF(_xlpm.colText&lt;&gt;"",_xlpm.colStep,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowStep,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColStep,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowStep,IF(_xlpm.pairColText&lt;&gt;"",_xlpm.pairColStep,_xlpm.pairBoxStep)))))),_xlpm.stepText,IF(_xlpm.rowText&lt;&gt;"",_xlpm.rowText,IF(_xlpm.colText&lt;&gt;"",_xlpm.colText,IF(_xlpm.claimRowText&lt;&gt;"",_xlpm.claimRowText,IF(_xlpm.claimColText&lt;&gt;"",_xlpm.claimColText,IF(_xlpm.pairRowText&lt;&gt;"",_xlpm.pairRowText,IF(_xlpm.pairColText&lt;&gt;"",_xlpm.pairColText,_xlpm.pairBoxText)))))),_xlpm.adv,IF(OR(_xlpm.bad,_xlpm.basic&lt;&gt;""),"",_xlpm.stepText),_xlpm.state,IF(_xlpm.bad,"CONTRADICTION",IF(_xlpm.basic&lt;&gt;"","ASSIGNMENT",IF(_xlpm.adv="","STABLE",IF(_xlpm.steps&gt;=_xlpm.lim,"LIMIT","CONTINUE")))),IF(_xlpm.state="CONTINUE",_xlfn.LET(_xlpm.next,SDKP_ApplyStep(_xlpm.c,_xlpm.step),IF(SDKP_HasProgress(_xlpm.c,_xlpm.next),SDKP_ChainLoop(_xlpm.board,_xlpm.next,_xlpm.steps+1,_xlpm.lim,IF(_xlpm.log="",_xlpm.adv,_xlpm.log&amp;CHAR(10)&amp;_xlpm.adv)),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,"NO_PROGRESS",_xlpm.steps,"",_xlpm.adv,_xlpm.log,"","","","")))))),_xlfn.VSTACK(_xlpm.c,_xlfn.MAKEARRAY(1,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,CHOOSE(_xlpm.k,_xlpm.state,_xlpm.steps,_xlpm.basic,_xlpm.adv,_xlpm.log,"","","","")))))))</definedName>
+    <definedName name="SDKP_ClaimingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingColStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_ClaimingColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.i,_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,0,_xlpm.k),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.rs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.rs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*(_xlpm.band-1),_xlpm.bc,1+3*QUOTIENT(_xlpm.k-1,3),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.cc&lt;&gt;_xlpm.k)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.rs&amp;"C"&amp;_xlpm.k),_xlpm.b,3*(_xlpm.band-1)+1+QUOTIENT(_xlpm.k-1,3),_xlpm.displayText,"Claiming column · Column "&amp;_xlpm.k&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".",IF(_xlpm.txt&lt;&gt;"",_xlfn.HSTACK("Claiming column",_xlpm.sourceText,_xlpm.d&amp;"",_xlpm.txt,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
+    <definedName name="SDKP_ClaimingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_ClaimingRowStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_ClaimingRowStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.i,_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.i-1,9)+1,_xlpm.d,MOD(_xlpm.i-1,9)+1,_xlpm.v,INDEX(_xlpm.c,_xlpm.r,0),_xlpm.m,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.v&amp;"")),_xlpm.n,SUM(--_xlpm.m),_xlpm.cs,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.m,""),_xlpm.bands,1+QUOTIENT(_xlpm.cs-1,3),_xlpm.one,IF(_xlpm.n&gt;1,MIN(_xlpm.bands)=MAX(_xlpm.bands),FALSE),_xlpm.band,IF(_xlpm.one,INDEX(_xlpm.bands,1,1),1),_xlpm.br,1+3*QUOTIENT(_xlpm.r-1,3),_xlpm.bc,1+3*(_xlpm.band-1),_xlpm.sub,INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),_xlpm.rr,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.br+_xlpm.x-1)),_xlpm.cc,_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.x,_xlpm.y,_xlpm.bc+_xlpm.y-1)),_xlpm.tm,IF(_xlpm.one,(_xlpm.rr&lt;&gt;_xlpm.r)*ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.sub&amp;"")),FALSE),_xlpm.targets,_xlfn._xlws.FILTER("R"&amp;_xlfn.TOCOL(_xlpm.rr)&amp;"C"&amp;_xlfn.TOCOL(_xlpm.cc),_xlfn.TOCOL(_xlpm.tm),""),_xlpm.txt,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targets),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,"R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.cs),_xlpm.b,3*QUOTIENT(_xlpm.r-1,3)+_xlpm.band,_xlpm.displayText,"Claiming row · Row "&amp;_xlpm.r&amp;" confines digit "&amp;_xlpm.d&amp;" to box "&amp;_xlpm.b&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.d&amp;" from "&amp;_xlpm.txt&amp;".",IF(_xlpm.txt&lt;&gt;"",_xlfn.HSTACK("Claiming row",_xlpm.sourceText,_xlpm.d&amp;"",_xlpm.txt,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
+    <definedName name="SDKP_Contradiction">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.conflict,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,--SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k))))&gt;0,_xlpm.deadCell,SUM(--((_xlpm.board="")*(_xlpm.c="")))&gt;0,_xlpm.rowMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,_xlpm.r,0)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;"")))=0))))&gt;0,_xlpm.colMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--AND(SUM(--(INDEX(_xlpm.board,0,_xlpm.k)=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;"")))=0))))&gt;0,_xlpm.boxMissing,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.bv,_xlfn.TOCOL(INDEX(_xlpm.board,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.cv,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--AND(SUM(--(_xlpm.bv=_xlpm.d))=0,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.cv&amp;"")))=0)))))&gt;0,OR(_xlpm.conflict,_xlpm.deadCell,_xlpm.rowMissing,_xlpm.colMissing,_xlpm.boxMissing,SDKP_ForcedConflict(_xlpm.board,_xlpm.c))))</definedName>
+    <definedName name="SDKP_ForcedConflict">_xlfn.LAMBDA(_xlpm.board,_xlpm.c,_xlfn.LET(_xlpm.forced,IF((_xlpm.board="")*(LEN(_xlpm.c&amp;"")=1),_xlpm.c&amp;"",""),_xlpm.rowBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,_xlpm.r,0)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.colBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,--(SUM(--(INDEX(_xlpm.forced,0,_xlpm.k)=_xlpm.d&amp;""))&gt;1))))&gt;0,_xlpm.boxBad,SUM(_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.v,_xlfn.TOCOL(INDEX(_xlpm.forced,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),--(SUM(--(_xlpm.v=_xlpm.d&amp;""))&gt;1)))))&gt;0,OR(_xlpm.rowBad,_xlpm.colBad,_xlpm.boxBad)))</definedName>
+    <definedName name="SDKP_HasProgress">_xlfn.LAMBDA(_xlpm.before,_xlpm.after,SUM(LEN(_xlpm.after&amp;""))&lt;SUM(LEN(_xlpm.before&amp;"")))</definedName>
+    <definedName name="SDKP_HiddenBox">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.b,_xlpm.d,_xlfn.LET(_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc))&amp;"")))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.b,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.br,1+3*QUOTIENT(_xlpm.b-1,3),_xlpm.bc,1+3*MOD(_xlpm.b-1,3),_xlpm.x,_xlfn.TOCOL(INDEX(_xlpm.c,_xlfn.SEQUENCE(3,,_xlpm.br),_xlfn.SEQUENCE(,3,_xlpm.bc)),0,FALSE),_xlpm.q,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",_xlpm.x&amp;""))),_xlpm.r,_xlpm.br+QUOTIENT(_xlpm.q-1,3),_xlpm.k,_xlpm.bc+MOD(_xlpm.q-1,3),"Hidden single in box · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in box "&amp;_xlpm.b&amp;"."))))</definedName>
+    <definedName name="SDKP_HiddenCol">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.k,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.k,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.r,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,0,_xlpm.k)&amp;""))),"Hidden single in column · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in column "&amp;_xlpm.k&amp;"."))))</definedName>
+    <definedName name="SDKP_HiddenRow">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.n,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.d,SUM(--ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))))),_xlpm.p,IFERROR(_xlfn.XMATCH(1,_xlfn.TOCOL(_xlpm.n)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.d,MOD(_xlpm.p-1,9)+1,_xlpm.k,_xlfn.XMATCH(TRUE,ISNUMBER(SEARCH(_xlpm.d&amp;"",INDEX(_xlpm.c,_xlpm.r,0)&amp;""))),"Hidden single in row · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · Digit "&amp;_xlpm.d&amp;" appears in only one candidate set in row "&amp;_xlpm.r&amp;"."))))</definedName>
+    <definedName name="SDKP_Naked">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.c,_xlpm.inputCandidates,_xlpm.m,LEN(_xlpm.c)=1,_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlfn.TOCOL(_xlpm.m)),0),IF(_xlpm.p=0,"",_xlfn.LET(_xlpm.r,QUOTIENT(_xlpm.p-1,9)+1,_xlpm.k,MOD(_xlpm.p-1,9)+1,_xlpm.d,INDEX(_xlpm.c,_xlpm.r,_xlpm.k),"Naked single · R"&amp;_xlpm.r&amp;"C"&amp;_xlpm.k&amp;" = "&amp;_xlpm.d&amp;" · This is the only legal candidate remaining in the square."))))</definedName>
+    <definedName name="SDKP_NakedPairBox">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairBoxStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_NakedPairBoxStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.rowNum-1,3),_xlpm.boxStartCol,1+3*QUOTIENT(_xlpm.colNum-1,3),_xlpm.unitVals,_xlfn.TOCOL(INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)))&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondIndex,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.rowCoords,_xlpm.boxStartRow+QUOTIENT(_xlfn.SEQUENCE(9)-1,3),_xlpm.colCoords,_xlpm.boxStartCol+MOD(_xlfn.SEQUENCE(9)-1,3),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstIndex)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondIndex),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoords&amp;"C"&amp;_xlpm.colCoords,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.firstRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.firstIndex-1,3),_xlpm.firstCol,_xlpm.boxStartCol+MOD(_xlpm.firstIndex-1,3),_xlpm.secondRow,_xlpm.boxStartRow+QUOTIENT(_xlpm.secondIndex-1,3),_xlpm.secondCol,_xlpm.boxStartCol+MOD(_xlpm.secondIndex-1,3),_xlpm.boxNum,1+3*QUOTIENT(_xlpm.rowNum-1,3)+QUOTIENT(_xlpm.colNum-1,3),_xlpm.sourceText,"R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;", R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol,_xlpm.displayText,"Naked pair in box · R"&amp;_xlpm.firstRow&amp;"C"&amp;_xlpm.firstCol&amp;" and R"&amp;_xlpm.secondRow&amp;"C"&amp;_xlpm.secondCol&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" in box "&amp;_xlpm.boxNum&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in box",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
+    <definedName name="SDKP_NakedPairCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairColStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_NakedPairColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.colNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.rowNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,0,_xlpm.colNum)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,ROWS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlfn.SEQUENCE(9)&amp;"C"&amp;_xlpm.colNum,_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.sourceText,"R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;", R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum,_xlpm.displayText,"Naked pair in column · R"&amp;_xlpm.firstPos&amp;"C"&amp;_xlpm.colNum&amp;" and R"&amp;_xlpm.secondPos&amp;"C"&amp;_xlpm.colNum&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in column",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
+    <definedName name="SDKP_NakedPairRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_NakedPairRowStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_NakedPairRowStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.rowNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.colNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.pairText,INDEX(_xlpm.candMatrix,_xlpm.rowNum,_xlpm.colNum)&amp;"",_xlpm.unitVals,INDEX(_xlpm.candMatrix,_xlpm.rowNum,0)&amp;"",_xlpm.pairFlag,AND(LEN(_xlpm.pairText)=2,SUM(--(_xlpm.unitVals=_xlpm.pairText))=2),_xlpm.pairPositions,_xlfn._xlws.FILTER(_xlfn.SEQUENCE(,9),_xlpm.unitVals=_xlpm.pairText,""),_xlpm.firstPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,1),0),_xlpm.secondPos,IF(_xlpm.pairFlag,INDEX(_xlpm.pairPositions,1,COLUMNS(_xlpm.pairPositions)),0),_xlpm.otherMask,(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.firstPos)*(_xlfn.SEQUENCE(,9)&lt;&gt;_xlpm.secondPos),_xlpm.hitMask,IF(_xlpm.pairFlag,_xlpm.otherMask*((ISNUMBER(SEARCH(LEFT(_xlpm.pairText,1),_xlpm.unitVals))+ISNUMBER(SEARCH(RIGHT(_xlpm.pairText,1),_xlpm.unitVals)))&gt;0),_xlfn.SEQUENCE(,9)=0),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlfn.SEQUENCE(,9),_xlpm.hitMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.sourceText,"R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;", R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos,_xlpm.displayText,"Naked pair in row · R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.firstPos&amp;" and R"&amp;_xlpm.rowNum&amp;"C"&amp;_xlpm.secondPos&amp;" contain only "&amp;LEFT(_xlpm.pairText,1)&amp;"/"&amp;RIGHT(_xlpm.pairText,1)&amp;" · Remove "&amp;LEFT(_xlpm.pairText,1)&amp;" and "&amp;RIGHT(_xlpm.pairText,1)&amp;" from "&amp;_xlpm.targetText&amp;".",IF(_xlpm.targetText&lt;&gt;"",_xlfn.HSTACK("Naked pair in row",_xlpm.sourceText,_xlpm.pairText,_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
+    <definedName name="SDKP_PointingCol">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_PointingColStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_PointingColStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.boxNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.digitNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.boxNum-1,3),_xlpm.boxStartCol,1+3*MOD(_xlpm.boxNum-1,3),_xlpm.boxCandidates,INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)),_xlpm.candidateMask,ISNUMBER(SEARCH(_xlpm.digitNum&amp;"",_xlpm.boxCandidates&amp;"")),_xlpm.candidateCount,SUM(--_xlpm.candidateMask),_xlpm.rowCoordinates,_xlfn.TOCOL(_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.rowOffset,_xlpm.colOffset,_xlpm.boxStartRow+_xlpm.rowOffset-1))),_xlpm.colCoordinates,_xlfn.TOCOL(_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.rowOffset,_xlpm.colOffset,_xlpm.boxStartCol+_xlpm.colOffset-1))),_xlpm.candidateCols,_xlfn._xlws.FILTER(_xlpm.colCoordinates,_xlfn.TOCOL(_xlpm.candidateMask),""),_xlpm.sourceCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoordinates&amp;"C"&amp;_xlpm.colCoordinates,_xlfn.TOCOL(_xlpm.candidateMask),""),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.sourceCells),_xlpm.singleCol,IF(_xlpm.candidateCount&gt;1,MIN(_xlpm.candidateCols)=MAX(_xlpm.candidateCols),FALSE),_xlpm.targetCol,IF(_xlpm.singleCol,INDEX(_xlpm.candidateCols,1),1),_xlpm.colCandidates,_xlfn.CHOOSECOLS(_xlpm.candMatrix,_xlpm.targetCol)&amp;"",_xlpm.rowNumbers,_xlfn.SEQUENCE(9),_xlpm.outsideMask,((_xlpm.rowNumbers&lt;_xlpm.boxStartRow)+(_xlpm.rowNumbers&gt;_xlpm.boxStartRow+2))&gt;0,_xlpm.containsMask,ISNUMBER(SEARCH(_xlpm.digitNum&amp;"",_xlpm.colCandidates)),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowNumbers&amp;"C"&amp;_xlpm.targetCol,_xlpm.outsideMask*_xlpm.containsMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.displayText,"Pointing column · Box "&amp;_xlpm.boxNum&amp;" confines digit "&amp;_xlpm.digitNum&amp;" to column "&amp;_xlpm.targetCol&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.digitNum&amp;" from "&amp;_xlpm.targetText&amp;".",IF(AND(_xlpm.singleCol,_xlpm.targetText&lt;&gt;""),_xlfn.HSTACK("Pointing column",_xlpm.sourceText,_xlpm.digitNum&amp;"",_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
+    <definedName name="SDKP_PointingRow">_xlfn.LAMBDA(_xlpm.inputCandidates,INDEX(SDKP_PointingRowStep(_xlpm.inputCandidates),1,5))</definedName>
+    <definedName name="SDKP_PointingRowStep">_xlfn.LAMBDA(_xlpm.inputCandidates,_xlfn.LET(_xlpm.candMatrix,_xlpm.inputCandidates,_xlpm.detect,_xlfn.LAMBDA(_xlpm.scanIndex,_xlfn.LET(_xlpm.boxNum,QUOTIENT(_xlpm.scanIndex-1,9)+1,_xlpm.digitNum,MOD(_xlpm.scanIndex-1,9)+1,_xlpm.boxStartRow,1+3*QUOTIENT(_xlpm.boxNum-1,3),_xlpm.boxStartCol,1+3*MOD(_xlpm.boxNum-1,3),_xlpm.boxCandidates,INDEX(_xlpm.candMatrix,_xlfn.SEQUENCE(3,,_xlpm.boxStartRow),_xlfn.SEQUENCE(,3,_xlpm.boxStartCol)),_xlpm.candidateMask,ISNUMBER(SEARCH(_xlpm.digitNum&amp;"",_xlpm.boxCandidates&amp;"")),_xlpm.candidateCount,SUM(--_xlpm.candidateMask),_xlpm.rowCoordinates,_xlfn.TOCOL(_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.rowOffset,_xlpm.colOffset,_xlpm.boxStartRow+_xlpm.rowOffset-1))),_xlpm.colCoordinates,_xlfn.TOCOL(_xlfn.MAKEARRAY(3,3,_xlfn.LAMBDA(_xlpm.rowOffset,_xlpm.colOffset,_xlpm.boxStartCol+_xlpm.colOffset-1))),_xlpm.candidateRows,_xlfn._xlws.FILTER(_xlpm.rowCoordinates,_xlfn.TOCOL(_xlpm.candidateMask),""),_xlpm.sourceCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.rowCoordinates&amp;"C"&amp;_xlpm.colCoordinates,_xlfn.TOCOL(_xlpm.candidateMask),""),_xlpm.sourceText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.sourceCells),_xlpm.singleRow,IF(_xlpm.candidateCount&gt;1,MIN(_xlpm.candidateRows)=MAX(_xlpm.candidateRows),FALSE),_xlpm.targetRow,IF(_xlpm.singleRow,INDEX(_xlpm.candidateRows,1),1),_xlpm.rowCandidates,_xlfn.CHOOSEROWS(_xlpm.candMatrix,_xlpm.targetRow)&amp;"",_xlpm.columnNumbers,_xlfn.SEQUENCE(,9),_xlpm.outsideMask,((_xlpm.columnNumbers&lt;_xlpm.boxStartCol)+(_xlpm.columnNumbers&gt;_xlpm.boxStartCol+2))&gt;0,_xlpm.containsMask,ISNUMBER(SEARCH(_xlpm.digitNum&amp;"",_xlpm.rowCandidates)),_xlpm.targetCells,_xlfn._xlws.FILTER("R"&amp;_xlpm.targetRow&amp;"C"&amp;_xlpm.columnNumbers,_xlpm.outsideMask*_xlpm.containsMask,""),_xlpm.targetText,_xlfn.TEXTJOIN(", ",TRUE,_xlpm.targetCells),_xlpm.displayText,"Pointing row · Box "&amp;_xlpm.boxNum&amp;" confines digit "&amp;_xlpm.digitNum&amp;" to row "&amp;_xlpm.targetRow&amp;" via "&amp;_xlpm.sourceText&amp;" · Remove "&amp;_xlpm.digitNum&amp;" from "&amp;_xlpm.targetText&amp;".",IF(AND(_xlpm.singleRow,_xlpm.targetText&lt;&gt;""),_xlfn.HSTACK("Pointing row",_xlpm.sourceText,_xlpm.digitNum&amp;"",_xlpm.targetText,_xlpm.displayText),_xlfn.HSTACK("","","","","")))),_xlpm.hits,_xlfn.MAP(_xlfn.SEQUENCE(81),_xlfn.LAMBDA(_xlpm.i,INDEX(_xlpm.detect(_xlpm.i),1,1)&lt;&gt;"")),_xlpm.p,IFERROR(_xlfn.XMATCH(TRUE,_xlpm.hits),0),IF(_xlpm.p=0,_xlfn.HSTACK("","","","",""),_xlpm.detect(_xlpm.p))))</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -133,7 +165,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -155,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="700">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -1741,12 +1773,6 @@
   </si>
   <si>
     <t>No solution-backed value is presented as logical deduction</t>
-  </si>
-  <si>
-    <t>All published engines use the player-safe Coach wrappers</t>
-  </si>
-  <si>
-    <t>Hint and Trace share the transparent fallback contract</t>
   </si>
   <si>
     <t>PLAYER-SAFE COACH FALLBACK</t>
@@ -2077,6 +2103,225 @@
   </si>
   <si>
     <t>Claiming row · Row 2 confines digit 3 to box 3 via R2C7, R2C8 · Remove 3 from R3C7.</t>
+  </si>
+  <si>
+    <t>All published engines use player-safe Coach paths</t>
+  </si>
+  <si>
+    <t>Four standard wrappers plus Master shared-chain fallback contract</t>
+  </si>
+  <si>
+    <t>STRUCTURED CANDIDATE CHAIN</t>
+  </si>
+  <si>
+    <t>Pointing-row step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Technique, sources, digits, targets and display text are separate</t>
+  </si>
+  <si>
+    <t>Structured apply ignores display wording</t>
+  </si>
+  <si>
+    <t>Targets and digits, not prose delimiters, drive removal</t>
+  </si>
+  <si>
+    <t>Structured Pointing slice preserves chain result</t>
+  </si>
+  <si>
+    <t>Master fixture still stops after two eliminations at R6C7 = 1</t>
+  </si>
+  <si>
+    <t>Pointing-column step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Duplicate forced singles in a row are contradictory</t>
+  </si>
+  <si>
+    <t>Two empty cells in row 1 are both forced to digit 1</t>
+  </si>
+  <si>
+    <t>Duplicate forced singles in a column are contradictory</t>
+  </si>
+  <si>
+    <t>Two empty cells in column 1 are both forced to digit 1</t>
+  </si>
+  <si>
+    <t>Duplicate forced singles in a box are contradictory</t>
+  </si>
+  <si>
+    <t>R1C1 and R2C2 force digit 1 in the same box only</t>
+  </si>
+  <si>
+    <t>Separated forced singles remain viable</t>
+  </si>
+  <si>
+    <t>R1C1 and R4C4 do not share a row, column or box</t>
+  </si>
+  <si>
+    <t>No-op elimination must not count as chain progress</t>
+  </si>
+  <si>
+    <t>Removing absent digit 9 leaves R1C1 candidates 12</t>
+  </si>
+  <si>
+    <t>Effective elimination counts as chain progress</t>
+  </si>
+  <si>
+    <t>Removing digit 1 changes R1C1 candidates 12 to 2</t>
+  </si>
+  <si>
+    <t>Candidate expansion must not count as progress</t>
+  </si>
+  <si>
+    <t>Growing R1C1 from 12 to 123 cannot continue the chain</t>
+  </si>
+  <si>
+    <t>Claiming-row step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Structured Claiming-row apply ignores display wording</t>
+  </si>
+  <si>
+    <t>Digit and target fields, not prose, remove 3 from R3C7</t>
+  </si>
+  <si>
+    <t>Claiming-row public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Public wrapper returns structured field 5</t>
+  </si>
+  <si>
+    <t>Claiming-column step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Structured Claiming-column apply ignores display wording</t>
+  </si>
+  <si>
+    <t>Digit and target fields, not prose, remove 3 from R7C3</t>
+  </si>
+  <si>
+    <t>Claiming-column public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Naked-pair-row step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Pair sources, digits, target and display text stay separate</t>
+  </si>
+  <si>
+    <t>Structured naked-pair-row apply ignores wording</t>
+  </si>
+  <si>
+    <t>Pair digits and target remove 4/7 from R4C7</t>
+  </si>
+  <si>
+    <t>Naked-pair-row public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Old entry returns structured display field</t>
+  </si>
+  <si>
+    <t>Three matching pairs do not form a naked pair</t>
+  </si>
+  <si>
+    <t>Exactly two matching cells are required</t>
+  </si>
+  <si>
+    <t>Naked-pair-column step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Structured naked-pair-column apply ignores wording</t>
+  </si>
+  <si>
+    <t>Pair digits and target remove 4/7 from R7C6</t>
+  </si>
+  <si>
+    <t>Naked-pair-column public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Three matching column pairs do not form a naked pair</t>
+  </si>
+  <si>
+    <t>Existing naked-pair-box wording maps off-diagonal cells</t>
+  </si>
+  <si>
+    <t>Pair sources and target are mapped in row order</t>
+  </si>
+  <si>
+    <t>Naked-pair-box step exposes structured action fields</t>
+  </si>
+  <si>
+    <t>Off-diagonal source pair and target stay separate</t>
+  </si>
+  <si>
+    <t>Structured naked-pair-box apply ignores wording</t>
+  </si>
+  <si>
+    <t>Pair digits remove 4/7 from R3C1</t>
+  </si>
+  <si>
+    <t>Naked-pair-box public wording remains compatible</t>
+  </si>
+  <si>
+    <t>Legacy entry returns the structured display field</t>
+  </si>
+  <si>
+    <t>Three matching box pairs do not form a naked pair</t>
+  </si>
+  <si>
+    <t>Exactly two matching box cells are required</t>
+  </si>
+  <si>
+    <t>Naked-pair-box step preserves middle-box identity</t>
+  </si>
+  <si>
+    <t>Box 5 maps off-diagonal pair to R6C4</t>
+  </si>
+  <si>
+    <t>Chain uses box elimination before the next assignment</t>
+  </si>
+  <si>
+    <t>Box pair removes 4/7 then reveals R3C1=8</t>
+  </si>
+  <si>
+    <t>Chain reports limit with pending elimination</t>
+  </si>
+  <si>
+    <t>Zero budget preserves candidates and pending box hint</t>
+  </si>
+  <si>
+    <t>Chain reports stable without applicable strategy</t>
+  </si>
+  <si>
+    <t>Full candidate matrix has no assignment or elimination</t>
+  </si>
+  <si>
+    <t>Chain reports contradiction for a dead cell</t>
+  </si>
+  <si>
+    <t>Empty R1C1 candidate stops before hint or elimination</t>
+  </si>
+  <si>
+    <t>Chain rebuilds candidates and hint after entry removal</t>
+  </si>
+  <si>
+    <t>R8C3 entry yields STABLE; blank board replays original assignment</t>
+  </si>
+  <si>
+    <t>Wrong entry stops guidance and removal restores the chain</t>
+  </si>
+  <si>
+    <t>Duplicate 1 flags both cells; clean board returns the original assignment</t>
+  </si>
+  <si>
+    <t>Chain enforces the eight-step boundary</t>
+  </si>
+  <si>
+    <t>Nine pointing patterns execute eight steps then retain the ninth as pending</t>
+  </si>
+  <si>
+    <t>Prototype Candidate Chain</t>
   </si>
 </sst>
 </file>
@@ -5038,6 +5283,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{FECC495D-41B9-7E46-A267-65DF3721832B}">
+  <we:reference id="wa200010215" version="2.0.0.1" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200010215" version="2.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="bps.codex_control.document_id" value="&quot;0c4a3077-fb42-4288-8e29-294003ec3652&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A9B5CCF-D0DB-3147-8E44-107C505B5881}">
   <sheetPr codeName="Sheet1">
@@ -5051,7 +5318,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="34" customHeight="1">
       <c r="A1" s="95" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B1" s="96"/>
       <c r="C1" s="96"/>
@@ -5065,7 +5332,7 @@
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
       <c r="A2" s="97" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B2" s="97"/>
       <c r="C2" s="97"/>
@@ -5200,7 +5467,7 @@
     </row>
     <row r="10" spans="1:10" ht="20" customHeight="1">
       <c r="A10" s="72" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B10" s="72"/>
       <c r="C10" s="72"/>
@@ -5214,7 +5481,7 @@
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1">
       <c r="A11" s="76" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B11" s="76"/>
       <c r="C11" s="76"/>
@@ -5256,7 +5523,7 @@
     </row>
     <row r="14" spans="1:10" ht="26" customHeight="1">
       <c r="A14" s="76" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B14" s="76"/>
       <c r="C14" s="76"/>
@@ -5284,7 +5551,7 @@
     </row>
     <row r="16" spans="1:10" ht="26" customHeight="1">
       <c r="A16" s="76" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="B16" s="76"/>
       <c r="C16" s="76"/>
@@ -5312,7 +5579,7 @@
     </row>
     <row r="18" spans="1:10" ht="30" customHeight="1">
       <c r="A18" s="76" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="B18" s="93"/>
       <c r="C18" s="93"/>
@@ -5352,7 +5619,7 @@
     </row>
     <row r="21" spans="1:10" ht="22" customHeight="1">
       <c r="A21" s="94" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B21" s="94"/>
       <c r="C21" s="94"/>
@@ -5366,7 +5633,7 @@
     </row>
     <row r="22" spans="1:10" ht="22" customHeight="1">
       <c r="A22" s="94" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B22" s="94"/>
       <c r="C22" s="94"/>
@@ -5380,7 +5647,7 @@
     </row>
     <row r="23" spans="1:10" ht="22" customHeight="1">
       <c r="A23" s="76" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B23" s="93"/>
       <c r="C23" s="93"/>
@@ -5394,7 +5661,7 @@
     </row>
     <row r="24" spans="1:10" ht="22" customHeight="1">
       <c r="A24" s="76" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B24" s="93"/>
       <c r="C24" s="93"/>
@@ -5408,7 +5675,7 @@
     </row>
     <row r="25" spans="1:10" ht="22" customHeight="1">
       <c r="A25" s="76" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B25" s="93"/>
       <c r="C25" s="93"/>
@@ -5422,7 +5689,7 @@
     </row>
     <row r="26" spans="1:10" ht="28" customHeight="1">
       <c r="A26" s="76" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="B26" s="93"/>
       <c r="C26" s="93"/>
@@ -5436,7 +5703,7 @@
     </row>
     <row r="27" spans="1:10" ht="34" customHeight="1">
       <c r="A27" s="103" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="B27" s="104"/>
       <c r="C27" s="104"/>
@@ -5476,7 +5743,7 @@
     </row>
     <row r="30" spans="1:10" ht="24" customHeight="1">
       <c r="A30" s="76" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B30" s="76"/>
       <c r="C30" s="76"/>
@@ -5490,7 +5757,7 @@
     </row>
     <row r="31" spans="1:10" ht="24" customHeight="1">
       <c r="A31" s="76" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B31" s="76"/>
       <c r="C31" s="76"/>
@@ -5504,7 +5771,7 @@
     </row>
     <row r="32" spans="1:10" ht="24" customHeight="1">
       <c r="A32" s="76" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="B32" s="76"/>
       <c r="C32" s="76"/>
@@ -5518,7 +5785,7 @@
     </row>
     <row r="33" spans="1:10" ht="24" customHeight="1">
       <c r="A33" s="76" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="B33" s="93"/>
       <c r="C33" s="93"/>
@@ -5532,7 +5799,7 @@
     </row>
     <row r="34" spans="1:10" ht="30" customHeight="1">
       <c r="A34" s="76" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="B34" s="93"/>
       <c r="C34" s="93"/>
@@ -5546,7 +5813,7 @@
     </row>
     <row r="35" spans="1:10" ht="30" customHeight="1">
       <c r="A35" s="76" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="B35" s="93"/>
       <c r="C35" s="93"/>
@@ -5624,7 +5891,7 @@
       <c r="B40" s="70"/>
       <c r="C40" s="70"/>
       <c r="D40" s="71" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E40" s="71"/>
       <c r="F40" s="71"/>
@@ -5656,7 +5923,7 @@
       <c r="B42" s="68"/>
       <c r="C42" s="68"/>
       <c r="D42" s="69" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E42" s="69"/>
       <c r="F42" s="69"/>
@@ -5679,7 +5946,7 @@
     </row>
     <row r="44" spans="1:10" ht="20" customHeight="1">
       <c r="A44" s="72" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B44" s="72"/>
       <c r="C44" s="72"/>
@@ -5693,13 +5960,13 @@
     </row>
     <row r="45" spans="1:10" ht="30" customHeight="1">
       <c r="A45" s="80" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B45" s="81"/>
       <c r="C45" s="81"/>
       <c r="D45" s="77" t="str">
         <f ca="1">COUNTIF(_Tests!$E:$E,"PASS")&amp;" checks passing · "&amp;COUNTIF(_Tests!$E:$E,"SKIP")&amp;" on demand"</f>
-        <v>93 checks passing · 18 on demand</v>
+        <v>131 checks passing · 18 on demand</v>
       </c>
       <c r="E45" s="78"/>
       <c r="F45" s="78"/>
@@ -5710,7 +5977,7 @@
     </row>
     <row r="46" spans="1:10" ht="30" customHeight="1">
       <c r="A46" s="80" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="B46" s="81"/>
       <c r="C46" s="81"/>
@@ -5752,7 +6019,7 @@
     </row>
     <row r="49" spans="1:10" ht="30" customHeight="1">
       <c r="A49" s="76" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="B49" s="76"/>
       <c r="C49" s="76"/>
@@ -5766,7 +6033,7 @@
     </row>
     <row r="50" spans="1:10" ht="26" customHeight="1">
       <c r="A50" s="76" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="B50" s="76"/>
       <c r="C50" s="76"/>
@@ -5780,7 +6047,7 @@
     </row>
     <row r="51" spans="1:10" ht="34" customHeight="1">
       <c r="A51" s="76" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B51" s="76"/>
       <c r="C51" s="76"/>
@@ -5806,7 +6073,7 @@
     </row>
     <row r="53" spans="1:10" ht="20" customHeight="1">
       <c r="A53" s="72" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="B53" s="72"/>
       <c r="C53" s="72"/>
@@ -5820,12 +6087,12 @@
     </row>
     <row r="54" spans="1:10" ht="24" customHeight="1">
       <c r="A54" s="73" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B54" s="73"/>
       <c r="C54" s="73"/>
       <c r="D54" s="74" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E54" s="74"/>
       <c r="F54" s="74"/>
@@ -5836,7 +6103,7 @@
     </row>
     <row r="55" spans="1:10" ht="24" customHeight="1">
       <c r="A55" s="70" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B55" s="70"/>
       <c r="C55" s="70"/>
@@ -5853,12 +6120,12 @@
     </row>
     <row r="56" spans="1:10" ht="24" customHeight="1">
       <c r="A56" s="70" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="B56" s="70"/>
       <c r="C56" s="70"/>
       <c r="D56" s="71" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="E56" s="71"/>
       <c r="F56" s="71"/>
@@ -5869,12 +6136,12 @@
     </row>
     <row r="57" spans="1:10" ht="24" customHeight="1">
       <c r="A57" s="70" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B57" s="70"/>
       <c r="C57" s="70"/>
       <c r="D57" s="71" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E57" s="71"/>
       <c r="F57" s="71"/>
@@ -5885,12 +6152,12 @@
     </row>
     <row r="58" spans="1:10" ht="30" customHeight="1">
       <c r="A58" s="68" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B58" s="68"/>
       <c r="C58" s="68"/>
       <c r="D58" s="69" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E58" s="69"/>
       <c r="F58" s="69"/>
@@ -5901,12 +6168,12 @@
     </row>
     <row r="59" spans="1:10" ht="30" customHeight="1">
       <c r="A59" s="68" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B59" s="68"/>
       <c r="C59" s="68"/>
       <c r="D59" s="69" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="E59" s="69"/>
       <c r="F59" s="69"/>
@@ -12851,7 +13118,7 @@
   <sheetPr codeName="Sheet13">
     <tabColor rgb="FF0B5A2B"/>
   </sheetPr>
-  <dimension ref="A1:T100"/>
+  <dimension ref="A1:T111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -13278,351 +13545,351 @@
     <row r="15" spans="1:10">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="str" cm="1">
-        <f t="array" ref="B15">SDK_Candidates($B$3:$J$11,1,1)</f>
+        <f t="array" ref="B15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C15" s="3" t="str" cm="1">
-        <f t="array" ref="C15">SDK_Candidates($B$3:$J$11,1,2)</f>
+        <f t="array" ref="C15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2568</v>
       </c>
       <c r="D15" s="3" t="str" cm="1">
-        <f t="array" ref="D15">SDK_Candidates($B$3:$J$11,1,3)</f>
+        <f t="array" ref="D15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2468</v>
       </c>
       <c r="E15" s="3" t="str" cm="1">
-        <f t="array" ref="E15">SDK_Candidates($B$3:$J$11,1,4)</f>
+        <f t="array" ref="E15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>458</v>
       </c>
       <c r="F15" s="3" t="str" cm="1">
-        <f t="array" ref="F15">SDK_Candidates($B$3:$J$11,1,5)</f>
+        <f t="array" ref="F15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>345</v>
       </c>
       <c r="G15" s="3" t="str" cm="1">
-        <f t="array" ref="G15">SDK_Candidates($B$3:$J$11,1,6)</f>
+        <f t="array" ref="G15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H15" s="3" t="str" cm="1">
-        <f t="array" ref="H15">SDK_Candidates($B$3:$J$11,1,7)</f>
+        <f t="array" ref="H15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>246</v>
       </c>
       <c r="I15" s="3" t="str" cm="1">
-        <f t="array" ref="I15">SDK_Candidates($B$3:$J$11,1,8)</f>
+        <f t="array" ref="I15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J15" s="3" t="str" cm="1">
-        <f t="array" ref="J15">SDK_Candidates($B$3:$J$11,1,9)</f>
+        <f t="array" ref="J15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>346</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="str" cm="1">
-        <f t="array" ref="B16">SDK_Candidates($B$3:$J$11,2,1)</f>
+        <f t="array" ref="B16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>457</v>
       </c>
       <c r="C16" s="3" t="str" cm="1">
-        <f t="array" ref="C16">SDK_Candidates($B$3:$J$11,2,2)</f>
+        <f t="array" ref="C16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D16" s="3" t="str" cm="1">
-        <f t="array" ref="D16">SDK_Candidates($B$3:$J$11,2,3)</f>
+        <f t="array" ref="D16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>46</v>
       </c>
       <c r="E16" s="3" t="str" cm="1">
-        <f t="array" ref="E16">SDK_Candidates($B$3:$J$11,2,4)</f>
+        <f t="array" ref="E16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1459</v>
       </c>
       <c r="F16" s="3" t="str" cm="1">
-        <f t="array" ref="F16">SDK_Candidates($B$3:$J$11,2,5)</f>
+        <f t="array" ref="F16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G16" s="3" t="str" cm="1">
-        <f t="array" ref="G16">SDK_Candidates($B$3:$J$11,2,6)</f>
+        <f t="array" ref="G16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>159</v>
       </c>
       <c r="H16" s="3" t="str" cm="1">
-        <f t="array" ref="H16">SDK_Candidates($B$3:$J$11,2,7)</f>
+        <f t="array" ref="H16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1467</v>
       </c>
       <c r="I16" s="3" t="str" cm="1">
-        <f t="array" ref="I16">SDK_Candidates($B$3:$J$11,2,8)</f>
+        <f t="array" ref="I16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>467</v>
       </c>
       <c r="J16" s="3" t="str" cm="1">
-        <f t="array" ref="J16">SDK_Candidates($B$3:$J$11,2,9)</f>
+        <f t="array" ref="J16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="str" cm="1">
-        <f t="array" ref="B17">SDK_Candidates($B$3:$J$11,3,1)</f>
+        <f t="array" ref="B17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2478</v>
       </c>
       <c r="C17" s="3" t="str" cm="1">
-        <f t="array" ref="C17">SDK_Candidates($B$3:$J$11,3,2)</f>
+        <f t="array" ref="C17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>278</v>
       </c>
       <c r="D17" s="3" t="str" cm="1">
-        <f t="array" ref="D17">SDK_Candidates($B$3:$J$11,3,3)</f>
+        <f t="array" ref="D17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E17" s="3" t="str" cm="1">
-        <f t="array" ref="E17">SDK_Candidates($B$3:$J$11,3,4)</f>
+        <f t="array" ref="E17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="str" cm="1">
-        <f t="array" ref="F17">SDK_Candidates($B$3:$J$11,3,5)</f>
+        <f t="array" ref="F17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>134</v>
       </c>
       <c r="G17" s="3" t="str" cm="1">
-        <f t="array" ref="G17">SDK_Candidates($B$3:$J$11,3,6)</f>
+        <f t="array" ref="G17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>138</v>
       </c>
       <c r="H17" s="3" t="str" cm="1">
-        <f t="array" ref="H17">SDK_Candidates($B$3:$J$11,3,7)</f>
+        <f t="array" ref="H17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I17" s="3" t="str" cm="1">
-        <f t="array" ref="I17">SDK_Candidates($B$3:$J$11,3,8)</f>
+        <f t="array" ref="I17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2347</v>
       </c>
       <c r="J17" s="3" t="str" cm="1">
-        <f t="array" ref="J17">SDK_Candidates($B$3:$J$11,3,9)</f>
+        <f t="array" ref="J17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="str" cm="1">
-        <f t="array" ref="B18">SDK_Candidates($B$3:$J$11,4,1)</f>
+        <f t="array" ref="B18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2478</v>
       </c>
       <c r="C18" s="3" t="str" cm="1">
-        <f t="array" ref="C18">SDK_Candidates($B$3:$J$11,4,2)</f>
+        <f t="array" ref="C18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>278</v>
       </c>
       <c r="D18" s="3" t="str" cm="1">
-        <f t="array" ref="D18">SDK_Candidates($B$3:$J$11,4,3)</f>
+        <f t="array" ref="D18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E18" s="3" t="str" cm="1">
-        <f t="array" ref="E18">SDK_Candidates($B$3:$J$11,4,4)</f>
+        <f t="array" ref="E18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="str" cm="1">
-        <f t="array" ref="F18">SDK_Candidates($B$3:$J$11,4,5)</f>
+        <f t="array" ref="F18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>167</v>
       </c>
       <c r="G18" s="3" t="str" cm="1">
-        <f t="array" ref="G18">SDK_Candidates($B$3:$J$11,4,6)</f>
+        <f t="array" ref="G18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>126</v>
       </c>
       <c r="H18" s="3" t="str" cm="1">
-        <f t="array" ref="H18">SDK_Candidates($B$3:$J$11,4,7)</f>
+        <f t="array" ref="H18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I18" s="3" t="str" cm="1">
-        <f t="array" ref="I18">SDK_Candidates($B$3:$J$11,4,8)</f>
+        <f t="array" ref="I18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4678</v>
       </c>
       <c r="J18" s="3" t="str" cm="1">
-        <f t="array" ref="J18">SDK_Candidates($B$3:$J$11,4,9)</f>
+        <f t="array" ref="J18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="str" cm="1">
-        <f t="array" ref="B19">SDK_Candidates($B$3:$J$11,5,1)</f>
+        <f t="array" ref="B19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>479</v>
       </c>
       <c r="C19" s="3" t="str" cm="1">
-        <f t="array" ref="C19">SDK_Candidates($B$3:$J$11,5,2)</f>
+        <f t="array" ref="C19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D19" s="3" t="str" cm="1">
-        <f t="array" ref="D19">SDK_Candidates($B$3:$J$11,5,3)</f>
+        <f t="array" ref="D19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>34</v>
       </c>
       <c r="E19" s="3" t="str" cm="1">
-        <f t="array" ref="E19">SDK_Candidates($B$3:$J$11,5,4)</f>
+        <f t="array" ref="E19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>579</v>
       </c>
       <c r="F19" s="3" t="str" cm="1">
-        <f t="array" ref="F19">SDK_Candidates($B$3:$J$11,5,5)</f>
+        <f t="array" ref="F19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G19" s="3" t="str" cm="1">
-        <f t="array" ref="G19">SDK_Candidates($B$3:$J$11,5,6)</f>
+        <f t="array" ref="G19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>569</v>
       </c>
       <c r="H19" s="3" t="str" cm="1">
-        <f t="array" ref="H19">SDK_Candidates($B$3:$J$11,5,7)</f>
+        <f t="array" ref="H19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>467</v>
       </c>
       <c r="I19" s="3" t="str" cm="1">
-        <f t="array" ref="I19">SDK_Candidates($B$3:$J$11,5,8)</f>
+        <f t="array" ref="I19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>34567</v>
       </c>
       <c r="J19" s="3" t="str" cm="1">
-        <f t="array" ref="J19">SDK_Candidates($B$3:$J$11,5,9)</f>
+        <f t="array" ref="J19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="str" cm="1">
-        <f t="array" ref="B20">SDK_Candidates($B$3:$J$11,6,1)</f>
+        <f t="array" ref="B20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C20" s="3" t="str" cm="1">
-        <f t="array" ref="C20">SDK_Candidates($B$3:$J$11,6,2)</f>
+        <f t="array" ref="C20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2789</v>
       </c>
       <c r="D20" s="3" t="str" cm="1">
-        <f t="array" ref="D20">SDK_Candidates($B$3:$J$11,6,3)</f>
+        <f t="array" ref="D20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>238</v>
       </c>
       <c r="E20" s="3" t="str" cm="1">
-        <f t="array" ref="E20">SDK_Candidates($B$3:$J$11,6,4)</f>
+        <f t="array" ref="E20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12579</v>
       </c>
       <c r="F20" s="3" t="str" cm="1">
-        <f t="array" ref="F20">SDK_Candidates($B$3:$J$11,6,5)</f>
+        <f t="array" ref="F20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1579</v>
       </c>
       <c r="G20" s="3" t="str" cm="1">
-        <f t="array" ref="G20">SDK_Candidates($B$3:$J$11,6,6)</f>
+        <f t="array" ref="G20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H20" s="3" t="str" cm="1">
-        <f t="array" ref="H20">SDK_Candidates($B$3:$J$11,6,7)</f>
+        <f t="array" ref="H20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>178</v>
       </c>
       <c r="I20" s="3" t="str" cm="1">
-        <f t="array" ref="I20">SDK_Candidates($B$3:$J$11,6,8)</f>
+        <f t="array" ref="I20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3578</v>
       </c>
       <c r="J20" s="3" t="str" cm="1">
-        <f t="array" ref="J20">SDK_Candidates($B$3:$J$11,6,9)</f>
+        <f t="array" ref="J20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="str" cm="1">
-        <f t="array" ref="B21">SDK_Candidates($B$3:$J$11,7,1)</f>
+        <f t="array" ref="B21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C21" s="3" t="str" cm="1">
-        <f t="array" ref="C21">SDK_Candidates($B$3:$J$11,7,2)</f>
+        <f t="array" ref="C21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>25689</v>
       </c>
       <c r="D21" s="3" t="str" cm="1">
-        <f t="array" ref="D21">SDK_Candidates($B$3:$J$11,7,3)</f>
+        <f t="array" ref="D21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>268</v>
       </c>
       <c r="E21" s="3" t="str" cm="1">
-        <f t="array" ref="E21">SDK_Candidates($B$3:$J$11,7,4)</f>
+        <f t="array" ref="E21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>245789</v>
       </c>
       <c r="F21" s="3" t="str" cm="1">
-        <f t="array" ref="F21">SDK_Candidates($B$3:$J$11,7,5)</f>
+        <f t="array" ref="F21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>45679</v>
       </c>
       <c r="G21" s="3" t="str" cm="1">
-        <f t="array" ref="G21">SDK_Candidates($B$3:$J$11,7,6)</f>
+        <f t="array" ref="G21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>25689</v>
       </c>
       <c r="H21" s="3" t="str" cm="1">
-        <f t="array" ref="H21">SDK_Candidates($B$3:$J$11,7,7)</f>
+        <f t="array" ref="H21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2468</v>
       </c>
       <c r="I21" s="3" t="str" cm="1">
-        <f t="array" ref="I21">SDK_Candidates($B$3:$J$11,7,8)</f>
+        <f t="array" ref="I21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J21" s="3" t="str" cm="1">
-        <f t="array" ref="J21">SDK_Candidates($B$3:$J$11,7,9)</f>
+        <f t="array" ref="J21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4569</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="str" cm="1">
-        <f t="array" ref="B22">SDK_Candidates($B$3:$J$11,8,1)</f>
+        <f t="array" ref="B22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2589</v>
       </c>
       <c r="C22" s="3" t="str" cm="1">
-        <f t="array" ref="C22">SDK_Candidates($B$3:$J$11,8,2)</f>
+        <f t="array" ref="C22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D22" s="3" t="str" cm="1">
-        <f t="array" ref="D22">SDK_Candidates($B$3:$J$11,8,3)</f>
+        <f t="array" ref="D22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1268</v>
       </c>
       <c r="E22" s="3" t="str" cm="1">
-        <f t="array" ref="E22">SDK_Candidates($B$3:$J$11,8,4)</f>
+        <f t="array" ref="E22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12589</v>
       </c>
       <c r="F22" s="3" t="str" cm="1">
-        <f t="array" ref="F22">SDK_Candidates($B$3:$J$11,8,5)</f>
+        <f t="array" ref="F22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13569</v>
       </c>
       <c r="G22" s="3" t="str" cm="1">
-        <f t="array" ref="G22">SDK_Candidates($B$3:$J$11,8,6)</f>
+        <f t="array" ref="G22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1235689</v>
       </c>
       <c r="H22" s="3" t="str" cm="1">
-        <f t="array" ref="H22">SDK_Candidates($B$3:$J$11,8,7)</f>
+        <f t="array" ref="H22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>268</v>
       </c>
       <c r="I22" s="3" t="str" cm="1">
-        <f t="array" ref="I22">SDK_Candidates($B$3:$J$11,8,8)</f>
+        <f t="array" ref="I22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2568</v>
       </c>
       <c r="J22" s="3" t="str" cm="1">
-        <f t="array" ref="J22">SDK_Candidates($B$3:$J$11,8,9)</f>
+        <f t="array" ref="J22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="str" cm="1">
-        <f t="array" ref="B23">SDK_Candidates($B$3:$J$11,9,1)</f>
+        <f t="array" ref="B23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2589</v>
       </c>
       <c r="C23" s="3" t="str" cm="1">
-        <f t="array" ref="C23">SDK_Candidates($B$3:$J$11,9,2)</f>
+        <f t="array" ref="C23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>25689</v>
       </c>
       <c r="D23" s="3" t="str" cm="1">
-        <f t="array" ref="D23">SDK_Candidates($B$3:$J$11,9,3)</f>
+        <f t="array" ref="D23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E23" s="3" t="str" cm="1">
-        <f t="array" ref="E23">SDK_Candidates($B$3:$J$11,9,4)</f>
+        <f t="array" ref="E23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>124589</v>
       </c>
       <c r="F23" s="3" t="str" cm="1">
-        <f t="array" ref="F23">SDK_Candidates($B$3:$J$11,9,5)</f>
+        <f t="array" ref="F23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>14569</v>
       </c>
       <c r="G23" s="3" t="str" cm="1">
-        <f t="array" ref="G23">SDK_Candidates($B$3:$J$11,9,6)</f>
+        <f t="array" ref="G23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>125689</v>
       </c>
       <c r="H23" s="3" t="str" cm="1">
-        <f t="array" ref="H23">SDK_Candidates($B$3:$J$11,9,7)</f>
+        <f t="array" ref="H23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I23" s="3" t="str" cm="1">
-        <f t="array" ref="I23">SDK_Candidates($B$3:$J$11,9,8)</f>
+        <f t="array" ref="I23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>24568</v>
       </c>
       <c r="J23" s="3" t="str" cm="1">
-        <f t="array" ref="J23">SDK_Candidates($B$3:$J$11,9,9)</f>
+        <f t="array" ref="J23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4569</v>
       </c>
     </row>
@@ -14790,7 +15057,7 @@
         <v>74</v>
       </c>
       <c r="B88" s="7" t="str" cm="1">
-        <f t="array" ref="B88">IF(OR('05 Master'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",SDK_PlayerHint($B$3:$J$11,$B$39:$J$47))</f>
+        <f t="array" ref="B88">IF(OR('05 Master'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",IF($L$111="ASSIGNMENT",$N$111,IF($L$111="LIMIT","Candidate chain limit reached after "&amp;$M$111&amp;" elimination step(s).",IF($L$111="CONTRADICTION","Candidate chain contradiction detected.",SDK_FallbackReveal($B$3:$J$11,$B$39:$J$47)))))</f>
         <v>Hidden single in column · R8C3 = 1 · Digit 1 appears in only one candidate set in column 3.</v>
       </c>
       <c r="C88" s="7"/>
@@ -14816,8 +15083,8 @@
       <c r="A89" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B89" s="7" t="str" cm="1">
-        <f t="array" ref="B89">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),1)</f>
+      <c r="B89" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;1,"Technique — "&amp;INDEX(_xlpm.parts,1,1)&amp;" | Pattern — "&amp;INDEX(_xlpm.parts,1,2),"Status — "&amp;INDEX(_xlpm.parts,1,1))))</f>
         <v>Technique — Hidden single in column | Pattern — R8C3 = 1</v>
       </c>
       <c r="C89" s="7"/>
@@ -14845,8 +15112,8 @@
       <c r="A90" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B90" s="7" t="str" cm="1">
-        <f t="array" ref="B90">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),2)</f>
+      <c r="B90" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;2,"Action — "&amp;_xlfn.TEXTJOIN(" · ",TRUE,_xlfn.DROP(_xlpm.parts,,2)),"Action — No further supported step.")))</f>
         <v>Action — Digit 1 appears in only one candidate set in column 3.</v>
       </c>
       <c r="C90" s="7"/>
@@ -15097,6 +15364,302 @@
       </c>
       <c r="B100" t="str" cm="1">
         <f t="array" ref="B100">IF('05 Master'!$AS$11="Verify",IF(COUNTIF($B$51:$J$59,TRUE)&gt;0,"CONFLICT",SDK_SolveStatus($B$3:$J$11)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="1:20">
+      <c r="L101" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="102" spans="1:20">
+      <c r="L102" t="str" cm="1">
+        <f t="array" ref="L102:T111">SDKP_Chain($B$3:$J$11,8)</f>
+        <v/>
+      </c>
+      <c r="M102" t="str">
+        <v>2568</v>
+      </c>
+      <c r="N102" t="str">
+        <v>2468</v>
+      </c>
+      <c r="O102" t="str">
+        <v>458</v>
+      </c>
+      <c r="P102" t="str">
+        <v>345</v>
+      </c>
+      <c r="Q102" t="str">
+        <v/>
+      </c>
+      <c r="R102" t="str">
+        <v>246</v>
+      </c>
+      <c r="S102" t="str">
+        <v/>
+      </c>
+      <c r="T102" t="str">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="103" spans="1:20">
+      <c r="L103" t="str">
+        <v>457</v>
+      </c>
+      <c r="M103" t="str">
+        <v/>
+      </c>
+      <c r="N103" t="str">
+        <v>46</v>
+      </c>
+      <c r="O103" t="str">
+        <v>1459</v>
+      </c>
+      <c r="P103" t="str">
+        <v/>
+      </c>
+      <c r="Q103" t="str">
+        <v>159</v>
+      </c>
+      <c r="R103" t="str">
+        <v>1467</v>
+      </c>
+      <c r="S103" t="str">
+        <v>467</v>
+      </c>
+      <c r="T103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104" spans="1:20">
+      <c r="L104" t="str">
+        <v>2478</v>
+      </c>
+      <c r="M104" t="str">
+        <v>278</v>
+      </c>
+      <c r="N104" t="str">
+        <v/>
+      </c>
+      <c r="O104" t="str">
+        <v/>
+      </c>
+      <c r="P104" t="str">
+        <v>134</v>
+      </c>
+      <c r="Q104" t="str">
+        <v>138</v>
+      </c>
+      <c r="R104" t="str">
+        <v/>
+      </c>
+      <c r="S104" t="str">
+        <v>2347</v>
+      </c>
+      <c r="T104" t="str">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="105" spans="1:20">
+      <c r="L105" t="str">
+        <v>2478</v>
+      </c>
+      <c r="M105" t="str">
+        <v>278</v>
+      </c>
+      <c r="N105" t="str">
+        <v/>
+      </c>
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v>167</v>
+      </c>
+      <c r="Q105" t="str">
+        <v>126</v>
+      </c>
+      <c r="R105" t="str">
+        <v/>
+      </c>
+      <c r="S105" t="str">
+        <v>4678</v>
+      </c>
+      <c r="T105" t="str">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="106" spans="1:20">
+      <c r="L106" t="str">
+        <v>479</v>
+      </c>
+      <c r="M106" t="str">
+        <v/>
+      </c>
+      <c r="N106" t="str">
+        <v>34</v>
+      </c>
+      <c r="O106" t="str">
+        <v>579</v>
+      </c>
+      <c r="P106" t="str">
+        <v/>
+      </c>
+      <c r="Q106" t="str">
+        <v>569</v>
+      </c>
+      <c r="R106" t="str">
+        <v>467</v>
+      </c>
+      <c r="S106" t="str">
+        <v>34567</v>
+      </c>
+      <c r="T106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107" spans="1:20">
+      <c r="L107" t="str">
+        <v/>
+      </c>
+      <c r="M107" t="str">
+        <v>2789</v>
+      </c>
+      <c r="N107" t="str">
+        <v>238</v>
+      </c>
+      <c r="O107" t="str">
+        <v>12579</v>
+      </c>
+      <c r="P107" t="str">
+        <v>1579</v>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107" t="str">
+        <v>178</v>
+      </c>
+      <c r="S107" t="str">
+        <v>3578</v>
+      </c>
+      <c r="T107" t="str">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="108" spans="1:20">
+      <c r="L108" t="str">
+        <v/>
+      </c>
+      <c r="M108" t="str">
+        <v>25689</v>
+      </c>
+      <c r="N108" t="str">
+        <v>268</v>
+      </c>
+      <c r="O108" t="str">
+        <v>245789</v>
+      </c>
+      <c r="P108" t="str">
+        <v>45679</v>
+      </c>
+      <c r="Q108" t="str">
+        <v>25689</v>
+      </c>
+      <c r="R108" t="str">
+        <v>2468</v>
+      </c>
+      <c r="S108" t="str">
+        <v/>
+      </c>
+      <c r="T108" t="str">
+        <v>4569</v>
+      </c>
+    </row>
+    <row r="109" spans="1:20">
+      <c r="L109" t="str">
+        <v>2589</v>
+      </c>
+      <c r="M109" t="str">
+        <v/>
+      </c>
+      <c r="N109" t="str">
+        <v>1268</v>
+      </c>
+      <c r="O109" t="str">
+        <v>12589</v>
+      </c>
+      <c r="P109" t="str">
+        <v>13569</v>
+      </c>
+      <c r="Q109" t="str">
+        <v>1235689</v>
+      </c>
+      <c r="R109" t="str">
+        <v>268</v>
+      </c>
+      <c r="S109" t="str">
+        <v>2568</v>
+      </c>
+      <c r="T109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110" spans="1:20">
+      <c r="L110" t="str">
+        <v>2589</v>
+      </c>
+      <c r="M110" t="str">
+        <v>25689</v>
+      </c>
+      <c r="N110" t="str">
+        <v/>
+      </c>
+      <c r="O110" t="str">
+        <v>124589</v>
+      </c>
+      <c r="P110" t="str">
+        <v>14569</v>
+      </c>
+      <c r="Q110" t="str">
+        <v>125689</v>
+      </c>
+      <c r="R110" t="str">
+        <v/>
+      </c>
+      <c r="S110" t="str">
+        <v>24568</v>
+      </c>
+      <c r="T110" t="str">
+        <v>4569</v>
+      </c>
+    </row>
+    <row r="111" spans="1:20">
+      <c r="L111" t="str">
+        <v>ASSIGNMENT</v>
+      </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111" t="str">
+        <v>Hidden single in column · R8C3 = 1 · Digit 1 appears in only one candidate set in column 3.</v>
+      </c>
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
+      <c r="S111" t="str">
+        <v/>
+      </c>
+      <c r="T111" t="str">
         <v/>
       </c>
     </row>
@@ -15146,7 +15709,7 @@
   <sheetData>
     <row r="1" spans="2:61" ht="27" customHeight="1">
       <c r="B1" s="113" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C1" s="113"/>
       <c r="D1" s="113"/>
@@ -19368,7 +19931,7 @@
   <sheetData>
     <row r="1" spans="2:61" ht="27" customHeight="1">
       <c r="B1" s="113" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="C1" s="113"/>
       <c r="D1" s="113"/>
@@ -23610,7 +24173,7 @@
   <sheetData>
     <row r="1" spans="2:61" ht="27" customHeight="1">
       <c r="B1" s="113" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C1" s="113"/>
       <c r="D1" s="113"/>
@@ -27828,7 +28391,7 @@
   <sheetData>
     <row r="1" spans="2:61" ht="27" customHeight="1">
       <c r="B1" s="113" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C1" s="113"/>
       <c r="D1" s="113"/>
@@ -32043,7 +32606,7 @@
   <sheetData>
     <row r="1" spans="2:61" ht="27" customHeight="1">
       <c r="B1" s="113" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C1" s="113"/>
       <c r="D1" s="113"/>
@@ -36232,7 +36795,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="27" customHeight="1" thickBot="1">
       <c r="A1" s="119" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="B1" s="120"/>
       <c r="C1" s="120"/>
@@ -36242,7 +36805,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1">
       <c r="A2" s="122" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="B2" s="122"/>
       <c r="C2" s="122"/>
@@ -36268,7 +36831,7 @@
     </row>
     <row r="5" spans="1:6" ht="22" customHeight="1">
       <c r="A5" s="124" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B5" s="124"/>
       <c r="C5" s="124"/>
@@ -37255,7 +37818,7 @@
         <v>511</v>
       </c>
       <c r="D63" s="66" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="E63" s="66" t="s">
         <v>512</v>
@@ -37294,7 +37857,7 @@
     </row>
     <row r="66" spans="1:6" ht="19" customHeight="1">
       <c r="A66" s="121" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="B66" s="121"/>
       <c r="C66" s="121"/>
@@ -37304,73 +37867,73 @@
     </row>
     <row r="67" spans="1:6" ht="42">
       <c r="A67" s="67" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="B67" s="66" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C67" s="66" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="66" t="s">
+        <v>528</v>
+      </c>
+      <c r="E67" s="66" t="s">
+        <v>529</v>
+      </c>
+      <c r="F67" s="66" t="s">
         <v>530</v>
-      </c>
-      <c r="E67" s="66" t="s">
-        <v>531</v>
-      </c>
-      <c r="F67" s="66" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="68" spans="1:6" ht="42">
       <c r="A68" s="67" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B68" s="66" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C68" s="66" t="s">
         <v>14</v>
       </c>
       <c r="D68" s="66" t="s">
+        <v>533</v>
+      </c>
+      <c r="E68" s="66" t="s">
+        <v>534</v>
+      </c>
+      <c r="F68" s="66" t="s">
         <v>535</v>
-      </c>
-      <c r="E68" s="66" t="s">
-        <v>536</v>
-      </c>
-      <c r="F68" s="66" t="s">
-        <v>537</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="28">
       <c r="A69" s="67" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B69" s="66" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C69" s="66" t="s">
         <v>14</v>
       </c>
       <c r="D69" s="66" t="s">
+        <v>538</v>
+      </c>
+      <c r="E69" s="66" t="s">
+        <v>539</v>
+      </c>
+      <c r="F69" s="66" t="s">
         <v>540</v>
-      </c>
-      <c r="E69" s="66" t="s">
-        <v>541</v>
-      </c>
-      <c r="F69" s="66" t="s">
-        <v>542</v>
       </c>
     </row>
     <row r="70" spans="1:6" ht="28">
       <c r="A70" s="67" t="s">
+        <v>541</v>
+      </c>
+      <c r="B70" s="66" t="s">
+        <v>542</v>
+      </c>
+      <c r="C70" s="66" t="s">
         <v>543</v>
-      </c>
-      <c r="B70" s="66" t="s">
-        <v>544</v>
-      </c>
-      <c r="C70" s="66" t="s">
-        <v>545</v>
       </c>
       <c r="D70" s="66" t="s">
         <v>256</v>
@@ -37379,7 +37942,7 @@
         <v>479</v>
       </c>
       <c r="F70" s="66" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
     </row>
   </sheetData>
@@ -37410,7 +37973,7 @@
   <sheetPr codeName="Sheet8">
     <tabColor rgb="FFA5A5A5"/>
   </sheetPr>
-  <dimension ref="A1:P162"/>
+  <dimension ref="A1:P202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -37680,7 +38243,7 @@
         <v>90</v>
       </c>
       <c r="C18" s="40" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D18" s="40" t="str" cm="1">
         <f t="array" ref="D18">SDK_PointingRowHint(_Engine!$B$27:$J$35)</f>
@@ -37699,7 +38262,7 @@
         <v>92</v>
       </c>
       <c r="C19" s="38" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D19" s="38" t="str" cm="1">
         <f t="array" ref="D19">SDK_HintClaiming(_Engine!$B$27:$J$35)</f>
@@ -39986,24 +40549,24 @@
     </row>
     <row r="138" spans="1:5">
       <c r="A138" t="s">
+        <v>597</v>
+      </c>
+      <c r="B138" t="s">
+        <v>598</v>
+      </c>
+      <c r="E138" t="s">
         <v>599</v>
-      </c>
-      <c r="B138" t="s">
-        <v>600</v>
-      </c>
-      <c r="E138" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="139" spans="1:5">
       <c r="A139" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B139" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E139" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -40089,16 +40652,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>525</v>
+        <v>627</v>
       </c>
       <c r="B145" t="s">
-        <v>526</v>
+        <v>628</v>
       </c>
       <c r="C145" t="b">
         <v>1</v>
       </c>
       <c r="D145" t="b">
-        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
+        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
         <v>1</v>
       </c>
       <c r="E145" t="str">
@@ -40108,10 +40671,10 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B146" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C146" t="b">
         <v>1</v>
@@ -40127,15 +40690,15 @@
     </row>
     <row r="147" spans="1:5">
       <c r="A147" s="54" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
     </row>
     <row r="148" spans="1:5">
       <c r="A148" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="B148" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C148" t="b">
         <v>1</v>
@@ -40151,15 +40714,15 @@
     </row>
     <row r="149" spans="1:5">
       <c r="A149" s="54" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="150" spans="1:5">
       <c r="A150" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B150" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C150" t="b">
         <v>1</v>
@@ -40175,10 +40738,10 @@
     </row>
     <row r="151" spans="1:5">
       <c r="A151" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B151" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C151" t="b">
         <v>1</v>
@@ -40194,10 +40757,10 @@
     </row>
     <row r="152" spans="1:5">
       <c r="A152" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B152" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C152" t="b">
         <v>1</v>
@@ -40213,10 +40776,10 @@
     </row>
     <row r="153" spans="1:5">
       <c r="A153" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B153" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C153" t="b">
         <v>1</v>
@@ -40232,10 +40795,10 @@
     </row>
     <row r="154" spans="1:5">
       <c r="A154" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B154" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C154" t="b">
         <v>1</v>
@@ -40251,10 +40814,10 @@
     </row>
     <row r="155" spans="1:5">
       <c r="A155" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B155" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C155" t="b">
         <v>1</v>
@@ -40270,10 +40833,10 @@
     </row>
     <row r="156" spans="1:5">
       <c r="A156" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B156" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C156" t="b">
         <v>1</v>
@@ -40289,10 +40852,10 @@
     </row>
     <row r="157" spans="1:5">
       <c r="A157" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B157" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C157" t="b">
         <v>1</v>
@@ -40308,10 +40871,10 @@
     </row>
     <row r="158" spans="1:5">
       <c r="A158" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="B158" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C158" t="b">
         <v>1</v>
@@ -40327,10 +40890,10 @@
     </row>
     <row r="159" spans="1:5">
       <c r="A159" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B159" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="C159" t="b">
         <v>1</v>
@@ -40346,10 +40909,10 @@
     </row>
     <row r="160" spans="1:5">
       <c r="A160" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="B160" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="C160" t="b">
         <v>1</v>
@@ -40365,10 +40928,10 @@
     </row>
     <row r="161" spans="1:5">
       <c r="A161" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="B161" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C161" t="b">
         <v>1</v>
@@ -40384,10 +40947,10 @@
     </row>
     <row r="162" spans="1:5">
       <c r="A162" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B162" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="C162" t="b">
         <v>1</v>
@@ -40398,6 +40961,751 @@
       </c>
       <c r="E162" t="str">
         <f>IF(D162=C162,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5">
+      <c r="A164" s="54" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5">
+      <c r="A165" t="s">
+        <v>630</v>
+      </c>
+      <c r="B165" t="s">
+        <v>631</v>
+      </c>
+      <c r="C165" t="b">
+        <v>1</v>
+      </c>
+      <c r="D165" t="b" cm="1">
+        <f t="array" ref="D165">IFERROR(_xlfn.LET(_xlpm.b,'_Engine Master'!$B$27:$J$35,_xlpm.a,SDK_SetCell(_xlpm.b,8,3,1),_xlpm.c,SDK_SetCell(_xlpm.a,1,2,6),_xlpm.d,SDK_SetCell(_xlpm.c,2,3,4),_xlpm.e,SDK_SetCell(_xlpm.d,5,3,3),_xlpm.f,SDK_SetCell(_xlpm.e,7,3,6),_xlpm.g,SDK_SetCell(_xlpm.f,2,1,5),_xlpm.s,SDKP_PointingRowStep(SDK_CandidateMatrix(_xlpm.g)),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Pointing row",INDEX(_xlpm.s,1,2)="R3C1, R3C2",INDEX(_xlpm.s,1,3)="7",INDEX(_xlpm.s,1,4)="R3C8",INDEX(_xlpm.s,1,5)="Pointing row · Box 1 confines digit 7 to row 3 via R3C1, R3C2 · Remove 7 from R3C8."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E165" t="str">
+        <f t="shared" ref="E165:E202" si="8">IF(D165=C165,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5">
+      <c r="A166" t="s">
+        <v>632</v>
+      </c>
+      <c r="B166" t="s">
+        <v>633</v>
+      </c>
+      <c r="C166" t="b">
+        <v>1</v>
+      </c>
+      <c r="D166" t="b">
+        <f>IFERROR(_xlfn.LET(_xlpm.b,'_Engine Master'!$B$27:$J$35,_xlpm.a,SDK_SetCell(_xlpm.b,8,3,1),_xlpm.c,SDK_SetCell(_xlpm.a,1,2,6),_xlpm.d,SDK_SetCell(_xlpm.c,2,3,4),_xlpm.e,SDK_SetCell(_xlpm.d,5,3,3),_xlpm.f,SDK_SetCell(_xlpm.e,7,3,6),_xlpm.g,SDK_SetCell(_xlpm.f,2,1,5),_xlpm.cands,SDK_CandidateMatrix(_xlpm.g),_xlpm.s,_xlfn.HSTACK("Pointing row","R3C1, R3C2","7","R3C8","wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.cands,_xlpm.s),INDEX(_xlpm.after,3,8)="234"),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E166" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5">
+      <c r="A167" t="s">
+        <v>634</v>
+      </c>
+      <c r="B167" t="s">
+        <v>635</v>
+      </c>
+      <c r="C167" t="b">
+        <v>1</v>
+      </c>
+      <c r="D167" t="b" cm="1">
+        <f t="array" ref="D167">IFERROR(_xlfn.LET(_xlpm.b,'_Engine Master'!$B$27:$J$35,_xlpm.a,SDK_SetCell(_xlpm.b,8,3,1),_xlpm.c,SDK_SetCell(_xlpm.a,1,2,6),_xlpm.d,SDK_SetCell(_xlpm.c,2,3,4),_xlpm.e,SDK_SetCell(_xlpm.d,5,3,3),_xlpm.f,SDK_SetCell(_xlpm.e,7,3,6),_xlpm.g,SDK_SetCell(_xlpm.f,2,1,5),_xlpm.chain,SDKP_Chain(_xlpm.g,8),SUM(--_xlfn.HSTACK(INDEX(_xlpm.chain,3,8)="234",INDEX(_xlpm.chain,2,7)="67",INDEX(_xlpm.chain,10,1)="ASSIGNMENT",INDEX(_xlpm.chain,10,2)=2,INDEX(_xlpm.chain,10,3)="Hidden single in column · R6C7 = 1 · Digit 1 appears in only one candidate set in column 7."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E167" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5">
+      <c r="A168" t="s">
+        <v>636</v>
+      </c>
+      <c r="B168" t="s">
+        <v>631</v>
+      </c>
+      <c r="C168" t="b">
+        <f>TRUE</f>
+        <v>1</v>
+      </c>
+      <c r="D168" t="b" cm="1">
+        <f t="array" ref="D168">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=3),"7",AND(_xlpm.r=2,_xlpm.k=3),"7",AND(_xlpm.r=8,_xlpm.k=3),"27",TRUE,""))),_xlpm.s,SDKP_PointingColStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Pointing column",INDEX(_xlpm.s,1,2)="R1C3, R2C3",INDEX(_xlpm.s,1,3)="7",INDEX(_xlpm.s,1,4)="R8C3",INDEX(_xlpm.s,1,5)="Pointing column · Box 1 confines digit 7 to column 3 via R1C3, R2C3 · Remove 7 from R8C3."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E168" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5">
+      <c r="A169" t="s">
+        <v>637</v>
+      </c>
+      <c r="B169" t="s">
+        <v>638</v>
+      </c>
+      <c r="C169" t="b">
+        <v>1</v>
+      </c>
+      <c r="D169" t="b" cm="1">
+        <f t="array" ref="D169">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,OR(_xlpm.k=1,_xlpm.k=2)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>1</v>
+      </c>
+      <c r="E169" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5">
+      <c r="A170" t="s">
+        <v>639</v>
+      </c>
+      <c r="B170" t="s">
+        <v>640</v>
+      </c>
+      <c r="C170" t="b">
+        <v>1</v>
+      </c>
+      <c r="D170" t="b" cm="1">
+        <f t="array" ref="D170">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.k=1,OR(_xlpm.r=1,_xlpm.r=2)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>1</v>
+      </c>
+      <c r="E170" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5">
+      <c r="A171" t="s">
+        <v>641</v>
+      </c>
+      <c r="B171" t="s">
+        <v>642</v>
+      </c>
+      <c r="C171" t="b">
+        <v>1</v>
+      </c>
+      <c r="D171" t="b" cm="1">
+        <f t="array" ref="D171">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(OR(AND(_xlpm.r=1,_xlpm.k=1),AND(_xlpm.r=2,_xlpm.k=2)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>1</v>
+      </c>
+      <c r="E171" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5">
+      <c r="A172" t="s">
+        <v>643</v>
+      </c>
+      <c r="B172" t="s">
+        <v>644</v>
+      </c>
+      <c r="C172" t="b">
+        <v>0</v>
+      </c>
+      <c r="D172" t="b" cm="1">
+        <f t="array" ref="D172">_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.cand,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(OR(AND(_xlpm.r=1,_xlpm.k=1),AND(_xlpm.r=4,_xlpm.k=4)),"1","123456789"))),SDKP_Contradiction(_xlpm.board,_xlpm.cand))</f>
+        <v>0</v>
+      </c>
+      <c r="E172" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5">
+      <c r="A173" t="s">
+        <v>645</v>
+      </c>
+      <c r="B173" t="s">
+        <v>646</v>
+      </c>
+      <c r="C173" t="b">
+        <v>1</v>
+      </c>
+      <c r="D173" t="b" cm="1">
+        <f t="array" ref="D173">_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"12",""))),_xlpm.s,_xlfn.HSTACK("Pointing row","R1C2","9","R1C1","probe"),_xlpm.next,SDKP_ApplyStep(_xlpm.c,_xlpm.s),IFERROR(AND(INDEX(_xlpm.next,1,1)="12",NOT(SDKP_HasProgress(_xlpm.c,_xlpm.next))),FALSE))</f>
+        <v>1</v>
+      </c>
+      <c r="E173" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5">
+      <c r="A174" t="s">
+        <v>647</v>
+      </c>
+      <c r="B174" t="s">
+        <v>648</v>
+      </c>
+      <c r="C174" t="b">
+        <v>1</v>
+      </c>
+      <c r="D174" t="b" cm="1">
+        <f t="array" ref="D174">_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"12",""))),_xlpm.s,_xlfn.HSTACK("Pointing row","R1C2","1","R1C1","probe"),_xlpm.next,SDKP_ApplyStep(_xlpm.c,_xlpm.s),IFERROR(AND(INDEX(_xlpm.next,1,1)="2",SDKP_HasProgress(_xlpm.c,_xlpm.next)),FALSE))</f>
+        <v>1</v>
+      </c>
+      <c r="E174" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5">
+      <c r="A175" t="s">
+        <v>649</v>
+      </c>
+      <c r="B175" t="s">
+        <v>650</v>
+      </c>
+      <c r="C175" t="b">
+        <v>1</v>
+      </c>
+      <c r="D175" t="b" cm="1">
+        <f t="array" ref="D175">_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"12",""))),_xlpm.next,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"123",""))),IFERROR(NOT(SDKP_HasProgress(_xlpm.c,_xlpm.next)),FALSE))</f>
+        <v>1</v>
+      </c>
+      <c r="E175" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5">
+      <c r="A176" t="s">
+        <v>651</v>
+      </c>
+      <c r="B176" t="s">
+        <v>631</v>
+      </c>
+      <c r="C176" t="b">
+        <v>1</v>
+      </c>
+      <c r="D176" t="b" cm="1">
+        <f t="array" ref="D176">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=2,OR(_xlpm.k=7,_xlpm.k=8)),"13",AND(_xlpm.r=3,_xlpm.k=7),"34",AND(_xlpm.r=2,_xlpm.k&lt;&gt;7,_xlpm.k&lt;&gt;8),"12456789",AND(OR(_xlpm.r=1,_xlpm.r=3),_xlpm.k&gt;=7,_xlpm.k&lt;=9),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingRowStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Claiming row",INDEX(_xlpm.s,1,2)="R2C7, R2C8",INDEX(_xlpm.s,1,3)="3",INDEX(_xlpm.s,1,4)="R3C7",INDEX(_xlpm.s,1,5)="Claiming row · Row 2 confines digit 3 to box 3 via R2C7, R2C8 · Remove 3 from R3C7."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E176" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5">
+      <c r="A177" t="s">
+        <v>652</v>
+      </c>
+      <c r="B177" t="s">
+        <v>653</v>
+      </c>
+      <c r="C177" t="b">
+        <v>1</v>
+      </c>
+      <c r="D177" t="b" cm="1">
+        <f t="array" ref="D177">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=2,OR(_xlpm.k=7,_xlpm.k=8)),"13",AND(_xlpm.r=3,_xlpm.k=7),"34",AND(_xlpm.r=2,_xlpm.k&lt;&gt;7,_xlpm.k&lt;&gt;8),"12456789",AND(OR(_xlpm.r=1,_xlpm.r=3),_xlpm.k&gt;=7,_xlpm.k&lt;=9),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingRowStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,3,7)="4",INDEX(_xlpm.after,2,7)="13")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E177" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5">
+      <c r="A178" t="s">
+        <v>654</v>
+      </c>
+      <c r="B178" t="s">
+        <v>655</v>
+      </c>
+      <c r="C178" t="b">
+        <v>1</v>
+      </c>
+      <c r="D178" t="b" cm="1">
+        <f t="array" ref="D178">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=2,OR(_xlpm.k=7,_xlpm.k=8)),"13",AND(_xlpm.r=3,_xlpm.k=7),"34",AND(_xlpm.r=2,_xlpm.k&lt;&gt;7,_xlpm.k&lt;&gt;8),"12456789",AND(OR(_xlpm.r=1,_xlpm.r=3),_xlpm.k&gt;=7,_xlpm.k&lt;=9),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingRowStep(_xlpm.c),SDKP_ClaimingRow(_xlpm.c)=INDEX(_xlpm.s,1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E178" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5">
+      <c r="A179" t="s">
+        <v>656</v>
+      </c>
+      <c r="B179" t="s">
+        <v>631</v>
+      </c>
+      <c r="C179" t="b">
+        <v>1</v>
+      </c>
+      <c r="D179" t="b" cm="1">
+        <f t="array" ref="D179">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=2,OR(_xlpm.r=7,_xlpm.r=8)),"13",AND(_xlpm.r=7,_xlpm.k=3),"34",AND(_xlpm.k=2,_xlpm.r&lt;&gt;7,_xlpm.r&lt;&gt;8),"12456789",AND(_xlpm.r&gt;=7,_xlpm.r&lt;=9,OR(_xlpm.k=1,_xlpm.k=3)),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingColStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Claiming column",INDEX(_xlpm.s,1,2)="R7C2, R8C2",INDEX(_xlpm.s,1,3)="3",INDEX(_xlpm.s,1,4)="R7C3",INDEX(_xlpm.s,1,5)="Claiming column · Column 2 confines digit 3 to box 7 via R7C2, R8C2 · Remove 3 from R7C3."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E179" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5">
+      <c r="A180" t="s">
+        <v>657</v>
+      </c>
+      <c r="B180" t="s">
+        <v>658</v>
+      </c>
+      <c r="C180" t="b">
+        <v>1</v>
+      </c>
+      <c r="D180" t="b" cm="1">
+        <f t="array" ref="D180">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=2,OR(_xlpm.r=7,_xlpm.r=8)),"13",AND(_xlpm.r=7,_xlpm.k=3),"34",AND(_xlpm.k=2,_xlpm.r&lt;&gt;7,_xlpm.r&lt;&gt;8),"12456789",AND(_xlpm.r&gt;=7,_xlpm.r&lt;=9,OR(_xlpm.k=1,_xlpm.k=3)),"12456789",TRUE,"123456789"))),_xlpm.s,SDKP_ClaimingColStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,7,3)="4",INDEX(_xlpm.after,7,2)="13")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E180" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5">
+      <c r="A181" t="s">
+        <v>659</v>
+      </c>
+      <c r="B181" t="s">
+        <v>655</v>
+      </c>
+      <c r="C181" t="b">
+        <v>1</v>
+      </c>
+      <c r="D181" t="b" cm="1">
+        <f t="array" ref="D181">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=2,OR(_xlpm.r=7,_xlpm.r=8)),"13",AND(_xlpm.r=7,_xlpm.k=3),"34",AND(_xlpm.k=2,_xlpm.r&lt;&gt;7,_xlpm.r&lt;&gt;8),"12456789",AND(_xlpm.r&gt;=7,_xlpm.r&lt;=9,OR(_xlpm.k=1,_xlpm.k=3)),"12456789",TRUE,"123456789"))),SDKP_ClaimingCol(_xlpm.c)=INDEX(SDKP_ClaimingColStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E181" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5">
+      <c r="A182" t="s">
+        <v>660</v>
+      </c>
+      <c r="B182" t="s">
+        <v>661</v>
+      </c>
+      <c r="C182" t="b">
+        <v>1</v>
+      </c>
+      <c r="D182" t="b" cm="1">
+        <f t="array" ref="D182">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairRowStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Naked pair in row",INDEX(_xlpm.s,1,2)="R4C2, R4C5",INDEX(_xlpm.s,1,3)="47",INDEX(_xlpm.s,1,4)="R4C7",INDEX(_xlpm.s,1,5)="Naked pair in row · R4C2 and R4C5 contain only 4/7 · Remove 4 and 7 from R4C7."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E182" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5">
+      <c r="A183" t="s">
+        <v>662</v>
+      </c>
+      <c r="B183" t="s">
+        <v>663</v>
+      </c>
+      <c r="C183" t="b">
+        <v>1</v>
+      </c>
+      <c r="D183" t="b" cm="1">
+        <f t="array" ref="D183">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairRowStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,4,7)="8",INDEX(_xlpm.after,4,2)="47")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E183" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5">
+      <c r="A184" t="s">
+        <v>664</v>
+      </c>
+      <c r="B184" t="s">
+        <v>665</v>
+      </c>
+      <c r="C184" t="b">
+        <v>1</v>
+      </c>
+      <c r="D184" t="b" cm="1">
+        <f t="array" ref="D184">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),SDKP_NakedPairRow(_xlpm.c)=INDEX(SDKP_NakedPairRowStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E184" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5">
+      <c r="A185" t="s">
+        <v>666</v>
+      </c>
+      <c r="B185" t="s">
+        <v>667</v>
+      </c>
+      <c r="C185" t="b">
+        <v>1</v>
+      </c>
+      <c r="D185" t="b" cm="1">
+        <f t="array" ref="D185">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,OR(_xlpm.k=2,_xlpm.k=5,_xlpm.k=8)),"47",AND(_xlpm.r=4,_xlpm.k=7),"478",_xlpm.r=4,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairRowStep(_xlpm.c),SUM(--(_xlpm.s=""))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E185" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5">
+      <c r="A186" t="s">
+        <v>668</v>
+      </c>
+      <c r="B186" t="s">
+        <v>661</v>
+      </c>
+      <c r="C186" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D186" t="b" cm="1">
+        <f t="array" ref="D186">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairColStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Naked pair in column",INDEX(_xlpm.s,1,2)="R2C6, R5C6",INDEX(_xlpm.s,1,3)="47",INDEX(_xlpm.s,1,4)="R7C6",INDEX(_xlpm.s,1,5)="Naked pair in column · R2C6 and R5C6 contain only 4/7 · Remove 4 and 7 from R7C6."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E186" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5">
+      <c r="A187" t="s">
+        <v>669</v>
+      </c>
+      <c r="B187" t="s">
+        <v>670</v>
+      </c>
+      <c r="C187" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D187" t="b" cm="1">
+        <f t="array" ref="D187">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairColStep(_xlpm.c),_xlpm.t,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.t),AND(INDEX(_xlpm.after,7,6)="8",INDEX(_xlpm.after,2,6)="47")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E187" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5">
+      <c r="A188" t="s">
+        <v>671</v>
+      </c>
+      <c r="B188" t="s">
+        <v>665</v>
+      </c>
+      <c r="C188" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D188" t="b" cm="1">
+        <f t="array" ref="D188">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),SDKP_NakedPairCol(_xlpm.c)=INDEX(SDKP_NakedPairColStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E188" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5">
+      <c r="A189" t="s">
+        <v>672</v>
+      </c>
+      <c r="B189" t="s">
+        <v>667</v>
+      </c>
+      <c r="C189" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D189" t="b" cm="1">
+        <f t="array" ref="D189">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.k=6,OR(_xlpm.r=2,_xlpm.r=5,_xlpm.r=8)),"47",AND(_xlpm.r=7,_xlpm.k=6),"478",_xlpm.k=6,"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairColStep(_xlpm.c),SUM(--(_xlpm.s=""))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E189" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5">
+      <c r="A190" t="s">
+        <v>673</v>
+      </c>
+      <c r="B190" t="s">
+        <v>674</v>
+      </c>
+      <c r="C190" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D190" t="b" cm="1">
+        <f t="array" ref="D190">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),SDKP_NakedPairBox(_xlpm.c)="Naked pair in box · R1C2 and R2C3 contain only 4/7 in box 1 · Remove 4 and 7 from R3C1."),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E190" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5">
+      <c r="A191" t="s">
+        <v>675</v>
+      </c>
+      <c r="B191" t="s">
+        <v>676</v>
+      </c>
+      <c r="C191" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D191" t="b" cm="1">
+        <f t="array" ref="D191">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),SUM(--_xlfn.HSTACK(INDEX(_xlpm.s,1,1)="Naked pair in box",INDEX(_xlpm.s,1,2)="R1C2, R2C3",INDEX(_xlpm.s,1,3)="47",INDEX(_xlpm.s,1,4)="R3C1",INDEX(_xlpm.s,1,5)="Naked pair in box · R1C2 and R2C3 contain only 4/7 in box 1 · Remove 4 and 7 from R3C1."))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E191" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5">
+      <c r="A192" t="s">
+        <v>677</v>
+      </c>
+      <c r="B192" t="s">
+        <v>678</v>
+      </c>
+      <c r="C192" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D192" t="b" cm="1">
+        <f t="array" ref="D192">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),_xlpm.action,_xlfn.HSTACK(INDEX(_xlpm.s,1,1),INDEX(_xlpm.s,1,2),INDEX(_xlpm.s,1,3),INDEX(_xlpm.s,1,4),"wording may change"),_xlpm.after,SDKP_ApplyStep(_xlpm.c,_xlpm.action),AND(INDEX(_xlpm.after,3,1)="8",INDEX(_xlpm.after,1,2)="47",INDEX(_xlpm.after,2,3)="47")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E192" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5">
+      <c r="A193" t="s">
+        <v>679</v>
+      </c>
+      <c r="B193" t="s">
+        <v>680</v>
+      </c>
+      <c r="C193" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D193" t="b" cm="1">
+        <f t="array" ref="D193">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),SDKP_NakedPairBox(_xlpm.c)=INDEX(SDKP_NakedPairBoxStep(_xlpm.c),1,5)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E193" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5">
+      <c r="A194" t="s">
+        <v>681</v>
+      </c>
+      <c r="B194" t="s">
+        <v>682</v>
+      </c>
+      <c r="C194" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D194" t="b" cm="1">
+        <f t="array" ref="D194">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),SUM(--(_xlpm.s=""))=5),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E194" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5">
+      <c r="A195" t="s">
+        <v>683</v>
+      </c>
+      <c r="B195" t="s">
+        <v>684</v>
+      </c>
+      <c r="C195" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D195" t="b" cm="1">
+        <f t="array" ref="D195">IFERROR(_xlfn.LET(_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=4,_xlpm.k=5),"47",AND(_xlpm.r=5,_xlpm.k=6),"47",AND(_xlpm.r=6,_xlpm.k=4),"478",AND(_xlpm.r&gt;=4,_xlpm.r&lt;=6,_xlpm.k&gt;=4,_xlpm.k&lt;=6),"1235689",TRUE,"123456789"))),_xlpm.s,SDKP_NakedPairBoxStep(_xlpm.c),AND(INDEX(_xlpm.s,1,2)="R4C5, R5C6",INDEX(_xlpm.s,1,4)="R6C4",ISNUMBER(SEARCH("in box 5",INDEX(_xlpm.s,1,5))))),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E195" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5">
+      <c r="A196" t="s">
+        <v>685</v>
+      </c>
+      <c r="B196" t="s">
+        <v>686</v>
+      </c>
+      <c r="C196" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D196" t="b" cm="1">
+        <f t="array" ref="D196">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,1,""),AND(INDEX(_xlpm.result,10,1)="ASSIGNMENT",INDEX(_xlpm.result,3,1)="8",ISNUMBER(SEARCH("Naked pair in box",INDEX(_xlpm.result,10,5))))),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E196" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5">
+      <c r="A197" t="s">
+        <v>687</v>
+      </c>
+      <c r="B197" t="s">
+        <v>688</v>
+      </c>
+      <c r="C197" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D197" t="b" cm="1">
+        <f t="array" ref="D197">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.IFS(AND(_xlpm.r=1,_xlpm.k=2),"47",AND(_xlpm.r=2,_xlpm.k=3),"47",AND(_xlpm.r=3,_xlpm.k=1),"478",AND(_xlpm.r&lt;=3,_xlpm.k&lt;=3),"1235689",TRUE,"123456789"))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,0,""),AND(INDEX(_xlpm.result,10,1)="LIMIT",INDEX(_xlpm.result,10,2)=0,INDEX(_xlpm.result,3,1)="478",ISNUMBER(SEARCH("Naked pair in box",INDEX(_xlpm.result,10,4))),INDEX(_xlpm.result,10,5)="")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E197" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5">
+      <c r="A198" t="s">
+        <v>689</v>
+      </c>
+      <c r="B198" t="s">
+        <v>690</v>
+      </c>
+      <c r="C198" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D198" t="b">
+        <f>IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"123456789")),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,2,""),AND(INDEX(_xlpm.result,10,1)="STABLE",INDEX(_xlpm.result,10,2)=0,INDEX(_xlpm.result,1,1)="123456789",INDEX(_xlpm.result,10,3)="",INDEX(_xlpm.result,10,4)="",INDEX(_xlpm.result,10,5)="")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E198" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5">
+      <c r="A199" t="s">
+        <v>691</v>
+      </c>
+      <c r="B199" t="s">
+        <v>692</v>
+      </c>
+      <c r="C199" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D199" t="b" cm="1">
+        <f t="array" ref="D199">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,IF(AND(_xlpm.r=1,_xlpm.k=1),"","123456789"))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,2,""),AND(INDEX(_xlpm.result,10,1)="CONTRADICTION",INDEX(_xlpm.result,10,2)=0,INDEX(_xlpm.result,1,1)="",INDEX(_xlpm.result,10,3)="",INDEX(_xlpm.result,10,4)="",INDEX(_xlpm.result,10,5)="")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E199" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5">
+      <c r="A200" t="s">
+        <v>693</v>
+      </c>
+      <c r="B200" t="s">
+        <v>694</v>
+      </c>
+      <c r="C200" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D200" t="b">
+        <f>IFERROR(_xlfn.LET(_xlpm.board,'_Engine Master'!$B$27:$J$35,_xlpm.entered,SDK_SetCell(_xlpm.board,8,3,1),_xlpm.afterEntry,SDKP_Chain(_xlpm.entered,8),_xlpm.afterDelete,SDKP_Chain(_xlpm.board,8),AND(INDEX(_xlpm.afterEntry,10,1)="STABLE",INDEX(_xlpm.afterEntry,8,3)="",INDEX(_xlpm.afterEntry,10,3)="",INDEX(_xlpm.afterDelete,10,1)="ASSIGNMENT",INDEX(_xlpm.afterDelete,10,2)=0,INDEX(_xlpm.afterDelete,8,3)="1268",INDEX(_xlpm.afterDelete,10,3)="Hidden single in column · R8C3 = 1 · Digit 1 appears in only one candidate set in column 3.")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E200" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5">
+      <c r="A201" t="s">
+        <v>695</v>
+      </c>
+      <c r="B201" t="s">
+        <v>696</v>
+      </c>
+      <c r="C201" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D201" t="b" cm="1">
+        <f t="array" ref="D201">IFERROR(_xlfn.LET(_xlpm.board,'_Engine Master'!$B$27:$J$35,_xlpm.wrong,SDK_SetCell(_xlpm.board,2,1,1),_xlpm.wrongChain,SDKP_Chain(_xlpm.wrong,8),_xlpm.recovered,SDKP_Chain(_xlpm.board,8),_xlpm.wrongConflicts,SUM(--_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,SDK_Conflict(_xlpm.wrong,_xlpm.r,_xlpm.k)))),_xlpm.cleanConflicts,SUM(--_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,SDK_Conflict(_xlpm.board,_xlpm.r,_xlpm.k)))),AND(_xlpm.wrongConflicts=2,SDK_Conflict(_xlpm.wrong,1,1),SDK_Conflict(_xlpm.wrong,2,1),INDEX(_xlpm.wrongChain,10,1)="CONTRADICTION",INDEX(_xlpm.wrongChain,10,2)=0,_xlpm.cleanConflicts=0,INDEX(_xlpm.recovered,10,1)="ASSIGNMENT",INDEX(_xlpm.recovered,2,1)="457",INDEX(_xlpm.recovered,10,3)="Hidden single in column · R8C3 = 1 · Digit 1 appears in only one candidate set in column 3.")),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E201" t="str">
+        <f t="shared" si="8"/>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5">
+      <c r="A202" t="s">
+        <v>697</v>
+      </c>
+      <c r="B202" t="s">
+        <v>698</v>
+      </c>
+      <c r="C202" t="b">
+        <f>TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D202" t="b" cm="1">
+        <f t="array" ref="D202">IFERROR(_xlfn.LET(_xlpm.board,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,"")),_xlpm.digits,_xlfn.SEQUENCE(9),_xlpm.c,_xlfn.MAKEARRAY(9,9,_xlfn.LAMBDA(_xlpm.r,_xlpm.k,_xlfn.LET(_xlpm.b,1+3*QUOTIENT(_xlpm.r-1,3),_xlfn.TEXTJOIN("",TRUE,_xlfn._xlws.FILTER(_xlpm.digits,NOT((_xlpm.k&lt;=3)*(_xlpm.digits&gt;=_xlpm.b)*(_xlpm.digits&lt;=_xlpm.b+2)*(_xlpm.digits&lt;&gt;_xlpm.r))))))),_xlpm.result,SDKP_ChainLoop(_xlpm.board,_xlpm.c,0,8,""),_xlpm.log,INDEX(_xlpm.result,10,5),AND(INDEX(_xlpm.result,10,1)="LIMIT",INDEX(_xlpm.result,10,2)=8,INDEX(_xlpm.result,1,4)="23456789",INDEX(_xlpm.result,8,4)="12345679",INDEX(_xlpm.result,9,4)="123456789",ISNUMBER(SEARCH("Pointing row",INDEX(_xlpm.result,10,4))),LEN(_xlpm.log)-LEN(SUBSTITUTE(_xlpm.log,CHAR(10),""))+1=8)),FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="E202" t="str">
+        <f t="shared" si="8"/>
         <v>PASS</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate Expert candidate chain to production
</commit_message>
<xml_diff>
--- a/Sudoku/sudoku.xlsx
+++ b/Sudoku/sudoku.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEB8E379-B146-B447-AB9F-81140D0CB4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5F9E922-F291-CC40-80C6-F4274ECEE6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="700">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="701">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2105,12 +2105,6 @@
     <t>Claiming row · Row 2 confines digit 3 to box 3 via R2C7, R2C8 · Remove 3 from R3C7.</t>
   </si>
   <si>
-    <t>All published engines use player-safe Coach paths</t>
-  </si>
-  <si>
-    <t>Four standard wrappers plus Master shared-chain fallback contract</t>
-  </si>
-  <si>
     <t>STRUCTURED CANDIDATE CHAIN</t>
   </si>
   <si>
@@ -2322,6 +2316,15 @@
   </si>
   <si>
     <t>Prototype Candidate Chain</t>
+  </si>
+  <si>
+    <t>Published engines use player-safe Coach paths</t>
+  </si>
+  <si>
+    <t>Three standard wrappers plus Expert and Master chain fallback contracts</t>
+  </si>
+  <si>
+    <t>Candidate Chain</t>
   </si>
 </sst>
 </file>
@@ -10842,7 +10845,7 @@
   <sheetPr codeName="Sheet12">
     <tabColor rgb="FF0B5A2B"/>
   </sheetPr>
-  <dimension ref="A1:T100"/>
+  <dimension ref="A1:T111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -11269,351 +11272,351 @@
     <row r="15" spans="1:10">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="str" cm="1">
-        <f t="array" ref="B15">SDK_Candidates($B$3:$J$11,1,1)</f>
+        <f t="array" ref="B15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12456</v>
       </c>
       <c r="C15" s="3" t="str" cm="1">
-        <f t="array" ref="C15">SDK_Candidates($B$3:$J$11,1,2)</f>
+        <f t="array" ref="C15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D15" s="3" t="str" cm="1">
-        <f t="array" ref="D15">SDK_Candidates($B$3:$J$11,1,3)</f>
+        <f t="array" ref="D15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>156</v>
       </c>
       <c r="E15" s="3" t="str" cm="1">
-        <f t="array" ref="E15">SDK_Candidates($B$3:$J$11,1,4)</f>
+        <f t="array" ref="E15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>67</v>
       </c>
       <c r="F15" s="3" t="str" cm="1">
-        <f t="array" ref="F15">SDK_Candidates($B$3:$J$11,1,5)</f>
+        <f t="array" ref="F15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12467</v>
       </c>
       <c r="G15" s="3" t="str" cm="1">
-        <f t="array" ref="G15">SDK_Candidates($B$3:$J$11,1,6)</f>
+        <f t="array" ref="G15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>146</v>
       </c>
       <c r="H15" s="3" t="str" cm="1">
-        <f t="array" ref="H15">SDK_Candidates($B$3:$J$11,1,7)</f>
+        <f t="array" ref="H15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4679</v>
       </c>
       <c r="I15" s="3" t="str" cm="1">
-        <f t="array" ref="I15">SDK_Candidates($B$3:$J$11,1,8)</f>
+        <f t="array" ref="I15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J15" s="3" t="str" cm="1">
-        <f t="array" ref="J15">SDK_Candidates($B$3:$J$11,1,9)</f>
+        <f t="array" ref="J15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4679</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="str" cm="1">
-        <f t="array" ref="B16">SDK_Candidates($B$3:$J$11,2,1)</f>
+        <f t="array" ref="B16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12468</v>
       </c>
       <c r="C16" s="3" t="str" cm="1">
-        <f t="array" ref="C16">SDK_Candidates($B$3:$J$11,2,2)</f>
+        <f t="array" ref="C16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1468</v>
       </c>
       <c r="D16" s="3" t="str" cm="1">
-        <f t="array" ref="D16">SDK_Candidates($B$3:$J$11,2,3)</f>
+        <f t="array" ref="D16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E16" s="3" t="str" cm="1">
-        <f t="array" ref="E16">SDK_Candidates($B$3:$J$11,2,4)</f>
+        <f t="array" ref="E16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3678</v>
       </c>
       <c r="F16" s="3" t="str" cm="1">
-        <f t="array" ref="F16">SDK_Candidates($B$3:$J$11,2,5)</f>
+        <f t="array" ref="F16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1234678</v>
       </c>
       <c r="G16" s="3" t="str" cm="1">
-        <f t="array" ref="G16">SDK_Candidates($B$3:$J$11,2,6)</f>
+        <f t="array" ref="G16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13468</v>
       </c>
       <c r="H16" s="3" t="str" cm="1">
-        <f t="array" ref="H16">SDK_Candidates($B$3:$J$11,2,7)</f>
+        <f t="array" ref="H16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I16" s="3" t="str" cm="1">
-        <f t="array" ref="I16">SDK_Candidates($B$3:$J$11,2,8)</f>
+        <f t="array" ref="I16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1467</v>
       </c>
       <c r="J16" s="3" t="str" cm="1">
-        <f t="array" ref="J16">SDK_Candidates($B$3:$J$11,2,9)</f>
+        <f t="array" ref="J16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3467</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="str" cm="1">
-        <f t="array" ref="B17">SDK_Candidates($B$3:$J$11,3,1)</f>
+        <f t="array" ref="B17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1468</v>
       </c>
       <c r="C17" s="3" t="str" cm="1">
-        <f t="array" ref="C17">SDK_Candidates($B$3:$J$11,3,2)</f>
+        <f t="array" ref="C17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1468</v>
       </c>
       <c r="D17" s="3" t="str" cm="1">
-        <f t="array" ref="D17">SDK_Candidates($B$3:$J$11,3,3)</f>
+        <f t="array" ref="D17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E17" s="3" t="str" cm="1">
-        <f t="array" ref="E17">SDK_Candidates($B$3:$J$11,3,4)</f>
+        <f t="array" ref="E17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="str" cm="1">
-        <f t="array" ref="F17">SDK_Candidates($B$3:$J$11,3,5)</f>
+        <f t="array" ref="F17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13468</v>
       </c>
       <c r="G17" s="3" t="str" cm="1">
-        <f t="array" ref="G17">SDK_Candidates($B$3:$J$11,3,6)</f>
+        <f t="array" ref="G17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H17" s="3" t="str" cm="1">
-        <f t="array" ref="H17">SDK_Candidates($B$3:$J$11,3,7)</f>
+        <f t="array" ref="H17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I17" s="3" t="str" cm="1">
-        <f t="array" ref="I17">SDK_Candidates($B$3:$J$11,3,8)</f>
+        <f t="array" ref="I17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>146</v>
       </c>
       <c r="J17" s="3" t="str" cm="1">
-        <f t="array" ref="J17">SDK_Candidates($B$3:$J$11,3,9)</f>
+        <f t="array" ref="J17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>346</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="str" cm="1">
-        <f t="array" ref="B18">SDK_Candidates($B$3:$J$11,4,1)</f>
+        <f t="array" ref="B18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C18" s="3" t="str" cm="1">
-        <f t="array" ref="C18">SDK_Candidates($B$3:$J$11,4,2)</f>
+        <f t="array" ref="C18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>46</v>
       </c>
       <c r="D18" s="3" t="str" cm="1">
-        <f t="array" ref="D18">SDK_Candidates($B$3:$J$11,4,3)</f>
+        <f t="array" ref="D18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>36</v>
       </c>
       <c r="E18" s="3" t="str" cm="1">
-        <f t="array" ref="E18">SDK_Candidates($B$3:$J$11,4,4)</f>
+        <f t="array" ref="E18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="str" cm="1">
-        <f t="array" ref="F18">SDK_Candidates($B$3:$J$11,4,5)</f>
+        <f t="array" ref="F18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>36</v>
       </c>
       <c r="G18" s="3" t="str" cm="1">
-        <f t="array" ref="G18">SDK_Candidates($B$3:$J$11,4,6)</f>
+        <f t="array" ref="G18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H18" s="3" t="str" cm="1">
-        <f t="array" ref="H18">SDK_Candidates($B$3:$J$11,4,7)</f>
+        <f t="array" ref="H18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>469</v>
       </c>
       <c r="I18" s="3" t="str" cm="1">
-        <f t="array" ref="I18">SDK_Candidates($B$3:$J$11,4,8)</f>
+        <f t="array" ref="I18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>246</v>
       </c>
       <c r="J18" s="3" t="str" cm="1">
-        <f t="array" ref="J18">SDK_Candidates($B$3:$J$11,4,9)</f>
+        <f t="array" ref="J18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="str" cm="1">
-        <f t="array" ref="B19">SDK_Candidates($B$3:$J$11,5,1)</f>
+        <f t="array" ref="B19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>14568</v>
       </c>
       <c r="C19" s="3" t="str" cm="1">
-        <f t="array" ref="C19">SDK_Candidates($B$3:$J$11,5,2)</f>
+        <f t="array" ref="C19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D19" s="3" t="str" cm="1">
-        <f t="array" ref="D19">SDK_Candidates($B$3:$J$11,5,3)</f>
+        <f t="array" ref="D19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1568</v>
       </c>
       <c r="E19" s="3" t="str" cm="1">
-        <f t="array" ref="E19">SDK_Candidates($B$3:$J$11,5,4)</f>
+        <f t="array" ref="E19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>678</v>
       </c>
       <c r="F19" s="3" t="str" cm="1">
-        <f t="array" ref="F19">SDK_Candidates($B$3:$J$11,5,5)</f>
+        <f t="array" ref="F19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G19" s="3" t="str" cm="1">
-        <f t="array" ref="G19">SDK_Candidates($B$3:$J$11,5,6)</f>
+        <f t="array" ref="G19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>68</v>
       </c>
       <c r="H19" s="3" t="str" cm="1">
-        <f t="array" ref="H19">SDK_Candidates($B$3:$J$11,5,7)</f>
+        <f t="array" ref="H19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>467</v>
       </c>
       <c r="I19" s="3" t="str" cm="1">
-        <f t="array" ref="I19">SDK_Candidates($B$3:$J$11,5,8)</f>
+        <f t="array" ref="I19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J19" s="3" t="str" cm="1">
-        <f t="array" ref="J19">SDK_Candidates($B$3:$J$11,5,9)</f>
+        <f t="array" ref="J19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4567</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="str" cm="1">
-        <f t="array" ref="B20">SDK_Candidates($B$3:$J$11,6,1)</f>
+        <f t="array" ref="B20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C20" s="3" t="str" cm="1">
-        <f t="array" ref="C20">SDK_Candidates($B$3:$J$11,6,2)</f>
+        <f t="array" ref="C20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>568</v>
       </c>
       <c r="D20" s="3" t="str" cm="1">
-        <f t="array" ref="D20">SDK_Candidates($B$3:$J$11,6,3)</f>
+        <f t="array" ref="D20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3568</v>
       </c>
       <c r="E20" s="3" t="str" cm="1">
-        <f t="array" ref="E20">SDK_Candidates($B$3:$J$11,6,4)</f>
+        <f t="array" ref="E20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F20" s="3" t="str" cm="1">
-        <f t="array" ref="F20">SDK_Candidates($B$3:$J$11,6,5)</f>
+        <f t="array" ref="F20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3678</v>
       </c>
       <c r="G20" s="3" t="str" cm="1">
-        <f t="array" ref="G20">SDK_Candidates($B$3:$J$11,6,6)</f>
+        <f t="array" ref="G20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H20" s="3" t="str" cm="1">
-        <f t="array" ref="H20">SDK_Candidates($B$3:$J$11,6,7)</f>
+        <f t="array" ref="H20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>67</v>
       </c>
       <c r="I20" s="3" t="str" cm="1">
-        <f t="array" ref="I20">SDK_Candidates($B$3:$J$11,6,8)</f>
+        <f t="array" ref="I20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>567</v>
       </c>
       <c r="J20" s="3" t="str" cm="1">
-        <f t="array" ref="J20">SDK_Candidates($B$3:$J$11,6,9)</f>
+        <f t="array" ref="J20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="str" cm="1">
-        <f t="array" ref="B21">SDK_Candidates($B$3:$J$11,7,1)</f>
+        <f t="array" ref="B21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3568</v>
       </c>
       <c r="C21" s="3" t="str" cm="1">
-        <f t="array" ref="C21">SDK_Candidates($B$3:$J$11,7,2)</f>
+        <f t="array" ref="C21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>5689</v>
       </c>
       <c r="D21" s="3" t="str" cm="1">
-        <f t="array" ref="D21">SDK_Candidates($B$3:$J$11,7,3)</f>
+        <f t="array" ref="D21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E21" s="3" t="str" cm="1">
-        <f t="array" ref="E21">SDK_Candidates($B$3:$J$11,7,4)</f>
+        <f t="array" ref="E21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F21" s="3" t="str" cm="1">
-        <f t="array" ref="F21">SDK_Candidates($B$3:$J$11,7,5)</f>
+        <f t="array" ref="F21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3568</v>
       </c>
       <c r="G21" s="3" t="str" cm="1">
-        <f t="array" ref="G21">SDK_Candidates($B$3:$J$11,7,6)</f>
+        <f t="array" ref="G21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H21" s="3" t="str" cm="1">
-        <f t="array" ref="H21">SDK_Candidates($B$3:$J$11,7,7)</f>
+        <f t="array" ref="H21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I21" s="3" t="str" cm="1">
-        <f t="array" ref="I21">SDK_Candidates($B$3:$J$11,7,8)</f>
+        <f t="array" ref="I21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>56</v>
       </c>
       <c r="J21" s="3" t="str" cm="1">
-        <f t="array" ref="J21">SDK_Candidates($B$3:$J$11,7,9)</f>
+        <f t="array" ref="J21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>356</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="str" cm="1">
-        <f t="array" ref="B22">SDK_Candidates($B$3:$J$11,8,1)</f>
+        <f t="array" ref="B22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1356</v>
       </c>
       <c r="C22" s="3" t="str" cm="1">
-        <f t="array" ref="C22">SDK_Candidates($B$3:$J$11,8,2)</f>
+        <f t="array" ref="C22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1569</v>
       </c>
       <c r="D22" s="3" t="str" cm="1">
-        <f t="array" ref="D22">SDK_Candidates($B$3:$J$11,8,3)</f>
+        <f t="array" ref="D22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E22" s="3" t="str" cm="1">
-        <f t="array" ref="E22">SDK_Candidates($B$3:$J$11,8,4)</f>
+        <f t="array" ref="E22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>369</v>
       </c>
       <c r="F22" s="3" t="str" cm="1">
-        <f t="array" ref="F22">SDK_Candidates($B$3:$J$11,8,5)</f>
+        <f t="array" ref="F22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13456</v>
       </c>
       <c r="G22" s="3" t="str" cm="1">
-        <f t="array" ref="G22">SDK_Candidates($B$3:$J$11,8,6)</f>
+        <f t="array" ref="G22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1346</v>
       </c>
       <c r="H22" s="3" t="str" cm="1">
-        <f t="array" ref="H22">SDK_Candidates($B$3:$J$11,8,7)</f>
+        <f t="array" ref="H22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I22" s="3" t="str" cm="1">
-        <f t="array" ref="I22">SDK_Candidates($B$3:$J$11,8,8)</f>
+        <f t="array" ref="I22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4567</v>
       </c>
       <c r="J22" s="3" t="str" cm="1">
-        <f t="array" ref="J22">SDK_Candidates($B$3:$J$11,8,9)</f>
+        <f t="array" ref="J22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>34567</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="str" cm="1">
-        <f t="array" ref="B23">SDK_Candidates($B$3:$J$11,9,1)</f>
+        <f t="array" ref="B23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13568</v>
       </c>
       <c r="C23" s="3" t="str" cm="1">
-        <f t="array" ref="C23">SDK_Candidates($B$3:$J$11,9,2)</f>
+        <f t="array" ref="C23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D23" s="3" t="str" cm="1">
-        <f t="array" ref="D23">SDK_Candidates($B$3:$J$11,9,3)</f>
+        <f t="array" ref="D23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13568</v>
       </c>
       <c r="E23" s="3" t="str" cm="1">
-        <f t="array" ref="E23">SDK_Candidates($B$3:$J$11,9,4)</f>
+        <f t="array" ref="E23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>368</v>
       </c>
       <c r="F23" s="3" t="str" cm="1">
-        <f t="array" ref="F23">SDK_Candidates($B$3:$J$11,9,5)</f>
+        <f t="array" ref="F23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>134568</v>
       </c>
       <c r="G23" s="3" t="str" cm="1">
-        <f t="array" ref="G23">SDK_Candidates($B$3:$J$11,9,6)</f>
+        <f t="array" ref="G23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13468</v>
       </c>
       <c r="H23" s="3" t="str" cm="1">
-        <f t="array" ref="H23">SDK_Candidates($B$3:$J$11,9,7)</f>
+        <f t="array" ref="H23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>346</v>
       </c>
       <c r="I23" s="3" t="str" cm="1">
-        <f t="array" ref="I23">SDK_Candidates($B$3:$J$11,9,8)</f>
+        <f t="array" ref="I23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J23" s="3" t="str" cm="1">
-        <f t="array" ref="J23">SDK_Candidates($B$3:$J$11,9,9)</f>
+        <f t="array" ref="J23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23456</v>
       </c>
     </row>
@@ -12789,7 +12792,7 @@
         <v>74</v>
       </c>
       <c r="B88" s="7" t="str" cm="1">
-        <f t="array" ref="B88">IF(OR('04 Expert'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",SDK_PlayerHint($B$3:$J$11,$B$39:$J$47))</f>
+        <f t="array" ref="B88">IF(OR('04 Expert'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",IF($L$111="ASSIGNMENT",$N$111,IF($L$111="LIMIT","Candidate chain limit reached after "&amp;$M$111&amp;" elimination step(s).",IF($L$111="CONTRADICTION","Candidate chain contradiction detected.",SDK_FallbackReveal($B$3:$J$11,$B$39:$J$47)))))</f>
         <v>Hidden single in row · R4C8 = 2 · Digit 2 appears in only one candidate set in row 4.</v>
       </c>
       <c r="C88" s="7"/>
@@ -12815,8 +12818,8 @@
       <c r="A89" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B89" s="7" t="str" cm="1">
-        <f t="array" ref="B89">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),1)</f>
+      <c r="B89" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;1,"Technique — "&amp;INDEX(_xlpm.parts,1,1)&amp;" | Pattern — "&amp;INDEX(_xlpm.parts,1,2),"Status — "&amp;INDEX(_xlpm.parts,1,1))))</f>
         <v>Technique — Hidden single in row | Pattern — R4C8 = 2</v>
       </c>
       <c r="C89" s="7"/>
@@ -12844,8 +12847,8 @@
       <c r="A90" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B90" s="7" t="str" cm="1">
-        <f t="array" ref="B90">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),2)</f>
+      <c r="B90" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;2,"Action — "&amp;_xlfn.TEXTJOIN(" · ",TRUE,_xlfn.DROP(_xlpm.parts,,2)),"Action — No further supported step.")))</f>
         <v>Action — Digit 2 appears in only one candidate set in row 4.</v>
       </c>
       <c r="C90" s="7"/>
@@ -13096,6 +13099,302 @@
       </c>
       <c r="B100" t="str" cm="1">
         <f t="array" ref="B100">IF('04 Expert'!$AS$11="Verify",IF(COUNTIF($B$51:$J$59,TRUE)&gt;0,"CONFLICT",SDK_SolveStatus($B$3:$J$11)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="1:20">
+      <c r="L101" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="102" spans="1:20">
+      <c r="L102" t="str" cm="1">
+        <f t="array" ref="L102:T111">SDKP_Chain($B$3:$J$11,8)</f>
+        <v>12456</v>
+      </c>
+      <c r="M102" t="str">
+        <v/>
+      </c>
+      <c r="N102" t="str">
+        <v>156</v>
+      </c>
+      <c r="O102" t="str">
+        <v>67</v>
+      </c>
+      <c r="P102" t="str">
+        <v>12467</v>
+      </c>
+      <c r="Q102" t="str">
+        <v>146</v>
+      </c>
+      <c r="R102" t="str">
+        <v>4679</v>
+      </c>
+      <c r="S102" t="str">
+        <v/>
+      </c>
+      <c r="T102" t="str">
+        <v>4679</v>
+      </c>
+    </row>
+    <row r="103" spans="1:20">
+      <c r="L103" t="str">
+        <v>12468</v>
+      </c>
+      <c r="M103" t="str">
+        <v>1468</v>
+      </c>
+      <c r="N103" t="str">
+        <v/>
+      </c>
+      <c r="O103" t="str">
+        <v>3678</v>
+      </c>
+      <c r="P103" t="str">
+        <v>1234678</v>
+      </c>
+      <c r="Q103" t="str">
+        <v>13468</v>
+      </c>
+      <c r="R103" t="str">
+        <v/>
+      </c>
+      <c r="S103" t="str">
+        <v>1467</v>
+      </c>
+      <c r="T103" t="str">
+        <v>3467</v>
+      </c>
+    </row>
+    <row r="104" spans="1:20">
+      <c r="L104" t="str">
+        <v>1468</v>
+      </c>
+      <c r="M104" t="str">
+        <v>1468</v>
+      </c>
+      <c r="N104" t="str">
+        <v/>
+      </c>
+      <c r="O104" t="str">
+        <v/>
+      </c>
+      <c r="P104" t="str">
+        <v>13468</v>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
+      </c>
+      <c r="R104" t="str">
+        <v/>
+      </c>
+      <c r="S104" t="str">
+        <v>146</v>
+      </c>
+      <c r="T104" t="str">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="105" spans="1:20">
+      <c r="L105" t="str">
+        <v/>
+      </c>
+      <c r="M105" t="str">
+        <v>46</v>
+      </c>
+      <c r="N105" t="str">
+        <v>36</v>
+      </c>
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v>36</v>
+      </c>
+      <c r="Q105" t="str">
+        <v/>
+      </c>
+      <c r="R105" t="str">
+        <v>469</v>
+      </c>
+      <c r="S105" t="str">
+        <v>246</v>
+      </c>
+      <c r="T105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106" spans="1:20">
+      <c r="L106" t="str">
+        <v>14568</v>
+      </c>
+      <c r="M106" t="str">
+        <v/>
+      </c>
+      <c r="N106" t="str">
+        <v>1568</v>
+      </c>
+      <c r="O106" t="str">
+        <v>678</v>
+      </c>
+      <c r="P106" t="str">
+        <v/>
+      </c>
+      <c r="Q106" t="str">
+        <v>68</v>
+      </c>
+      <c r="R106" t="str">
+        <v>467</v>
+      </c>
+      <c r="S106" t="str">
+        <v/>
+      </c>
+      <c r="T106" t="str">
+        <v>4567</v>
+      </c>
+    </row>
+    <row r="107" spans="1:20">
+      <c r="L107" t="str">
+        <v/>
+      </c>
+      <c r="M107" t="str">
+        <v>568</v>
+      </c>
+      <c r="N107" t="str">
+        <v>3568</v>
+      </c>
+      <c r="O107" t="str">
+        <v/>
+      </c>
+      <c r="P107" t="str">
+        <v>3678</v>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107" t="str">
+        <v>67</v>
+      </c>
+      <c r="S107" t="str">
+        <v>567</v>
+      </c>
+      <c r="T107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="1:20">
+      <c r="L108" t="str">
+        <v>3568</v>
+      </c>
+      <c r="M108" t="str">
+        <v>5689</v>
+      </c>
+      <c r="N108" t="str">
+        <v/>
+      </c>
+      <c r="O108" t="str">
+        <v/>
+      </c>
+      <c r="P108" t="str">
+        <v>3568</v>
+      </c>
+      <c r="Q108" t="str">
+        <v/>
+      </c>
+      <c r="R108" t="str">
+        <v/>
+      </c>
+      <c r="S108" t="str">
+        <v>56</v>
+      </c>
+      <c r="T108" t="str">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="109" spans="1:20">
+      <c r="L109" t="str">
+        <v>1356</v>
+      </c>
+      <c r="M109" t="str">
+        <v>1569</v>
+      </c>
+      <c r="N109" t="str">
+        <v/>
+      </c>
+      <c r="O109" t="str">
+        <v>369</v>
+      </c>
+      <c r="P109" t="str">
+        <v>13456</v>
+      </c>
+      <c r="Q109" t="str">
+        <v>1346</v>
+      </c>
+      <c r="R109" t="str">
+        <v/>
+      </c>
+      <c r="S109" t="str">
+        <v>4567</v>
+      </c>
+      <c r="T109" t="str">
+        <v>34567</v>
+      </c>
+    </row>
+    <row r="110" spans="1:20">
+      <c r="L110" t="str">
+        <v>13568</v>
+      </c>
+      <c r="M110" t="str">
+        <v/>
+      </c>
+      <c r="N110" t="str">
+        <v>13568</v>
+      </c>
+      <c r="O110" t="str">
+        <v>368</v>
+      </c>
+      <c r="P110" t="str">
+        <v>134568</v>
+      </c>
+      <c r="Q110" t="str">
+        <v>13468</v>
+      </c>
+      <c r="R110" t="str">
+        <v>346</v>
+      </c>
+      <c r="S110" t="str">
+        <v/>
+      </c>
+      <c r="T110" t="str">
+        <v>23456</v>
+      </c>
+    </row>
+    <row r="111" spans="1:20">
+      <c r="L111" t="str">
+        <v>ASSIGNMENT</v>
+      </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111" t="str">
+        <v>Hidden single in row · R4C8 = 2 · Digit 2 appears in only one candidate set in row 4.</v>
+      </c>
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
+      <c r="S111" t="str">
+        <v/>
+      </c>
+      <c r="T111" t="str">
         <v/>
       </c>
     </row>
@@ -15369,7 +15668,7 @@
     </row>
     <row r="101" spans="1:20">
       <c r="L101" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
     </row>
     <row r="102" spans="1:20">
@@ -40652,16 +40951,16 @@
     </row>
     <row r="145" spans="1:5">
       <c r="A145" t="s">
-        <v>627</v>
+        <v>698</v>
       </c>
       <c r="B145" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
       <c r="C145" t="b">
         <v>1</v>
       </c>
       <c r="D145" t="b">
-        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
+        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
         <v>1</v>
       </c>
       <c r="E145" t="str">
@@ -40966,15 +41265,15 @@
     </row>
     <row r="164" spans="1:5">
       <c r="A164" s="54" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="165" spans="1:5">
       <c r="A165" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B165" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C165" t="b">
         <v>1</v>
@@ -40990,10 +41289,10 @@
     </row>
     <row r="166" spans="1:5">
       <c r="A166" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B166" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="C166" t="b">
         <v>1</v>
@@ -41009,10 +41308,10 @@
     </row>
     <row r="167" spans="1:5">
       <c r="A167" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B167" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="C167" t="b">
         <v>1</v>
@@ -41028,10 +41327,10 @@
     </row>
     <row r="168" spans="1:5">
       <c r="A168" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B168" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C168" t="b">
         <f>TRUE</f>
@@ -41048,10 +41347,10 @@
     </row>
     <row r="169" spans="1:5">
       <c r="A169" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B169" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="C169" t="b">
         <v>1</v>
@@ -41067,10 +41366,10 @@
     </row>
     <row r="170" spans="1:5">
       <c r="A170" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B170" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C170" t="b">
         <v>1</v>
@@ -41086,10 +41385,10 @@
     </row>
     <row r="171" spans="1:5">
       <c r="A171" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B171" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="C171" t="b">
         <v>1</v>
@@ -41105,10 +41404,10 @@
     </row>
     <row r="172" spans="1:5">
       <c r="A172" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B172" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="C172" t="b">
         <v>0</v>
@@ -41124,10 +41423,10 @@
     </row>
     <row r="173" spans="1:5">
       <c r="A173" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B173" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="C173" t="b">
         <v>1</v>
@@ -41143,10 +41442,10 @@
     </row>
     <row r="174" spans="1:5">
       <c r="A174" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B174" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="C174" t="b">
         <v>1</v>
@@ -41162,10 +41461,10 @@
     </row>
     <row r="175" spans="1:5">
       <c r="A175" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B175" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C175" t="b">
         <v>1</v>
@@ -41181,10 +41480,10 @@
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B176" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C176" t="b">
         <v>1</v>
@@ -41200,10 +41499,10 @@
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B177" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="C177" t="b">
         <v>1</v>
@@ -41219,10 +41518,10 @@
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="B178" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C178" t="b">
         <v>1</v>
@@ -41238,10 +41537,10 @@
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="B179" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C179" t="b">
         <v>1</v>
@@ -41257,10 +41556,10 @@
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B180" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C180" t="b">
         <v>1</v>
@@ -41276,10 +41575,10 @@
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="B181" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C181" t="b">
         <v>1</v>
@@ -41295,10 +41594,10 @@
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B182" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C182" t="b">
         <v>1</v>
@@ -41314,10 +41613,10 @@
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B183" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="C183" t="b">
         <v>1</v>
@@ -41333,10 +41632,10 @@
     </row>
     <row r="184" spans="1:5">
       <c r="A184" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="B184" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C184" t="b">
         <v>1</v>
@@ -41352,10 +41651,10 @@
     </row>
     <row r="185" spans="1:5">
       <c r="A185" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="B185" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C185" t="b">
         <v>1</v>
@@ -41371,10 +41670,10 @@
     </row>
     <row r="186" spans="1:5">
       <c r="A186" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="B186" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C186" t="b">
         <f>TRUE()</f>
@@ -41391,10 +41690,10 @@
     </row>
     <row r="187" spans="1:5">
       <c r="A187" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B187" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="C187" t="b">
         <f>TRUE()</f>
@@ -41411,10 +41710,10 @@
     </row>
     <row r="188" spans="1:5">
       <c r="A188" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B188" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C188" t="b">
         <f>TRUE()</f>
@@ -41431,10 +41730,10 @@
     </row>
     <row r="189" spans="1:5">
       <c r="A189" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="B189" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C189" t="b">
         <f>TRUE()</f>
@@ -41451,10 +41750,10 @@
     </row>
     <row r="190" spans="1:5">
       <c r="A190" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B190" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="C190" t="b">
         <f>TRUE()</f>
@@ -41471,10 +41770,10 @@
     </row>
     <row r="191" spans="1:5">
       <c r="A191" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="B191" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C191" t="b">
         <f>TRUE()</f>
@@ -41491,10 +41790,10 @@
     </row>
     <row r="192" spans="1:5">
       <c r="A192" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="B192" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C192" t="b">
         <f>TRUE()</f>
@@ -41511,10 +41810,10 @@
     </row>
     <row r="193" spans="1:5">
       <c r="A193" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B193" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C193" t="b">
         <f>TRUE()</f>
@@ -41531,10 +41830,10 @@
     </row>
     <row r="194" spans="1:5">
       <c r="A194" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="B194" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="C194" t="b">
         <f>TRUE()</f>
@@ -41551,10 +41850,10 @@
     </row>
     <row r="195" spans="1:5">
       <c r="A195" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="B195" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="C195" t="b">
         <f>TRUE()</f>
@@ -41571,10 +41870,10 @@
     </row>
     <row r="196" spans="1:5">
       <c r="A196" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B196" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C196" t="b">
         <f>TRUE()</f>
@@ -41591,10 +41890,10 @@
     </row>
     <row r="197" spans="1:5">
       <c r="A197" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="B197" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C197" t="b">
         <f>TRUE()</f>
@@ -41611,10 +41910,10 @@
     </row>
     <row r="198" spans="1:5">
       <c r="A198" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B198" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C198" t="b">
         <f>TRUE()</f>
@@ -41631,10 +41930,10 @@
     </row>
     <row r="199" spans="1:5">
       <c r="A199" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B199" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C199" t="b">
         <f>TRUE()</f>
@@ -41651,10 +41950,10 @@
     </row>
     <row r="200" spans="1:5">
       <c r="A200" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="B200" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C200" t="b">
         <f>TRUE()</f>
@@ -41671,10 +41970,10 @@
     </row>
     <row r="201" spans="1:5">
       <c r="A201" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="B201" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C201" t="b">
         <f>TRUE()</f>
@@ -41691,10 +41990,10 @@
     </row>
     <row r="202" spans="1:5">
       <c r="A202" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="B202" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C202" t="b">
         <f>TRUE()</f>

</xml_diff>

<commit_message>
Migrate Hard candidate chain to production
</commit_message>
<xml_diff>
--- a/Sudoku/sudoku.xlsx
+++ b/Sudoku/sudoku.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5F9E922-F291-CC40-80C6-F4274ECEE6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A514DE9A-54AF-E94C-A608-9B97EC3E5F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="701">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2321,10 +2321,10 @@
     <t>Published engines use player-safe Coach paths</t>
   </si>
   <si>
-    <t>Three standard wrappers plus Expert and Master chain fallback contracts</t>
-  </si>
-  <si>
     <t>Candidate Chain</t>
+  </si>
+  <si>
+    <t>Two standard wrappers plus Hard, Expert, and Master chain fallback contracts</t>
   </si>
 </sst>
 </file>
@@ -8567,7 +8567,7 @@
   <sheetPr codeName="Sheet11">
     <tabColor rgb="FF0B5A2B"/>
   </sheetPr>
-  <dimension ref="A1:T100"/>
+  <dimension ref="A1:T111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -8994,351 +8994,351 @@
     <row r="15" spans="1:10">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="str" cm="1">
-        <f t="array" ref="B15">SDK_Candidates($B$3:$J$11,1,1)</f>
+        <f t="array" ref="B15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23468</v>
       </c>
       <c r="C15" s="3" t="str" cm="1">
-        <f t="array" ref="C15">SDK_Candidates($B$3:$J$11,1,2)</f>
+        <f t="array" ref="C15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1468</v>
       </c>
       <c r="D15" s="3" t="str" cm="1">
-        <f t="array" ref="D15">SDK_Candidates($B$3:$J$11,1,3)</f>
+        <f t="array" ref="D15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>123568</v>
       </c>
       <c r="E15" s="3" t="str" cm="1">
-        <f t="array" ref="E15">SDK_Candidates($B$3:$J$11,1,4)</f>
+        <f t="array" ref="E15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>368</v>
       </c>
       <c r="F15" s="3" t="str" cm="1">
-        <f t="array" ref="F15">SDK_Candidates($B$3:$J$11,1,5)</f>
+        <f t="array" ref="F15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1368</v>
       </c>
       <c r="G15" s="3" t="str" cm="1">
-        <f t="array" ref="G15">SDK_Candidates($B$3:$J$11,1,6)</f>
+        <f t="array" ref="G15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>136</v>
       </c>
       <c r="H15" s="3" t="str" cm="1">
-        <f t="array" ref="H15">SDK_Candidates($B$3:$J$11,1,7)</f>
+        <f t="array" ref="H15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I15" s="3" t="str" cm="1">
-        <f t="array" ref="I15">SDK_Candidates($B$3:$J$11,1,8)</f>
+        <f t="array" ref="I15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>35</v>
       </c>
       <c r="J15" s="3" t="str" cm="1">
-        <f t="array" ref="J15">SDK_Candidates($B$3:$J$11,1,9)</f>
+        <f t="array" ref="J15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="str" cm="1">
-        <f t="array" ref="B16">SDK_Candidates($B$3:$J$11,2,1)</f>
+        <f t="array" ref="B16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>367</v>
       </c>
       <c r="C16" s="3" t="str" cm="1">
-        <f t="array" ref="C16">SDK_Candidates($B$3:$J$11,2,2)</f>
+        <f t="array" ref="C16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>679</v>
       </c>
       <c r="D16" s="3" t="str" cm="1">
-        <f t="array" ref="D16">SDK_Candidates($B$3:$J$11,2,3)</f>
+        <f t="array" ref="D16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3569</v>
       </c>
       <c r="E16" s="3" t="str" cm="1">
-        <f t="array" ref="E16">SDK_Candidates($B$3:$J$11,2,4)</f>
+        <f t="array" ref="E16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F16" s="3" t="str" cm="1">
-        <f t="array" ref="F16">SDK_Candidates($B$3:$J$11,2,5)</f>
+        <f t="array" ref="F16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G16" s="3" t="str" cm="1">
-        <f t="array" ref="G16">SDK_Candidates($B$3:$J$11,2,6)</f>
+        <f t="array" ref="G16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>36</v>
       </c>
       <c r="H16" s="3" t="str" cm="1">
-        <f t="array" ref="H16">SDK_Candidates($B$3:$J$11,2,7)</f>
+        <f t="array" ref="H16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I16" s="3" t="str" cm="1">
-        <f t="array" ref="I16">SDK_Candidates($B$3:$J$11,2,8)</f>
+        <f t="array" ref="I16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J16" s="3" t="str" cm="1">
-        <f t="array" ref="J16">SDK_Candidates($B$3:$J$11,2,9)</f>
+        <f t="array" ref="J16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="str" cm="1">
-        <f t="array" ref="B17">SDK_Candidates($B$3:$J$11,3,1)</f>
+        <f t="array" ref="B17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>348</v>
       </c>
       <c r="C17" s="3" t="str" cm="1">
-        <f t="array" ref="C17">SDK_Candidates($B$3:$J$11,3,2)</f>
+        <f t="array" ref="C17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1489</v>
       </c>
       <c r="D17" s="3" t="str" cm="1">
-        <f t="array" ref="D17">SDK_Candidates($B$3:$J$11,3,3)</f>
+        <f t="array" ref="D17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1389</v>
       </c>
       <c r="E17" s="3" t="str" cm="1">
-        <f t="array" ref="E17">SDK_Candidates($B$3:$J$11,3,4)</f>
+        <f t="array" ref="E17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F17" s="3" t="str" cm="1">
-        <f t="array" ref="F17">SDK_Candidates($B$3:$J$11,3,5)</f>
+        <f t="array" ref="F17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1389</v>
       </c>
       <c r="G17" s="3" t="str" cm="1">
-        <f t="array" ref="G17">SDK_Candidates($B$3:$J$11,3,6)</f>
+        <f t="array" ref="G17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H17" s="3" t="str" cm="1">
-        <f t="array" ref="H17">SDK_Candidates($B$3:$J$11,3,7)</f>
+        <f t="array" ref="H17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>34</v>
       </c>
       <c r="I17" s="3" t="str" cm="1">
-        <f t="array" ref="I17">SDK_Candidates($B$3:$J$11,3,8)</f>
+        <f t="array" ref="I17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J17" s="3" t="str" cm="1">
-        <f t="array" ref="J17">SDK_Candidates($B$3:$J$11,3,9)</f>
+        <f t="array" ref="J17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="str" cm="1">
-        <f t="array" ref="B18">SDK_Candidates($B$3:$J$11,4,1)</f>
+        <f t="array" ref="B18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C18" s="3" t="str" cm="1">
-        <f t="array" ref="C18">SDK_Candidates($B$3:$J$11,4,2)</f>
+        <f t="array" ref="C18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>678</v>
       </c>
       <c r="D18" s="3" t="str" cm="1">
-        <f t="array" ref="D18">SDK_Candidates($B$3:$J$11,4,3)</f>
+        <f t="array" ref="D18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2368</v>
       </c>
       <c r="E18" s="3" t="str" cm="1">
-        <f t="array" ref="E18">SDK_Candidates($B$3:$J$11,4,4)</f>
+        <f t="array" ref="E18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="str" cm="1">
-        <f t="array" ref="F18">SDK_Candidates($B$3:$J$11,4,5)</f>
+        <f t="array" ref="F18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>368</v>
       </c>
       <c r="G18" s="3" t="str" cm="1">
-        <f t="array" ref="G18">SDK_Candidates($B$3:$J$11,4,6)</f>
+        <f t="array" ref="G18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H18" s="3" t="str" cm="1">
-        <f t="array" ref="H18">SDK_Candidates($B$3:$J$11,4,7)</f>
+        <f t="array" ref="H18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>235678</v>
       </c>
       <c r="I18" s="3" t="str" cm="1">
-        <f t="array" ref="I18">SDK_Candidates($B$3:$J$11,4,8)</f>
+        <f t="array" ref="I18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3567</v>
       </c>
       <c r="J18" s="3" t="str" cm="1">
-        <f t="array" ref="J18">SDK_Candidates($B$3:$J$11,4,9)</f>
+        <f t="array" ref="J18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2358</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="str" cm="1">
-        <f t="array" ref="B19">SDK_Candidates($B$3:$J$11,5,1)</f>
+        <f t="array" ref="B19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23678</v>
       </c>
       <c r="C19" s="3" t="str" cm="1">
-        <f t="array" ref="C19">SDK_Candidates($B$3:$J$11,5,2)</f>
+        <f t="array" ref="C19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D19" s="3" t="str" cm="1">
-        <f t="array" ref="D19">SDK_Candidates($B$3:$J$11,5,3)</f>
+        <f t="array" ref="D19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23689</v>
       </c>
       <c r="E19" s="3" t="str" cm="1">
-        <f t="array" ref="E19">SDK_Candidates($B$3:$J$11,5,4)</f>
+        <f t="array" ref="E19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2368</v>
       </c>
       <c r="F19" s="3" t="str" cm="1">
-        <f t="array" ref="F19">SDK_Candidates($B$3:$J$11,5,5)</f>
+        <f t="array" ref="F19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1368</v>
       </c>
       <c r="G19" s="3" t="str" cm="1">
-        <f t="array" ref="G19">SDK_Candidates($B$3:$J$11,5,6)</f>
+        <f t="array" ref="G19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1236</v>
       </c>
       <c r="H19" s="3" t="str" cm="1">
-        <f t="array" ref="H19">SDK_Candidates($B$3:$J$11,5,7)</f>
+        <f t="array" ref="H19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23678</v>
       </c>
       <c r="I19" s="3" t="str" cm="1">
-        <f t="array" ref="I19">SDK_Candidates($B$3:$J$11,5,8)</f>
+        <f t="array" ref="I19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J19" s="3" t="str" cm="1">
-        <f t="array" ref="J19">SDK_Candidates($B$3:$J$11,5,9)</f>
+        <f t="array" ref="J19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1238</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="str" cm="1">
-        <f t="array" ref="B20">SDK_Candidates($B$3:$J$11,6,1)</f>
+        <f t="array" ref="B20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23468</v>
       </c>
       <c r="C20" s="3" t="str" cm="1">
-        <f t="array" ref="C20">SDK_Candidates($B$3:$J$11,6,2)</f>
+        <f t="array" ref="C20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>468</v>
       </c>
       <c r="D20" s="3" t="str" cm="1">
-        <f t="array" ref="D20">SDK_Candidates($B$3:$J$11,6,3)</f>
+        <f t="array" ref="D20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2368</v>
       </c>
       <c r="E20" s="3" t="str" cm="1">
-        <f t="array" ref="E20">SDK_Candidates($B$3:$J$11,6,4)</f>
+        <f t="array" ref="E20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F20" s="3" t="str" cm="1">
-        <f t="array" ref="F20">SDK_Candidates($B$3:$J$11,6,5)</f>
+        <f t="array" ref="F20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1368</v>
       </c>
       <c r="G20" s="3" t="str" cm="1">
-        <f t="array" ref="G20">SDK_Candidates($B$3:$J$11,6,6)</f>
+        <f t="array" ref="G20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H20" s="3" t="str" cm="1">
-        <f t="array" ref="H20">SDK_Candidates($B$3:$J$11,6,7)</f>
+        <f t="array" ref="H20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2368</v>
       </c>
       <c r="I20" s="3" t="str" cm="1">
-        <f t="array" ref="I20">SDK_Candidates($B$3:$J$11,6,8)</f>
+        <f t="array" ref="I20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>136</v>
       </c>
       <c r="J20" s="3" t="str" cm="1">
-        <f t="array" ref="J20">SDK_Candidates($B$3:$J$11,6,9)</f>
+        <f t="array" ref="J20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="str" cm="1">
-        <f t="array" ref="B21">SDK_Candidates($B$3:$J$11,7,1)</f>
+        <f t="array" ref="B21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C21" s="3" t="str" cm="1">
-        <f t="array" ref="C21">SDK_Candidates($B$3:$J$11,7,2)</f>
+        <f t="array" ref="C21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D21" s="3" t="str" cm="1">
-        <f t="array" ref="D21">SDK_Candidates($B$3:$J$11,7,3)</f>
+        <f t="array" ref="D21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>6</v>
       </c>
       <c r="E21" s="3" t="str" cm="1">
-        <f t="array" ref="E21">SDK_Candidates($B$3:$J$11,7,4)</f>
+        <f t="array" ref="E21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F21" s="3" t="str" cm="1">
-        <f t="array" ref="F21">SDK_Candidates($B$3:$J$11,7,5)</f>
+        <f t="array" ref="F21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3467</v>
       </c>
       <c r="G21" s="3" t="str" cm="1">
-        <f t="array" ref="G21">SDK_Candidates($B$3:$J$11,7,6)</f>
+        <f t="array" ref="G21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H21" s="3" t="str" cm="1">
-        <f t="array" ref="H21">SDK_Candidates($B$3:$J$11,7,7)</f>
+        <f t="array" ref="H21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>34567</v>
       </c>
       <c r="I21" s="3" t="str" cm="1">
-        <f t="array" ref="I21">SDK_Candidates($B$3:$J$11,7,8)</f>
+        <f t="array" ref="I21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3567</v>
       </c>
       <c r="J21" s="3" t="str" cm="1">
-        <f t="array" ref="J21">SDK_Candidates($B$3:$J$11,7,9)</f>
+        <f t="array" ref="J21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>345</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="str" cm="1">
-        <f t="array" ref="B22">SDK_Candidates($B$3:$J$11,8,1)</f>
+        <f t="array" ref="B22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>68</v>
       </c>
       <c r="C22" s="3" t="str" cm="1">
-        <f t="array" ref="C22">SDK_Candidates($B$3:$J$11,8,2)</f>
+        <f t="array" ref="C22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D22" s="3" t="str" cm="1">
-        <f t="array" ref="D22">SDK_Candidates($B$3:$J$11,8,3)</f>
+        <f t="array" ref="D22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E22" s="3" t="str" cm="1">
-        <f t="array" ref="E22">SDK_Candidates($B$3:$J$11,8,4)</f>
+        <f t="array" ref="E22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>26</v>
       </c>
       <c r="F22" s="3" t="str" cm="1">
-        <f t="array" ref="F22">SDK_Candidates($B$3:$J$11,8,5)</f>
+        <f t="array" ref="F22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G22" s="3" t="str" cm="1">
-        <f t="array" ref="G22">SDK_Candidates($B$3:$J$11,8,6)</f>
+        <f t="array" ref="G22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H22" s="3" t="str" cm="1">
-        <f t="array" ref="H22">SDK_Candidates($B$3:$J$11,8,7)</f>
+        <f t="array" ref="H22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2678</v>
       </c>
       <c r="I22" s="3" t="str" cm="1">
-        <f t="array" ref="I22">SDK_Candidates($B$3:$J$11,8,8)</f>
+        <f t="array" ref="I22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>167</v>
       </c>
       <c r="J22" s="3" t="str" cm="1">
-        <f t="array" ref="J22">SDK_Candidates($B$3:$J$11,8,9)</f>
+        <f t="array" ref="J22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="str" cm="1">
-        <f t="array" ref="B23">SDK_Candidates($B$3:$J$11,9,1)</f>
+        <f t="array" ref="B23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C23" s="3" t="str" cm="1">
-        <f t="array" ref="C23">SDK_Candidates($B$3:$J$11,9,2)</f>
+        <f t="array" ref="C23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>168</v>
       </c>
       <c r="D23" s="3" t="str" cm="1">
-        <f t="array" ref="D23">SDK_Candidates($B$3:$J$11,9,3)</f>
+        <f t="array" ref="D23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E23" s="3" t="str" cm="1">
-        <f t="array" ref="E23">SDK_Candidates($B$3:$J$11,9,4)</f>
+        <f t="array" ref="E23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>236</v>
       </c>
       <c r="F23" s="3" t="str" cm="1">
-        <f t="array" ref="F23">SDK_Candidates($B$3:$J$11,9,5)</f>
+        <f t="array" ref="F23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>346</v>
       </c>
       <c r="G23" s="3" t="str" cm="1">
-        <f t="array" ref="G23">SDK_Candidates($B$3:$J$11,9,6)</f>
+        <f t="array" ref="G23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>236</v>
       </c>
       <c r="H23" s="3" t="str" cm="1">
-        <f t="array" ref="H23">SDK_Candidates($B$3:$J$11,9,7)</f>
+        <f t="array" ref="H23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23468</v>
       </c>
       <c r="I23" s="3" t="str" cm="1">
-        <f t="array" ref="I23">SDK_Candidates($B$3:$J$11,9,8)</f>
+        <f t="array" ref="I23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1369</v>
       </c>
       <c r="J23" s="3" t="str" cm="1">
-        <f t="array" ref="J23">SDK_Candidates($B$3:$J$11,9,9)</f>
+        <f t="array" ref="J23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12348</v>
       </c>
     </row>
@@ -10516,7 +10516,7 @@
         <v>74</v>
       </c>
       <c r="B88" s="7" t="str" cm="1">
-        <f t="array" ref="B88">IF(OR('03 Hard'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",SDK_PlayerHint($B$3:$J$11,$B$39:$J$47))</f>
+        <f t="array" ref="B88">IF(OR('03 Hard'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",IF($L$111="ASSIGNMENT",$N$111,IF($L$111="LIMIT","Candidate chain limit reached after "&amp;$M$111&amp;" elimination step(s).",IF($L$111="CONTRADICTION","Candidate chain contradiction detected.",SDK_FallbackReveal($B$3:$J$11,$B$39:$J$47)))))</f>
         <v>Naked single · R7C3 = 6 · This is the only legal candidate remaining in the square.</v>
       </c>
       <c r="C88" s="7"/>
@@ -10542,8 +10542,8 @@
       <c r="A89" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B89" s="7" t="str" cm="1">
-        <f t="array" ref="B89">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),1)</f>
+      <c r="B89" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;1,"Technique — "&amp;INDEX(_xlpm.parts,1,1)&amp;" | Pattern — "&amp;INDEX(_xlpm.parts,1,2),"Status — "&amp;INDEX(_xlpm.parts,1,1))))</f>
         <v>Technique — Naked single | Pattern — R7C3 = 6</v>
       </c>
       <c r="C89" s="7"/>
@@ -10571,8 +10571,8 @@
       <c r="A90" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B90" s="7" t="str" cm="1">
-        <f t="array" ref="B90">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),2)</f>
+      <c r="B90" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;2,"Action — "&amp;_xlfn.TEXTJOIN(" · ",TRUE,_xlfn.DROP(_xlpm.parts,,2)),"Action — No further supported step.")))</f>
         <v>Action — This is the only legal candidate remaining in the square.</v>
       </c>
       <c r="C90" s="7"/>
@@ -10823,6 +10823,302 @@
       </c>
       <c r="B100" t="str" cm="1">
         <f t="array" ref="B100">IF('03 Hard'!$AS$11="Verify",IF(COUNTIF($B$51:$J$59,TRUE)&gt;0,"CONFLICT",SDK_SolveStatus($B$3:$J$11)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="1:20">
+      <c r="L101" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="102" spans="1:20">
+      <c r="L102" t="str" cm="1">
+        <f t="array" ref="L102:T111">SDKP_Chain($B$3:$J$11,8)</f>
+        <v>23468</v>
+      </c>
+      <c r="M102" t="str">
+        <v>1468</v>
+      </c>
+      <c r="N102" t="str">
+        <v>123568</v>
+      </c>
+      <c r="O102" t="str">
+        <v>368</v>
+      </c>
+      <c r="P102" t="str">
+        <v>1368</v>
+      </c>
+      <c r="Q102" t="str">
+        <v>136</v>
+      </c>
+      <c r="R102" t="str">
+        <v/>
+      </c>
+      <c r="S102" t="str">
+        <v>35</v>
+      </c>
+      <c r="T102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103" spans="1:20">
+      <c r="L103" t="str">
+        <v>367</v>
+      </c>
+      <c r="M103" t="str">
+        <v>679</v>
+      </c>
+      <c r="N103" t="str">
+        <v>3569</v>
+      </c>
+      <c r="O103" t="str">
+        <v/>
+      </c>
+      <c r="P103" t="str">
+        <v/>
+      </c>
+      <c r="Q103" t="str">
+        <v>36</v>
+      </c>
+      <c r="R103" t="str">
+        <v/>
+      </c>
+      <c r="S103" t="str">
+        <v/>
+      </c>
+      <c r="T103" t="str">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="104" spans="1:20">
+      <c r="L104" t="str">
+        <v>348</v>
+      </c>
+      <c r="M104" t="str">
+        <v>1489</v>
+      </c>
+      <c r="N104" t="str">
+        <v>1389</v>
+      </c>
+      <c r="O104" t="str">
+        <v/>
+      </c>
+      <c r="P104" t="str">
+        <v>1389</v>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
+      </c>
+      <c r="R104" t="str">
+        <v>34</v>
+      </c>
+      <c r="S104" t="str">
+        <v/>
+      </c>
+      <c r="T104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105" spans="1:20">
+      <c r="L105" t="str">
+        <v/>
+      </c>
+      <c r="M105" t="str">
+        <v>678</v>
+      </c>
+      <c r="N105" t="str">
+        <v>2368</v>
+      </c>
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v>368</v>
+      </c>
+      <c r="Q105" t="str">
+        <v/>
+      </c>
+      <c r="R105" t="str">
+        <v>235678</v>
+      </c>
+      <c r="S105" t="str">
+        <v>3567</v>
+      </c>
+      <c r="T105" t="str">
+        <v>2358</v>
+      </c>
+    </row>
+    <row r="106" spans="1:20">
+      <c r="L106" t="str">
+        <v>23678</v>
+      </c>
+      <c r="M106" t="str">
+        <v/>
+      </c>
+      <c r="N106" t="str">
+        <v>23689</v>
+      </c>
+      <c r="O106" t="str">
+        <v>2368</v>
+      </c>
+      <c r="P106" t="str">
+        <v>1368</v>
+      </c>
+      <c r="Q106" t="str">
+        <v>1236</v>
+      </c>
+      <c r="R106" t="str">
+        <v>23678</v>
+      </c>
+      <c r="S106" t="str">
+        <v/>
+      </c>
+      <c r="T106" t="str">
+        <v>1238</v>
+      </c>
+    </row>
+    <row r="107" spans="1:20">
+      <c r="L107" t="str">
+        <v>23468</v>
+      </c>
+      <c r="M107" t="str">
+        <v>468</v>
+      </c>
+      <c r="N107" t="str">
+        <v>2368</v>
+      </c>
+      <c r="O107" t="str">
+        <v/>
+      </c>
+      <c r="P107" t="str">
+        <v>1368</v>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107" t="str">
+        <v>2368</v>
+      </c>
+      <c r="S107" t="str">
+        <v>136</v>
+      </c>
+      <c r="T107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="1:20">
+      <c r="L108" t="str">
+        <v/>
+      </c>
+      <c r="M108" t="str">
+        <v/>
+      </c>
+      <c r="N108" t="str">
+        <v>6</v>
+      </c>
+      <c r="O108" t="str">
+        <v/>
+      </c>
+      <c r="P108" t="str">
+        <v>3467</v>
+      </c>
+      <c r="Q108" t="str">
+        <v/>
+      </c>
+      <c r="R108" t="str">
+        <v>34567</v>
+      </c>
+      <c r="S108" t="str">
+        <v>3567</v>
+      </c>
+      <c r="T108" t="str">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="109" spans="1:20">
+      <c r="L109" t="str">
+        <v>68</v>
+      </c>
+      <c r="M109" t="str">
+        <v/>
+      </c>
+      <c r="N109" t="str">
+        <v/>
+      </c>
+      <c r="O109" t="str">
+        <v>26</v>
+      </c>
+      <c r="P109" t="str">
+        <v/>
+      </c>
+      <c r="Q109" t="str">
+        <v/>
+      </c>
+      <c r="R109" t="str">
+        <v>2678</v>
+      </c>
+      <c r="S109" t="str">
+        <v>167</v>
+      </c>
+      <c r="T109" t="str">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="110" spans="1:20">
+      <c r="L110" t="str">
+        <v/>
+      </c>
+      <c r="M110" t="str">
+        <v>168</v>
+      </c>
+      <c r="N110" t="str">
+        <v/>
+      </c>
+      <c r="O110" t="str">
+        <v>236</v>
+      </c>
+      <c r="P110" t="str">
+        <v>346</v>
+      </c>
+      <c r="Q110" t="str">
+        <v>236</v>
+      </c>
+      <c r="R110" t="str">
+        <v>23468</v>
+      </c>
+      <c r="S110" t="str">
+        <v>1369</v>
+      </c>
+      <c r="T110" t="str">
+        <v>12348</v>
+      </c>
+    </row>
+    <row r="111" spans="1:20">
+      <c r="L111" t="str">
+        <v>ASSIGNMENT</v>
+      </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111" t="str">
+        <v>Naked single · R7C3 = 6 · This is the only legal candidate remaining in the square.</v>
+      </c>
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
+      <c r="S111" t="str">
+        <v/>
+      </c>
+      <c r="T111" t="str">
         <v/>
       </c>
     </row>
@@ -13104,7 +13400,7 @@
     </row>
     <row r="101" spans="1:20">
       <c r="L101" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="102" spans="1:20">
@@ -40954,13 +41250,13 @@
         <v>698</v>
       </c>
       <c r="B145" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C145" t="b">
         <v>1</v>
       </c>
       <c r="D145" t="b">
-        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
+        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
         <v>1</v>
       </c>
       <c r="E145" t="str">

</xml_diff>

<commit_message>
Migrate Medium candidate chain to production
</commit_message>
<xml_diff>
--- a/Sudoku/sudoku.xlsx
+++ b/Sudoku/sudoku.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A514DE9A-54AF-E94C-A608-9B97EC3E5F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9214672-A963-0F4E-B12F-662D471A5797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="701">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2324,7 +2324,7 @@
     <t>Candidate Chain</t>
   </si>
   <si>
-    <t>Two standard wrappers plus Hard, Expert, and Master chain fallback contracts</t>
+    <t>Easy standard wrapper plus Medium, Hard, Expert, and Master chain fallback contracts</t>
   </si>
 </sst>
 </file>
@@ -6273,7 +6273,7 @@
   <sheetPr codeName="Sheet10">
     <tabColor rgb="FF0B5A2B"/>
   </sheetPr>
-  <dimension ref="A1:T100"/>
+  <dimension ref="A1:T111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -6700,351 +6700,351 @@
     <row r="15" spans="1:10">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="str" cm="1">
-        <f t="array" ref="B15">SDK_Candidates($B$3:$J$11,1,1)</f>
+        <f t="array" ref="B15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>345</v>
       </c>
       <c r="C15" s="3" t="str" cm="1">
-        <f t="array" ref="C15">SDK_Candidates($B$3:$J$11,1,2)</f>
+        <f t="array" ref="C15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3</v>
       </c>
       <c r="D15" s="3" t="str" cm="1">
-        <f t="array" ref="D15">SDK_Candidates($B$3:$J$11,1,3)</f>
+        <f t="array" ref="D15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>5</v>
       </c>
       <c r="E15" s="3" t="str" cm="1">
-        <f t="array" ref="E15">SDK_Candidates($B$3:$J$11,1,4)</f>
+        <f t="array" ref="E15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F15" s="3" t="str" cm="1">
-        <f t="array" ref="F15">SDK_Candidates($B$3:$J$11,1,5)</f>
+        <f t="array" ref="F15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G15" s="3" t="str" cm="1">
-        <f t="array" ref="G15">SDK_Candidates($B$3:$J$11,1,6)</f>
+        <f t="array" ref="G15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>59</v>
       </c>
       <c r="H15" s="3" t="str" cm="1">
-        <f t="array" ref="H15">SDK_Candidates($B$3:$J$11,1,7)</f>
+        <f t="array" ref="H15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I15" s="3" t="str" cm="1">
-        <f t="array" ref="I15">SDK_Candidates($B$3:$J$11,1,8)</f>
+        <f t="array" ref="I15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>8</v>
       </c>
       <c r="J15" s="3" t="str" cm="1">
-        <f t="array" ref="J15">SDK_Candidates($B$3:$J$11,1,9)</f>
+        <f t="array" ref="J15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="str" cm="1">
-        <f t="array" ref="B16">SDK_Candidates($B$3:$J$11,2,1)</f>
+        <f t="array" ref="B16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C16" s="3" t="str" cm="1">
-        <f t="array" ref="C16">SDK_Candidates($B$3:$J$11,2,2)</f>
+        <f t="array" ref="C16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D16" s="3" t="str" cm="1">
-        <f t="array" ref="D16">SDK_Candidates($B$3:$J$11,2,3)</f>
+        <f t="array" ref="D16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>25</v>
       </c>
       <c r="E16" s="3" t="str" cm="1">
-        <f t="array" ref="E16">SDK_Candidates($B$3:$J$11,2,4)</f>
+        <f t="array" ref="E16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>5</v>
       </c>
       <c r="F16" s="3" t="str" cm="1">
-        <f t="array" ref="F16">SDK_Candidates($B$3:$J$11,2,5)</f>
+        <f t="array" ref="F16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G16" s="3" t="str" cm="1">
-        <f t="array" ref="G16">SDK_Candidates($B$3:$J$11,2,6)</f>
+        <f t="array" ref="G16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>15</v>
       </c>
       <c r="H16" s="3" t="str" cm="1">
-        <f t="array" ref="H16">SDK_Candidates($B$3:$J$11,2,7)</f>
+        <f t="array" ref="H16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>234</v>
       </c>
       <c r="I16" s="3" t="str" cm="1">
-        <f t="array" ref="I16">SDK_Candidates($B$3:$J$11,2,8)</f>
+        <f t="array" ref="I16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J16" s="3" t="str" cm="1">
-        <f t="array" ref="J16">SDK_Candidates($B$3:$J$11,2,9)</f>
+        <f t="array" ref="J16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="str" cm="1">
-        <f t="array" ref="B17">SDK_Candidates($B$3:$J$11,3,1)</f>
+        <f t="array" ref="B17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C17" s="3" t="str" cm="1">
-        <f t="array" ref="C17">SDK_Candidates($B$3:$J$11,3,2)</f>
+        <f t="array" ref="C17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D17" s="3" t="str" cm="1">
-        <f t="array" ref="D17">SDK_Candidates($B$3:$J$11,3,3)</f>
+        <f t="array" ref="D17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>27</v>
       </c>
       <c r="E17" s="3" t="str" cm="1">
-        <f t="array" ref="E17">SDK_Candidates($B$3:$J$11,3,4)</f>
+        <f t="array" ref="E17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>8</v>
       </c>
       <c r="F17" s="3" t="str" cm="1">
-        <f t="array" ref="F17">SDK_Candidates($B$3:$J$11,3,5)</f>
+        <f t="array" ref="F17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>38</v>
       </c>
       <c r="G17" s="3" t="str" cm="1">
-        <f t="array" ref="G17">SDK_Candidates($B$3:$J$11,3,6)</f>
+        <f t="array" ref="G17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H17" s="3" t="str" cm="1">
-        <f t="array" ref="H17">SDK_Candidates($B$3:$J$11,3,7)</f>
+        <f t="array" ref="H17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I17" s="3" t="str" cm="1">
-        <f t="array" ref="I17">SDK_Candidates($B$3:$J$11,3,8)</f>
+        <f t="array" ref="I17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>68</v>
       </c>
       <c r="J17" s="3" t="str" cm="1">
-        <f t="array" ref="J17">SDK_Candidates($B$3:$J$11,3,9)</f>
+        <f t="array" ref="J17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="str" cm="1">
-        <f t="array" ref="B18">SDK_Candidates($B$3:$J$11,4,1)</f>
+        <f t="array" ref="B18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C18" s="3" t="str" cm="1">
-        <f t="array" ref="C18">SDK_Candidates($B$3:$J$11,4,2)</f>
+        <f t="array" ref="C18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D18" s="3" t="str" cm="1">
-        <f t="array" ref="D18">SDK_Candidates($B$3:$J$11,4,3)</f>
+        <f t="array" ref="D18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>67</v>
       </c>
       <c r="E18" s="3" t="str" cm="1">
-        <f t="array" ref="E18">SDK_Candidates($B$3:$J$11,4,4)</f>
+        <f t="array" ref="E18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F18" s="3" t="str" cm="1">
-        <f t="array" ref="F18">SDK_Candidates($B$3:$J$11,4,5)</f>
+        <f t="array" ref="F18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>9</v>
       </c>
       <c r="G18" s="3" t="str" cm="1">
-        <f t="array" ref="G18">SDK_Candidates($B$3:$J$11,4,6)</f>
+        <f t="array" ref="G18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>579</v>
       </c>
       <c r="H18" s="3" t="str" cm="1">
-        <f t="array" ref="H18">SDK_Candidates($B$3:$J$11,4,7)</f>
+        <f t="array" ref="H18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>36</v>
       </c>
       <c r="I18" s="3" t="str" cm="1">
-        <f t="array" ref="I18">SDK_Candidates($B$3:$J$11,4,8)</f>
+        <f t="array" ref="I18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J18" s="3" t="str" cm="1">
-        <f t="array" ref="J18">SDK_Candidates($B$3:$J$11,4,9)</f>
+        <f t="array" ref="J18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>357</v>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="str" cm="1">
-        <f t="array" ref="B19">SDK_Candidates($B$3:$J$11,5,1)</f>
+        <f t="array" ref="B19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3</v>
       </c>
       <c r="C19" s="3" t="str" cm="1">
-        <f t="array" ref="C19">SDK_Candidates($B$3:$J$11,5,2)</f>
+        <f t="array" ref="C19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>137</v>
       </c>
       <c r="D19" s="3" t="str" cm="1">
-        <f t="array" ref="D19">SDK_Candidates($B$3:$J$11,5,3)</f>
+        <f t="array" ref="D19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E19" s="3" t="str" cm="1">
-        <f t="array" ref="E19">SDK_Candidates($B$3:$J$11,5,4)</f>
+        <f t="array" ref="E19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F19" s="3" t="str" cm="1">
-        <f t="array" ref="F19">SDK_Candidates($B$3:$J$11,5,5)</f>
+        <f t="array" ref="F19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>8</v>
       </c>
       <c r="G19" s="3" t="str" cm="1">
-        <f t="array" ref="G19">SDK_Candidates($B$3:$J$11,5,6)</f>
+        <f t="array" ref="G19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H19" s="3" t="str" cm="1">
-        <f t="array" ref="H19">SDK_Candidates($B$3:$J$11,5,7)</f>
+        <f t="array" ref="H19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I19" s="3" t="str" cm="1">
-        <f t="array" ref="I19">SDK_Candidates($B$3:$J$11,5,8)</f>
+        <f t="array" ref="I19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>15</v>
       </c>
       <c r="J19" s="3" t="str" cm="1">
-        <f t="array" ref="J19">SDK_Candidates($B$3:$J$11,5,9)</f>
+        <f t="array" ref="J19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>357</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="str" cm="1">
-        <f t="array" ref="B20">SDK_Candidates($B$3:$J$11,6,1)</f>
+        <f t="array" ref="B20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>9</v>
       </c>
       <c r="C20" s="3" t="str" cm="1">
-        <f t="array" ref="C20">SDK_Candidates($B$3:$J$11,6,2)</f>
+        <f t="array" ref="C20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D20" s="3" t="str" cm="1">
-        <f t="array" ref="D20">SDK_Candidates($B$3:$J$11,6,3)</f>
+        <f t="array" ref="D20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>167</v>
       </c>
       <c r="E20" s="3" t="str" cm="1">
-        <f t="array" ref="E20">SDK_Candidates($B$3:$J$11,6,4)</f>
+        <f t="array" ref="E20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>479</v>
       </c>
       <c r="F20" s="3" t="str" cm="1">
-        <f t="array" ref="F20">SDK_Candidates($B$3:$J$11,6,5)</f>
+        <f t="array" ref="F20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>49</v>
       </c>
       <c r="G20" s="3" t="str" cm="1">
-        <f t="array" ref="G20">SDK_Candidates($B$3:$J$11,6,6)</f>
+        <f t="array" ref="G20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H20" s="3" t="str" cm="1">
-        <f t="array" ref="H20">SDK_Candidates($B$3:$J$11,6,7)</f>
+        <f t="array" ref="H20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>16</v>
       </c>
       <c r="I20" s="3" t="str" cm="1">
-        <f t="array" ref="I20">SDK_Candidates($B$3:$J$11,6,8)</f>
+        <f t="array" ref="I20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J20" s="3" t="str" cm="1">
-        <f t="array" ref="J20">SDK_Candidates($B$3:$J$11,6,9)</f>
+        <f t="array" ref="J20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="str" cm="1">
-        <f t="array" ref="B21">SDK_Candidates($B$3:$J$11,7,1)</f>
+        <f t="array" ref="B21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>25</v>
       </c>
       <c r="C21" s="3" t="str" cm="1">
-        <f t="array" ref="C21">SDK_Candidates($B$3:$J$11,7,2)</f>
+        <f t="array" ref="C21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>16</v>
       </c>
       <c r="D21" s="3" t="str" cm="1">
-        <f t="array" ref="D21">SDK_Candidates($B$3:$J$11,7,3)</f>
+        <f t="array" ref="D21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E21" s="3" t="str" cm="1">
-        <f t="array" ref="E21">SDK_Candidates($B$3:$J$11,7,4)</f>
+        <f t="array" ref="E21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F21" s="3" t="str" cm="1">
-        <f t="array" ref="F21">SDK_Candidates($B$3:$J$11,7,5)</f>
+        <f t="array" ref="F21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2</v>
       </c>
       <c r="G21" s="3" t="str" cm="1">
-        <f t="array" ref="G21">SDK_Candidates($B$3:$J$11,7,6)</f>
+        <f t="array" ref="G21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>6</v>
       </c>
       <c r="H21" s="3" t="str" cm="1">
-        <f t="array" ref="H21">SDK_Candidates($B$3:$J$11,7,7)</f>
+        <f t="array" ref="H21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>128</v>
       </c>
       <c r="I21" s="3" t="str" cm="1">
-        <f t="array" ref="I21">SDK_Candidates($B$3:$J$11,7,8)</f>
+        <f t="array" ref="I21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J21" s="3" t="str" cm="1">
-        <f t="array" ref="J21">SDK_Candidates($B$3:$J$11,7,9)</f>
+        <f t="array" ref="J21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="str" cm="1">
-        <f t="array" ref="B22">SDK_Candidates($B$3:$J$11,8,1)</f>
+        <f t="array" ref="B22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2</v>
       </c>
       <c r="C22" s="3" t="str" cm="1">
-        <f t="array" ref="C22">SDK_Candidates($B$3:$J$11,8,2)</f>
+        <f t="array" ref="C22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D22" s="3" t="str" cm="1">
-        <f t="array" ref="D22">SDK_Candidates($B$3:$J$11,8,3)</f>
+        <f t="array" ref="D22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>128</v>
       </c>
       <c r="E22" s="3" t="str" cm="1">
-        <f t="array" ref="E22">SDK_Candidates($B$3:$J$11,8,4)</f>
+        <f t="array" ref="E22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>79</v>
       </c>
       <c r="F22" s="3" t="str" cm="1">
-        <f t="array" ref="F22">SDK_Candidates($B$3:$J$11,8,5)</f>
+        <f t="array" ref="F22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G22" s="3" t="str" cm="1">
-        <f t="array" ref="G22">SDK_Candidates($B$3:$J$11,8,6)</f>
+        <f t="array" ref="G22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>79</v>
       </c>
       <c r="H22" s="3" t="str" cm="1">
-        <f t="array" ref="H22">SDK_Candidates($B$3:$J$11,8,7)</f>
+        <f t="array" ref="H22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>128</v>
       </c>
       <c r="I22" s="3" t="str" cm="1">
-        <f t="array" ref="I22">SDK_Candidates($B$3:$J$11,8,8)</f>
+        <f t="array" ref="I22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J22" s="3" t="str" cm="1">
-        <f t="array" ref="J22">SDK_Candidates($B$3:$J$11,8,9)</f>
+        <f t="array" ref="J22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="str" cm="1">
-        <f t="array" ref="B23">SDK_Candidates($B$3:$J$11,9,1)</f>
+        <f t="array" ref="B23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C23" s="3" t="str" cm="1">
-        <f t="array" ref="C23">SDK_Candidates($B$3:$J$11,9,2)</f>
+        <f t="array" ref="C23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>6</v>
       </c>
       <c r="D23" s="3" t="str" cm="1">
-        <f t="array" ref="D23">SDK_Candidates($B$3:$J$11,9,3)</f>
+        <f t="array" ref="D23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E23" s="3" t="str" cm="1">
-        <f t="array" ref="E23">SDK_Candidates($B$3:$J$11,9,4)</f>
+        <f t="array" ref="E23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>49</v>
       </c>
       <c r="F23" s="3" t="str" cm="1">
-        <f t="array" ref="F23">SDK_Candidates($B$3:$J$11,9,5)</f>
+        <f t="array" ref="F23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G23" s="3" t="str" cm="1">
-        <f t="array" ref="G23">SDK_Candidates($B$3:$J$11,9,6)</f>
+        <f t="array" ref="G23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H23" s="3" t="str" cm="1">
-        <f t="array" ref="H23">SDK_Candidates($B$3:$J$11,9,7)</f>
+        <f t="array" ref="H23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2</v>
       </c>
       <c r="I23" s="3" t="str" cm="1">
-        <f t="array" ref="I23">SDK_Candidates($B$3:$J$11,9,8)</f>
+        <f t="array" ref="I23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>5</v>
       </c>
       <c r="J23" s="3" t="str" cm="1">
-        <f t="array" ref="J23">SDK_Candidates($B$3:$J$11,9,9)</f>
+        <f t="array" ref="J23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>259</v>
       </c>
     </row>
@@ -8238,7 +8238,7 @@
         <v>74</v>
       </c>
       <c r="B88" s="7" t="str" cm="1">
-        <f t="array" ref="B88">IF(OR('02 Medium'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",SDK_PlayerHint($B$3:$J$11,$B$39:$J$47))</f>
+        <f t="array" ref="B88">IF(OR('02 Medium'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",IF($L$111="ASSIGNMENT",$N$111,IF($L$111="LIMIT","Candidate chain limit reached after "&amp;$M$111&amp;" elimination step(s).",IF($L$111="CONTRADICTION","Candidate chain contradiction detected.",SDK_FallbackReveal($B$3:$J$11,$B$39:$J$47)))))</f>
         <v>Naked single · R1C2 = 3 · This is the only legal candidate remaining in the square.</v>
       </c>
       <c r="C88" s="7"/>
@@ -8264,8 +8264,8 @@
       <c r="A89" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B89" s="7" t="str" cm="1">
-        <f t="array" ref="B89">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),1)</f>
+      <c r="B89" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;1,"Technique — "&amp;INDEX(_xlpm.parts,1,1)&amp;" | Pattern — "&amp;INDEX(_xlpm.parts,1,2),"Status — "&amp;INDEX(_xlpm.parts,1,1))))</f>
         <v>Technique — Naked single | Pattern — R1C2 = 3</v>
       </c>
       <c r="C89" s="7"/>
@@ -8293,8 +8293,8 @@
       <c r="A90" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B90" s="7" t="str" cm="1">
-        <f t="array" ref="B90">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),2)</f>
+      <c r="B90" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;2,"Action — "&amp;_xlfn.TEXTJOIN(" · ",TRUE,_xlfn.DROP(_xlpm.parts,,2)),"Action — No further supported step.")))</f>
         <v>Action — This is the only legal candidate remaining in the square.</v>
       </c>
       <c r="C90" s="7"/>
@@ -8545,6 +8545,302 @@
       </c>
       <c r="B100" t="str" cm="1">
         <f t="array" ref="B100">IF('02 Medium'!$AS$11="Verify",IF(COUNTIF($B$51:$J$59,TRUE)&gt;0,"CONFLICT",SDK_SolveStatus($B$3:$J$11)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="1:20">
+      <c r="L101" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="102" spans="1:20">
+      <c r="L102" t="str" cm="1">
+        <f t="array" ref="L102:T111">SDKP_Chain($B$3:$J$11,8)</f>
+        <v>345</v>
+      </c>
+      <c r="M102" t="str">
+        <v>3</v>
+      </c>
+      <c r="N102" t="str">
+        <v>5</v>
+      </c>
+      <c r="O102" t="str">
+        <v/>
+      </c>
+      <c r="P102" t="str">
+        <v/>
+      </c>
+      <c r="Q102" t="str">
+        <v>59</v>
+      </c>
+      <c r="R102" t="str">
+        <v/>
+      </c>
+      <c r="S102" t="str">
+        <v>8</v>
+      </c>
+      <c r="T102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103" spans="1:20">
+      <c r="L103" t="str">
+        <v/>
+      </c>
+      <c r="M103" t="str">
+        <v/>
+      </c>
+      <c r="N103" t="str">
+        <v>25</v>
+      </c>
+      <c r="O103" t="str">
+        <v>5</v>
+      </c>
+      <c r="P103" t="str">
+        <v/>
+      </c>
+      <c r="Q103" t="str">
+        <v>15</v>
+      </c>
+      <c r="R103" t="str">
+        <v>234</v>
+      </c>
+      <c r="S103" t="str">
+        <v/>
+      </c>
+      <c r="T103" t="str">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="104" spans="1:20">
+      <c r="L104" t="str">
+        <v/>
+      </c>
+      <c r="M104" t="str">
+        <v/>
+      </c>
+      <c r="N104" t="str">
+        <v>27</v>
+      </c>
+      <c r="O104" t="str">
+        <v>8</v>
+      </c>
+      <c r="P104" t="str">
+        <v>38</v>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
+      </c>
+      <c r="R104" t="str">
+        <v/>
+      </c>
+      <c r="S104" t="str">
+        <v>68</v>
+      </c>
+      <c r="T104" t="str">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="105" spans="1:20">
+      <c r="L105" t="str">
+        <v/>
+      </c>
+      <c r="M105" t="str">
+        <v/>
+      </c>
+      <c r="N105" t="str">
+        <v>67</v>
+      </c>
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v>9</v>
+      </c>
+      <c r="Q105" t="str">
+        <v>579</v>
+      </c>
+      <c r="R105" t="str">
+        <v>36</v>
+      </c>
+      <c r="S105" t="str">
+        <v/>
+      </c>
+      <c r="T105" t="str">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="106" spans="1:20">
+      <c r="L106" t="str">
+        <v>3</v>
+      </c>
+      <c r="M106" t="str">
+        <v>137</v>
+      </c>
+      <c r="N106" t="str">
+        <v/>
+      </c>
+      <c r="O106" t="str">
+        <v/>
+      </c>
+      <c r="P106" t="str">
+        <v>8</v>
+      </c>
+      <c r="Q106" t="str">
+        <v/>
+      </c>
+      <c r="R106" t="str">
+        <v/>
+      </c>
+      <c r="S106" t="str">
+        <v>15</v>
+      </c>
+      <c r="T106" t="str">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="107" spans="1:20">
+      <c r="L107" t="str">
+        <v>9</v>
+      </c>
+      <c r="M107" t="str">
+        <v/>
+      </c>
+      <c r="N107" t="str">
+        <v>167</v>
+      </c>
+      <c r="O107" t="str">
+        <v>479</v>
+      </c>
+      <c r="P107" t="str">
+        <v>49</v>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107" t="str">
+        <v>16</v>
+      </c>
+      <c r="S107" t="str">
+        <v/>
+      </c>
+      <c r="T107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="1:20">
+      <c r="L108" t="str">
+        <v>25</v>
+      </c>
+      <c r="M108" t="str">
+        <v>16</v>
+      </c>
+      <c r="N108" t="str">
+        <v/>
+      </c>
+      <c r="O108" t="str">
+        <v/>
+      </c>
+      <c r="P108" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q108" t="str">
+        <v>6</v>
+      </c>
+      <c r="R108" t="str">
+        <v>128</v>
+      </c>
+      <c r="S108" t="str">
+        <v/>
+      </c>
+      <c r="T108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109" spans="1:20">
+      <c r="L109" t="str">
+        <v>2</v>
+      </c>
+      <c r="M109" t="str">
+        <v/>
+      </c>
+      <c r="N109" t="str">
+        <v>128</v>
+      </c>
+      <c r="O109" t="str">
+        <v>79</v>
+      </c>
+      <c r="P109" t="str">
+        <v/>
+      </c>
+      <c r="Q109" t="str">
+        <v>79</v>
+      </c>
+      <c r="R109" t="str">
+        <v>128</v>
+      </c>
+      <c r="S109" t="str">
+        <v/>
+      </c>
+      <c r="T109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110" spans="1:20">
+      <c r="L110" t="str">
+        <v/>
+      </c>
+      <c r="M110" t="str">
+        <v>6</v>
+      </c>
+      <c r="N110" t="str">
+        <v/>
+      </c>
+      <c r="O110" t="str">
+        <v>49</v>
+      </c>
+      <c r="P110" t="str">
+        <v/>
+      </c>
+      <c r="Q110" t="str">
+        <v/>
+      </c>
+      <c r="R110" t="str">
+        <v>2</v>
+      </c>
+      <c r="S110" t="str">
+        <v>5</v>
+      </c>
+      <c r="T110" t="str">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="111" spans="1:20">
+      <c r="L111" t="str">
+        <v>ASSIGNMENT</v>
+      </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111" t="str">
+        <v>Naked single · R1C2 = 3 · This is the only legal candidate remaining in the square.</v>
+      </c>
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
+      <c r="S111" t="str">
+        <v/>
+      </c>
+      <c r="T111" t="str">
         <v/>
       </c>
     </row>
@@ -41256,7 +41552,7 @@
         <v>1</v>
       </c>
       <c r="D145" t="b">
-        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
+        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
         <v>1</v>
       </c>
       <c r="E145" t="str">

</xml_diff>

<commit_message>
Migrate Easy candidate chain to production
</commit_message>
<xml_diff>
--- a/Sudoku/sudoku.xlsx
+++ b/Sudoku/sudoku.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiangyuan/Documents/learn/excel/vibexcel/Sudoku/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9214672-A963-0F4E-B12F-662D471A5797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D70BC31-F3D9-DD47-8026-B3D5BD7F8EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15740" xr2:uid="{2CEC70F3-4788-3E4C-8B6A-4C94D09786F3}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="701">
   <si>
     <t>SUDOKU ENGINE — 01 EASY</t>
   </si>
@@ -2324,7 +2324,7 @@
     <t>Candidate Chain</t>
   </si>
   <si>
-    <t>Easy standard wrapper plus Medium, Hard, Expert, and Master chain fallback contracts</t>
+    <t>All five published engines use chain Coach fallback contracts</t>
   </si>
 </sst>
 </file>
@@ -41552,7 +41552,7 @@
         <v>1</v>
       </c>
       <c r="D145" t="b">
-        <f ca="1">AND(ISNUMBER(SEARCH("SDK_PlayerHint",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
+        <f ca="1">AND(ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT(_Engine!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Medium'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Hard'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Expert'!$B$88))),ISNUMBER(SEARCH("$L$111=""ASSIGNMENT""",_xlfn.FORMULATEXT('_Engine Master'!$B$88))),ISNUMBER(SEARCH("SDK_FallbackReveal",_xlfn.FORMULATEXT('_Engine Master'!$B$88))))</f>
         <v>1</v>
       </c>
       <c r="E145" t="str">
@@ -42680,7 +42680,7 @@
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FF0B5A2B"/>
   </sheetPr>
-  <dimension ref="A1:T100"/>
+  <dimension ref="A1:T111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -43107,351 +43107,351 @@
     <row r="15" spans="1:10">
       <c r="A15" s="3"/>
       <c r="B15" s="3" t="str" cm="1">
-        <f t="array" ref="B15">SDK_Candidates($B$3:$J$11,1,1)</f>
+        <f t="array" ref="B15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C15" s="3" t="str" cm="1">
-        <f t="array" ref="C15">SDK_Candidates($B$3:$J$11,1,2)</f>
+        <f t="array" ref="C15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D15" s="3" t="str" cm="1">
-        <f t="array" ref="D15">SDK_Candidates($B$3:$J$11,1,3)</f>
+        <f t="array" ref="D15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>124</v>
       </c>
       <c r="E15" s="3" t="str" cm="1">
-        <f t="array" ref="E15">SDK_Candidates($B$3:$J$11,1,4)</f>
+        <f t="array" ref="E15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>26</v>
       </c>
       <c r="F15" s="3" t="str" cm="1">
-        <f t="array" ref="F15">SDK_Candidates($B$3:$J$11,1,5)</f>
+        <f t="array" ref="F15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G15" s="3" t="str" cm="1">
-        <f t="array" ref="G15">SDK_Candidates($B$3:$J$11,1,6)</f>
+        <f t="array" ref="G15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2468</v>
       </c>
       <c r="H15" s="3" t="str" cm="1">
-        <f t="array" ref="H15">SDK_Candidates($B$3:$J$11,1,7)</f>
+        <f t="array" ref="H15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1489</v>
       </c>
       <c r="I15" s="3" t="str" cm="1">
-        <f t="array" ref="I15">SDK_Candidates($B$3:$J$11,1,8)</f>
+        <f t="array" ref="I15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1249</v>
       </c>
       <c r="J15" s="3" t="str" cm="1">
-        <f t="array" ref="J15">SDK_Candidates($B$3:$J$11,1,9)</f>
+        <f t="array" ref="J15">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>248</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3"/>
       <c r="B16" s="3" t="str" cm="1">
-        <f t="array" ref="B16">SDK_Candidates($B$3:$J$11,2,1)</f>
+        <f t="array" ref="B16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C16" s="3" t="str" cm="1">
-        <f t="array" ref="C16">SDK_Candidates($B$3:$J$11,2,2)</f>
+        <f t="array" ref="C16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>247</v>
       </c>
       <c r="D16" s="3" t="str" cm="1">
-        <f t="array" ref="D16">SDK_Candidates($B$3:$J$11,2,3)</f>
+        <f t="array" ref="D16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>247</v>
       </c>
       <c r="E16" s="3" t="str" cm="1">
-        <f t="array" ref="E16">SDK_Candidates($B$3:$J$11,2,4)</f>
+        <f t="array" ref="E16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F16" s="3" t="str" cm="1">
-        <f t="array" ref="F16">SDK_Candidates($B$3:$J$11,2,5)</f>
+        <f t="array" ref="F16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G16" s="3" t="str" cm="1">
-        <f t="array" ref="G16">SDK_Candidates($B$3:$J$11,2,6)</f>
+        <f t="array" ref="G16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H16" s="3" t="str" cm="1">
-        <f t="array" ref="H16">SDK_Candidates($B$3:$J$11,2,7)</f>
+        <f t="array" ref="H16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3478</v>
       </c>
       <c r="I16" s="3" t="str" cm="1">
-        <f t="array" ref="I16">SDK_Candidates($B$3:$J$11,2,8)</f>
+        <f t="array" ref="I16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>234</v>
       </c>
       <c r="J16" s="3" t="str" cm="1">
-        <f t="array" ref="J16">SDK_Candidates($B$3:$J$11,2,9)</f>
+        <f t="array" ref="J16">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2478</v>
       </c>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3"/>
       <c r="B17" s="3" t="str" cm="1">
-        <f t="array" ref="B17">SDK_Candidates($B$3:$J$11,3,1)</f>
+        <f t="array" ref="B17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12</v>
       </c>
       <c r="C17" s="3" t="str" cm="1">
-        <f t="array" ref="C17">SDK_Candidates($B$3:$J$11,3,2)</f>
+        <f t="array" ref="C17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D17" s="3" t="str" cm="1">
-        <f t="array" ref="D17">SDK_Candidates($B$3:$J$11,3,3)</f>
+        <f t="array" ref="D17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="E17" s="3" t="str" cm="1">
-        <f t="array" ref="E17">SDK_Candidates($B$3:$J$11,3,4)</f>
+        <f t="array" ref="E17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23</v>
       </c>
       <c r="F17" s="3" t="str" cm="1">
-        <f t="array" ref="F17">SDK_Candidates($B$3:$J$11,3,5)</f>
+        <f t="array" ref="F17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>34</v>
       </c>
       <c r="G17" s="3" t="str" cm="1">
-        <f t="array" ref="G17">SDK_Candidates($B$3:$J$11,3,6)</f>
+        <f t="array" ref="G17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>24</v>
       </c>
       <c r="H17" s="3" t="str" cm="1">
-        <f t="array" ref="H17">SDK_Candidates($B$3:$J$11,3,7)</f>
+        <f t="array" ref="H17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>13457</v>
       </c>
       <c r="I17" s="3" t="str" cm="1">
-        <f t="array" ref="I17">SDK_Candidates($B$3:$J$11,3,8)</f>
+        <f t="array" ref="I17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J17" s="3" t="str" cm="1">
-        <f t="array" ref="J17">SDK_Candidates($B$3:$J$11,3,9)</f>
+        <f t="array" ref="J17">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3"/>
       <c r="B18" s="3" t="str" cm="1">
-        <f t="array" ref="B18">SDK_Candidates($B$3:$J$11,4,1)</f>
+        <f t="array" ref="B18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C18" s="3" t="str" cm="1">
-        <f t="array" ref="C18">SDK_Candidates($B$3:$J$11,4,2)</f>
+        <f t="array" ref="C18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>125</v>
       </c>
       <c r="D18" s="3" t="str" cm="1">
-        <f t="array" ref="D18">SDK_Candidates($B$3:$J$11,4,3)</f>
+        <f t="array" ref="D18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1259</v>
       </c>
       <c r="E18" s="3" t="str" cm="1">
-        <f t="array" ref="E18">SDK_Candidates($B$3:$J$11,4,4)</f>
+        <f t="array" ref="E18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>579</v>
       </c>
       <c r="F18" s="3" t="str" cm="1">
-        <f t="array" ref="F18">SDK_Candidates($B$3:$J$11,4,5)</f>
+        <f t="array" ref="F18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G18" s="3" t="str" cm="1">
-        <f t="array" ref="G18">SDK_Candidates($B$3:$J$11,4,6)</f>
+        <f t="array" ref="G18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>147</v>
       </c>
       <c r="H18" s="3" t="str" cm="1">
-        <f t="array" ref="H18">SDK_Candidates($B$3:$J$11,4,7)</f>
+        <f t="array" ref="H18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4579</v>
       </c>
       <c r="I18" s="3" t="str" cm="1">
-        <f t="array" ref="I18">SDK_Candidates($B$3:$J$11,4,8)</f>
+        <f t="array" ref="I18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2459</v>
       </c>
       <c r="J18" s="3" t="str" cm="1">
-        <f t="array" ref="J18">SDK_Candidates($B$3:$J$11,4,9)</f>
+        <f t="array" ref="J18">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3"/>
       <c r="B19" s="3" t="str" cm="1">
-        <f t="array" ref="B19">SDK_Candidates($B$3:$J$11,5,1)</f>
+        <f t="array" ref="B19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C19" s="3" t="str" cm="1">
-        <f t="array" ref="C19">SDK_Candidates($B$3:$J$11,5,2)</f>
+        <f t="array" ref="C19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>25</v>
       </c>
       <c r="D19" s="3" t="str" cm="1">
-        <f t="array" ref="D19">SDK_Candidates($B$3:$J$11,5,3)</f>
+        <f t="array" ref="D19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2569</v>
       </c>
       <c r="E19" s="3" t="str" cm="1">
-        <f t="array" ref="E19">SDK_Candidates($B$3:$J$11,5,4)</f>
+        <f t="array" ref="E19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F19" s="3" t="str" cm="1">
-        <f t="array" ref="F19">SDK_Candidates($B$3:$J$11,5,5)</f>
+        <f t="array" ref="F19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>5</v>
       </c>
       <c r="G19" s="3" t="str" cm="1">
-        <f t="array" ref="G19">SDK_Candidates($B$3:$J$11,5,6)</f>
+        <f t="array" ref="G19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H19" s="3" t="str" cm="1">
-        <f t="array" ref="H19">SDK_Candidates($B$3:$J$11,5,7)</f>
+        <f t="array" ref="H19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>579</v>
       </c>
       <c r="I19" s="3" t="str" cm="1">
-        <f t="array" ref="I19">SDK_Candidates($B$3:$J$11,5,8)</f>
+        <f t="array" ref="I19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>259</v>
       </c>
       <c r="J19" s="3" t="str" cm="1">
-        <f t="array" ref="J19">SDK_Candidates($B$3:$J$11,5,9)</f>
+        <f t="array" ref="J19">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3"/>
       <c r="B20" s="3" t="str" cm="1">
-        <f t="array" ref="B20">SDK_Candidates($B$3:$J$11,6,1)</f>
+        <f t="array" ref="B20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="C20" s="3" t="str" cm="1">
-        <f t="array" ref="C20">SDK_Candidates($B$3:$J$11,6,2)</f>
+        <f t="array" ref="C20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>15</v>
       </c>
       <c r="D20" s="3" t="str" cm="1">
-        <f t="array" ref="D20">SDK_Candidates($B$3:$J$11,6,3)</f>
+        <f t="array" ref="D20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1359</v>
       </c>
       <c r="E20" s="3" t="str" cm="1">
-        <f t="array" ref="E20">SDK_Candidates($B$3:$J$11,6,4)</f>
+        <f t="array" ref="E20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>59</v>
       </c>
       <c r="F20" s="3" t="str" cm="1">
-        <f t="array" ref="F20">SDK_Candidates($B$3:$J$11,6,5)</f>
+        <f t="array" ref="F20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G20" s="3" t="str" cm="1">
-        <f t="array" ref="G20">SDK_Candidates($B$3:$J$11,6,6)</f>
+        <f t="array" ref="G20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>14</v>
       </c>
       <c r="H20" s="3" t="str" cm="1">
-        <f t="array" ref="H20">SDK_Candidates($B$3:$J$11,6,7)</f>
+        <f t="array" ref="H20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4589</v>
       </c>
       <c r="I20" s="3" t="str" cm="1">
-        <f t="array" ref="I20">SDK_Candidates($B$3:$J$11,6,8)</f>
+        <f t="array" ref="I20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>459</v>
       </c>
       <c r="J20" s="3" t="str" cm="1">
-        <f t="array" ref="J20">SDK_Candidates($B$3:$J$11,6,9)</f>
+        <f t="array" ref="J20">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3"/>
       <c r="B21" s="3" t="str" cm="1">
-        <f t="array" ref="B21">SDK_Candidates($B$3:$J$11,7,1)</f>
+        <f t="array" ref="B21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>139</v>
       </c>
       <c r="C21" s="3" t="str" cm="1">
-        <f t="array" ref="C21">SDK_Candidates($B$3:$J$11,7,2)</f>
+        <f t="array" ref="C21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="D21" s="3" t="str" cm="1">
-        <f t="array" ref="D21">SDK_Candidates($B$3:$J$11,7,3)</f>
+        <f t="array" ref="D21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>134579</v>
       </c>
       <c r="E21" s="3" t="str" cm="1">
-        <f t="array" ref="E21">SDK_Candidates($B$3:$J$11,7,4)</f>
+        <f t="array" ref="E21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>357</v>
       </c>
       <c r="F21" s="3" t="str" cm="1">
-        <f t="array" ref="F21">SDK_Candidates($B$3:$J$11,7,5)</f>
+        <f t="array" ref="F21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>35</v>
       </c>
       <c r="G21" s="3" t="str" cm="1">
-        <f t="array" ref="G21">SDK_Candidates($B$3:$J$11,7,6)</f>
+        <f t="array" ref="G21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>7</v>
       </c>
       <c r="H21" s="3" t="str" cm="1">
-        <f t="array" ref="H21">SDK_Candidates($B$3:$J$11,7,7)</f>
+        <f t="array" ref="H21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="I21" s="3" t="str" cm="1">
-        <f t="array" ref="I21">SDK_Candidates($B$3:$J$11,7,8)</f>
+        <f t="array" ref="I21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J21" s="3" t="str" cm="1">
-        <f t="array" ref="J21">SDK_Candidates($B$3:$J$11,7,9)</f>
+        <f t="array" ref="J21">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="3"/>
       <c r="B22" s="3" t="str" cm="1">
-        <f t="array" ref="B22">SDK_Candidates($B$3:$J$11,8,1)</f>
+        <f t="array" ref="B22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>23</v>
       </c>
       <c r="C22" s="3" t="str" cm="1">
-        <f t="array" ref="C22">SDK_Candidates($B$3:$J$11,8,2)</f>
+        <f t="array" ref="C22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>278</v>
       </c>
       <c r="D22" s="3" t="str" cm="1">
-        <f t="array" ref="D22">SDK_Candidates($B$3:$J$11,8,3)</f>
+        <f t="array" ref="D22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>237</v>
       </c>
       <c r="E22" s="3" t="str" cm="1">
-        <f t="array" ref="E22">SDK_Candidates($B$3:$J$11,8,4)</f>
+        <f t="array" ref="E22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="F22" s="3" t="str" cm="1">
-        <f t="array" ref="F22">SDK_Candidates($B$3:$J$11,8,5)</f>
+        <f t="array" ref="F22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G22" s="3" t="str" cm="1">
-        <f t="array" ref="G22">SDK_Candidates($B$3:$J$11,8,6)</f>
+        <f t="array" ref="G22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="H22" s="3" t="str" cm="1">
-        <f t="array" ref="H22">SDK_Candidates($B$3:$J$11,8,7)</f>
+        <f t="array" ref="H22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>36</v>
       </c>
       <c r="I22" s="3" t="str" cm="1">
-        <f t="array" ref="I22">SDK_Candidates($B$3:$J$11,8,8)</f>
+        <f t="array" ref="I22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>3</v>
       </c>
       <c r="J22" s="3" t="str" cm="1">
-        <f t="array" ref="J22">SDK_Candidates($B$3:$J$11,8,9)</f>
+        <f t="array" ref="J22">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="str" cm="1">
-        <f t="array" ref="B23">SDK_Candidates($B$3:$J$11,9,1)</f>
+        <f t="array" ref="B23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>123</v>
       </c>
       <c r="C23" s="3" t="str" cm="1">
-        <f t="array" ref="C23">SDK_Candidates($B$3:$J$11,9,2)</f>
+        <f t="array" ref="C23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1245</v>
       </c>
       <c r="D23" s="3" t="str" cm="1">
-        <f t="array" ref="D23">SDK_Candidates($B$3:$J$11,9,3)</f>
+        <f t="array" ref="D23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>12345</v>
       </c>
       <c r="E23" s="3" t="str" cm="1">
-        <f t="array" ref="E23">SDK_Candidates($B$3:$J$11,9,4)</f>
+        <f t="array" ref="E23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>2356</v>
       </c>
       <c r="F23" s="3" t="str" cm="1">
-        <f t="array" ref="F23">SDK_Candidates($B$3:$J$11,9,5)</f>
+        <f t="array" ref="F23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="G23" s="3" t="str" cm="1">
-        <f t="array" ref="G23">SDK_Candidates($B$3:$J$11,9,6)</f>
+        <f t="array" ref="G23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>26</v>
       </c>
       <c r="H23" s="3" t="str" cm="1">
-        <f t="array" ref="H23">SDK_Candidates($B$3:$J$11,9,7)</f>
+        <f t="array" ref="H23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v>1346</v>
       </c>
       <c r="I23" s="3" t="str" cm="1">
-        <f t="array" ref="I23">SDK_Candidates($B$3:$J$11,9,8)</f>
+        <f t="array" ref="I23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
       <c r="J23" s="3" t="str" cm="1">
-        <f t="array" ref="J23">SDK_Candidates($B$3:$J$11,9,9)</f>
+        <f t="array" ref="J23">INDEX($L$102:$T$110,ROW()-14,COLUMN()-1)</f>
         <v/>
       </c>
     </row>
@@ -44633,7 +44633,7 @@
         <v>74</v>
       </c>
       <c r="B88" s="7" t="str" cm="1">
-        <f t="array" ref="B88">IF(OR('01 Easy'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",SDK_PlayerHint($B$3:$J$11,$B$39:$J$47))</f>
+        <f t="array" ref="B88">IF(OR('01 Easy'!$AS$11="Verify",COUNTIF($B$51:$J$59,TRUE)&gt;0,$B$99),"",IF($L$111="ASSIGNMENT",$N$111,IF($L$111="LIMIT","Candidate chain limit reached after "&amp;$M$111&amp;" elimination step(s).",IF($L$111="CONTRADICTION","Candidate chain contradiction detected.",SDK_FallbackReveal($B$3:$J$11,$B$39:$J$47)))))</f>
         <v>Naked single · R5C5 = 5 · This is the only legal candidate remaining in the square.</v>
       </c>
       <c r="C88" s="7"/>
@@ -44659,8 +44659,8 @@
       <c r="A89" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B89" s="7" t="str" cm="1">
-        <f t="array" ref="B89">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),1)</f>
+      <c r="B89" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;1,"Technique — "&amp;INDEX(_xlpm.parts,1,1)&amp;" | Pattern — "&amp;INDEX(_xlpm.parts,1,2),"Status — "&amp;INDEX(_xlpm.parts,1,1))))</f>
         <v>Technique — Naked single | Pattern — R5C5 = 5</v>
       </c>
       <c r="C89" s="7"/>
@@ -44688,8 +44688,8 @@
       <c r="A90" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B90" s="7" t="str" cm="1">
-        <f t="array" ref="B90">INDEX(SDK_PlayerTrace($B$3:$J$11,$B$39:$J$47),2)</f>
+      <c r="B90" s="7" t="str">
+        <f>IF($B$88="","",_xlfn.LET(_xlpm.parts,_xlfn.TEXTSPLIT($B$88," · "),_xlpm.partCount,COLUMNS(_xlpm.parts),IF(_xlpm.partCount&gt;2,"Action — "&amp;_xlfn.TEXTJOIN(" · ",TRUE,_xlfn.DROP(_xlpm.parts,,2)),"Action — No further supported step.")))</f>
         <v>Action — This is the only legal candidate remaining in the square.</v>
       </c>
       <c r="C90" s="7"/>
@@ -44943,6 +44943,302 @@
         <v/>
       </c>
     </row>
+    <row r="101" spans="1:20">
+      <c r="L101" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="102" spans="1:20">
+      <c r="L102" t="str" cm="1">
+        <f t="array" ref="L102:T111">SDKP_Chain($B$3:$J$11,8)</f>
+        <v/>
+      </c>
+      <c r="M102" t="str">
+        <v/>
+      </c>
+      <c r="N102" t="str">
+        <v>124</v>
+      </c>
+      <c r="O102" t="str">
+        <v>26</v>
+      </c>
+      <c r="P102" t="str">
+        <v/>
+      </c>
+      <c r="Q102" t="str">
+        <v>2468</v>
+      </c>
+      <c r="R102" t="str">
+        <v>1489</v>
+      </c>
+      <c r="S102" t="str">
+        <v>1249</v>
+      </c>
+      <c r="T102" t="str">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="103" spans="1:20">
+      <c r="L103" t="str">
+        <v/>
+      </c>
+      <c r="M103" t="str">
+        <v>247</v>
+      </c>
+      <c r="N103" t="str">
+        <v>247</v>
+      </c>
+      <c r="O103" t="str">
+        <v/>
+      </c>
+      <c r="P103" t="str">
+        <v/>
+      </c>
+      <c r="Q103" t="str">
+        <v/>
+      </c>
+      <c r="R103" t="str">
+        <v>3478</v>
+      </c>
+      <c r="S103" t="str">
+        <v>234</v>
+      </c>
+      <c r="T103" t="str">
+        <v>2478</v>
+      </c>
+    </row>
+    <row r="104" spans="1:20">
+      <c r="L104" t="str">
+        <v>12</v>
+      </c>
+      <c r="M104" t="str">
+        <v/>
+      </c>
+      <c r="N104" t="str">
+        <v/>
+      </c>
+      <c r="O104" t="str">
+        <v>23</v>
+      </c>
+      <c r="P104" t="str">
+        <v>34</v>
+      </c>
+      <c r="Q104" t="str">
+        <v>24</v>
+      </c>
+      <c r="R104" t="str">
+        <v>13457</v>
+      </c>
+      <c r="S104" t="str">
+        <v/>
+      </c>
+      <c r="T104" t="str">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="105" spans="1:20">
+      <c r="L105" t="str">
+        <v/>
+      </c>
+      <c r="M105" t="str">
+        <v>125</v>
+      </c>
+      <c r="N105" t="str">
+        <v>1259</v>
+      </c>
+      <c r="O105" t="str">
+        <v>579</v>
+      </c>
+      <c r="P105" t="str">
+        <v/>
+      </c>
+      <c r="Q105" t="str">
+        <v>147</v>
+      </c>
+      <c r="R105" t="str">
+        <v>4579</v>
+      </c>
+      <c r="S105" t="str">
+        <v>2459</v>
+      </c>
+      <c r="T105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106" spans="1:20">
+      <c r="L106" t="str">
+        <v/>
+      </c>
+      <c r="M106" t="str">
+        <v>25</v>
+      </c>
+      <c r="N106" t="str">
+        <v>2569</v>
+      </c>
+      <c r="O106" t="str">
+        <v/>
+      </c>
+      <c r="P106" t="str">
+        <v>5</v>
+      </c>
+      <c r="Q106" t="str">
+        <v/>
+      </c>
+      <c r="R106" t="str">
+        <v>579</v>
+      </c>
+      <c r="S106" t="str">
+        <v>259</v>
+      </c>
+      <c r="T106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107" spans="1:20">
+      <c r="L107" t="str">
+        <v/>
+      </c>
+      <c r="M107" t="str">
+        <v>15</v>
+      </c>
+      <c r="N107" t="str">
+        <v>1359</v>
+      </c>
+      <c r="O107" t="str">
+        <v>59</v>
+      </c>
+      <c r="P107" t="str">
+        <v/>
+      </c>
+      <c r="Q107" t="str">
+        <v>14</v>
+      </c>
+      <c r="R107" t="str">
+        <v>4589</v>
+      </c>
+      <c r="S107" t="str">
+        <v>459</v>
+      </c>
+      <c r="T107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108" spans="1:20">
+      <c r="L108" t="str">
+        <v>139</v>
+      </c>
+      <c r="M108" t="str">
+        <v/>
+      </c>
+      <c r="N108" t="str">
+        <v>134579</v>
+      </c>
+      <c r="O108" t="str">
+        <v>357</v>
+      </c>
+      <c r="P108" t="str">
+        <v>35</v>
+      </c>
+      <c r="Q108" t="str">
+        <v>7</v>
+      </c>
+      <c r="R108" t="str">
+        <v/>
+      </c>
+      <c r="S108" t="str">
+        <v/>
+      </c>
+      <c r="T108" t="str">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:20">
+      <c r="L109" t="str">
+        <v>23</v>
+      </c>
+      <c r="M109" t="str">
+        <v>278</v>
+      </c>
+      <c r="N109" t="str">
+        <v>237</v>
+      </c>
+      <c r="O109" t="str">
+        <v/>
+      </c>
+      <c r="P109" t="str">
+        <v/>
+      </c>
+      <c r="Q109" t="str">
+        <v/>
+      </c>
+      <c r="R109" t="str">
+        <v>36</v>
+      </c>
+      <c r="S109" t="str">
+        <v>3</v>
+      </c>
+      <c r="T109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110" spans="1:20">
+      <c r="L110" t="str">
+        <v>123</v>
+      </c>
+      <c r="M110" t="str">
+        <v>1245</v>
+      </c>
+      <c r="N110" t="str">
+        <v>12345</v>
+      </c>
+      <c r="O110" t="str">
+        <v>2356</v>
+      </c>
+      <c r="P110" t="str">
+        <v/>
+      </c>
+      <c r="Q110" t="str">
+        <v>26</v>
+      </c>
+      <c r="R110" t="str">
+        <v>1346</v>
+      </c>
+      <c r="S110" t="str">
+        <v/>
+      </c>
+      <c r="T110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111" spans="1:20">
+      <c r="L111" t="str">
+        <v>ASSIGNMENT</v>
+      </c>
+      <c r="M111">
+        <v>0</v>
+      </c>
+      <c r="N111" t="str">
+        <v>Naked single · R5C5 = 5 · This is the only legal candidate remaining in the square.</v>
+      </c>
+      <c r="O111" t="str">
+        <v/>
+      </c>
+      <c r="P111" t="str">
+        <v/>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
+      <c r="S111" t="str">
+        <v/>
+      </c>
+      <c r="T111" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B66:J66"/>

</xml_diff>